<commit_message>
test: add UPDATE condition hybrid expectations
</commit_message>
<xml_diff>
--- a/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
+++ b/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\Macro\SqlAnalyzerFormatter-feature\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DE4A88F-1CBE-4AE1-BC06-70C37B7DBCE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FA2F8A5-2DBC-4F24-993D-244F406887F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{41A826B0-B2A2-4DC8-9B04-8EFBE807DC37}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="60" activeTab="66" xr2:uid="{41A826B0-B2A2-4DC8-9B04-8EFBE807DC37}"/>
   </bookViews>
   <sheets>
     <sheet name="SEL-064" sheetId="66" r:id="rId1"/>
@@ -77,6 +77,9 @@
     <sheet name="SEL-003" sheetId="3" r:id="rId62"/>
     <sheet name="SEL-002" sheetId="2" r:id="rId63"/>
     <sheet name="SEL-001" sheetId="1" r:id="rId64"/>
+    <sheet name="SEL-065" sheetId="67" r:id="rId65"/>
+    <sheet name="SEL-066" sheetId="68" r:id="rId66"/>
+    <sheet name="SEL-067" sheetId="69" r:id="rId67"/>
   </sheets>
   <calcPr calcId="191029" calcMode="manual"/>
   <extLst>
@@ -88,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1156" uniqueCount="324">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1211" uniqueCount="337">
   <si>
     <t>＜DB入出力項目定義＞</t>
     <rPh sb="3" eb="10">
@@ -1393,6 +1396,45 @@
   <si>
     <t>EXISTS (SQ1)</t>
   </si>
+  <si>
+    <t>参照テーブル: ユーザー[users]、注文[tb2]</t>
+  </si>
+  <si>
+    <t>tb2.注文ユーザーID = users.ユーザーID</t>
+  </si>
+  <si>
+    <t>tb2.状態 = 'CANCELLED'</t>
+  </si>
+  <si>
+    <t>参照テーブル: ユーザー[users]、SQ1</t>
+  </si>
+  <si>
+    <t>'INACTIVE'</t>
+  </si>
+  <si>
+    <t>average_amount</t>
+  </si>
+  <si>
+    <t>AVG(tb2.金額)</t>
+  </si>
+  <si>
+    <t>'REVIEW'</t>
+  </si>
+  <si>
+    <t>tb1.金額 &gt; (SQ1)</t>
+  </si>
+  <si>
+    <t>参照テーブル: 注文[tb2]</t>
+  </si>
+  <si>
+    <t>tb2.注文日時 &lt; @cutoff</t>
+  </si>
+  <si>
+    <t>'ARCHIVED'</t>
+  </si>
+  <si>
+    <t>tb1.ユーザーID IN (SQ1)</t>
+  </si>
 </sst>
 </file>
 
@@ -1733,7 +1775,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1936,6 +1978,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="3" borderId="20" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="15" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -45051,6 +45096,3010 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{125A3CC4-F32F-4AFC-B49F-2EB086F762F7}">
+  <dimension ref="A1:CL11"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="90" width="1.75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="56" t="s">
+        <v>202</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
+      <c r="AD1" s="1"/>
+      <c r="AE1" s="1"/>
+      <c r="AF1" s="1"/>
+      <c r="AG1" s="1"/>
+      <c r="AH1" s="1"/>
+      <c r="AI1" s="1"/>
+      <c r="AJ1" s="1"/>
+      <c r="AK1" s="1"/>
+      <c r="AL1" s="1"/>
+      <c r="AM1" s="1"/>
+      <c r="AN1" s="1"/>
+      <c r="AO1" s="1"/>
+      <c r="AP1" s="1"/>
+      <c r="AQ1" s="1"/>
+      <c r="AR1" s="1"/>
+      <c r="AS1" s="1"/>
+      <c r="AT1" s="1"/>
+      <c r="AU1" s="1"/>
+      <c r="AV1" s="1"/>
+      <c r="AW1" s="1"/>
+      <c r="AX1" s="1"/>
+      <c r="AY1" s="1"/>
+      <c r="AZ1" s="1"/>
+      <c r="BA1" s="1"/>
+      <c r="BB1" s="1"/>
+      <c r="BC1" s="1"/>
+      <c r="BD1" s="1"/>
+      <c r="BE1" s="1"/>
+      <c r="BF1" s="1"/>
+      <c r="BG1" s="1"/>
+      <c r="BH1" s="1"/>
+      <c r="BI1" s="1"/>
+      <c r="BJ1" s="1"/>
+      <c r="BK1" s="1"/>
+      <c r="BL1" s="1"/>
+      <c r="BM1" s="1"/>
+      <c r="BN1" s="1"/>
+      <c r="BO1" s="1"/>
+      <c r="BP1" s="1"/>
+      <c r="BQ1" s="1"/>
+      <c r="BR1" s="1"/>
+      <c r="BS1" s="1"/>
+      <c r="BT1" s="1"/>
+      <c r="BU1" s="1"/>
+      <c r="BV1" s="1"/>
+      <c r="BW1" s="1"/>
+      <c r="BX1" s="1"/>
+      <c r="BY1" s="1"/>
+      <c r="BZ1" s="1"/>
+      <c r="CA1" s="1"/>
+      <c r="CB1" s="1"/>
+      <c r="CC1" s="1"/>
+      <c r="CD1" s="1"/>
+      <c r="CE1" s="1"/>
+      <c r="CF1" s="1"/>
+      <c r="CG1" s="1"/>
+      <c r="CH1" s="1"/>
+      <c r="CI1" s="1"/>
+      <c r="CJ1" s="1"/>
+      <c r="CK1" s="1"/>
+      <c r="CL1" s="1"/>
+    </row>
+    <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="56" t="s">
+        <v>324</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1"/>
+      <c r="W2" s="1"/>
+      <c r="X2" s="1"/>
+      <c r="Y2" s="1"/>
+      <c r="Z2" s="1"/>
+      <c r="AA2" s="1"/>
+      <c r="AB2" s="1"/>
+      <c r="AC2" s="1"/>
+      <c r="AD2" s="1"/>
+      <c r="AE2" s="1"/>
+      <c r="AF2" s="1"/>
+      <c r="AG2" s="1"/>
+      <c r="AH2" s="1"/>
+      <c r="AI2" s="1"/>
+      <c r="AJ2" s="1"/>
+      <c r="AK2" s="1"/>
+      <c r="AL2" s="1"/>
+      <c r="AM2" s="1"/>
+      <c r="AN2" s="1"/>
+      <c r="AO2" s="1"/>
+      <c r="AP2" s="1"/>
+      <c r="AQ2" s="1"/>
+      <c r="AR2" s="1"/>
+      <c r="AS2" s="1"/>
+      <c r="AT2" s="1"/>
+      <c r="AU2" s="1"/>
+      <c r="AV2" s="1"/>
+      <c r="AW2" s="1"/>
+      <c r="AX2" s="1"/>
+      <c r="AY2" s="1"/>
+      <c r="AZ2" s="1"/>
+      <c r="BA2" s="1"/>
+      <c r="BB2" s="1"/>
+      <c r="BC2" s="1"/>
+      <c r="BD2" s="1"/>
+      <c r="BE2" s="1"/>
+      <c r="BF2" s="1"/>
+      <c r="BG2" s="1"/>
+      <c r="BH2" s="1"/>
+      <c r="BI2" s="1"/>
+      <c r="BJ2" s="1"/>
+      <c r="BK2" s="1"/>
+      <c r="BL2" s="1"/>
+      <c r="BM2" s="1"/>
+      <c r="BN2" s="1"/>
+      <c r="BO2" s="1"/>
+      <c r="BP2" s="1"/>
+      <c r="BQ2" s="1"/>
+      <c r="BR2" s="1"/>
+      <c r="BS2" s="1"/>
+      <c r="BT2" s="1"/>
+      <c r="BU2" s="1"/>
+      <c r="BV2" s="1"/>
+      <c r="BW2" s="1"/>
+      <c r="BX2" s="1"/>
+      <c r="BY2" s="1"/>
+      <c r="BZ2" s="1"/>
+      <c r="CA2" s="1"/>
+      <c r="CB2" s="1"/>
+      <c r="CC2" s="1"/>
+      <c r="CD2" s="1"/>
+      <c r="CE2" s="1"/>
+      <c r="CF2" s="1"/>
+      <c r="CG2" s="1"/>
+      <c r="CH2" s="1"/>
+      <c r="CI2" s="1"/>
+      <c r="CJ2" s="1"/>
+      <c r="CK2" s="1"/>
+      <c r="CL2" s="1"/>
+    </row>
+    <row r="3" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="57" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="58" t="s">
+        <v>57</v>
+      </c>
+      <c r="H3" s="28"/>
+      <c r="I3" s="28"/>
+      <c r="J3" s="28"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="28"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="28"/>
+      <c r="O3" s="59" t="s">
+        <v>58</v>
+      </c>
+      <c r="P3" s="28"/>
+      <c r="Q3" s="59" t="s">
+        <v>308</v>
+      </c>
+      <c r="R3" s="28"/>
+      <c r="S3" s="28"/>
+      <c r="T3" s="28"/>
+      <c r="U3" s="28"/>
+      <c r="V3" s="28"/>
+      <c r="W3" s="28"/>
+      <c r="X3" s="28"/>
+      <c r="Y3" s="28"/>
+      <c r="Z3" s="28"/>
+      <c r="AA3" s="28"/>
+      <c r="AB3" s="28"/>
+      <c r="AC3" s="28"/>
+      <c r="AD3" s="28"/>
+      <c r="AE3" s="28"/>
+      <c r="AF3" s="28"/>
+      <c r="AG3" s="28"/>
+      <c r="AH3" s="28"/>
+      <c r="AI3" s="28"/>
+      <c r="AJ3" s="28"/>
+      <c r="AK3" s="28"/>
+      <c r="AL3" s="28"/>
+      <c r="AM3" s="28"/>
+      <c r="AN3" s="28"/>
+      <c r="AO3" s="28"/>
+      <c r="AP3" s="28"/>
+      <c r="AQ3" s="28"/>
+      <c r="AR3" s="28"/>
+      <c r="AS3" s="28"/>
+      <c r="AT3" s="28"/>
+      <c r="AU3" s="28"/>
+      <c r="AV3" s="28"/>
+      <c r="AW3" s="28"/>
+      <c r="AX3" s="28"/>
+      <c r="AY3" s="28"/>
+      <c r="AZ3" s="28"/>
+      <c r="BA3" s="28"/>
+      <c r="BB3" s="28"/>
+      <c r="BC3" s="28"/>
+      <c r="BD3" s="28"/>
+      <c r="BE3" s="28"/>
+      <c r="BF3" s="28"/>
+      <c r="BG3" s="28"/>
+      <c r="BH3" s="28"/>
+      <c r="BI3" s="28"/>
+      <c r="BJ3" s="28"/>
+      <c r="BK3" s="28"/>
+      <c r="BL3" s="28"/>
+      <c r="BM3" s="28"/>
+      <c r="BN3" s="28"/>
+      <c r="BO3" s="28"/>
+      <c r="BP3" s="28"/>
+      <c r="BQ3" s="28"/>
+      <c r="BR3" s="28"/>
+      <c r="BS3" s="28"/>
+      <c r="BT3" s="28"/>
+      <c r="BU3" s="28"/>
+      <c r="BV3" s="28"/>
+      <c r="BW3" s="28"/>
+      <c r="BX3" s="28"/>
+      <c r="BY3" s="28"/>
+      <c r="BZ3" s="28"/>
+      <c r="CA3" s="28"/>
+      <c r="CB3" s="28"/>
+      <c r="CC3" s="28"/>
+      <c r="CD3" s="28"/>
+      <c r="CE3" s="28"/>
+      <c r="CF3" s="28"/>
+      <c r="CG3" s="28"/>
+      <c r="CH3" s="28"/>
+      <c r="CI3" s="28"/>
+      <c r="CJ3" s="28"/>
+      <c r="CK3" s="28"/>
+      <c r="CL3" s="29"/>
+    </row>
+    <row r="4" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="57" t="s">
+        <v>113</v>
+      </c>
+      <c r="B4" s="26"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="28"/>
+      <c r="I4" s="28"/>
+      <c r="J4" s="28"/>
+      <c r="K4" s="28"/>
+      <c r="L4" s="28"/>
+      <c r="M4" s="28"/>
+      <c r="N4" s="28"/>
+      <c r="O4" s="28"/>
+      <c r="P4" s="28"/>
+      <c r="Q4" s="59" t="s">
+        <v>325</v>
+      </c>
+      <c r="R4" s="28"/>
+      <c r="S4" s="28"/>
+      <c r="T4" s="28"/>
+      <c r="U4" s="28"/>
+      <c r="V4" s="28"/>
+      <c r="W4" s="28"/>
+      <c r="X4" s="28"/>
+      <c r="Y4" s="28"/>
+      <c r="Z4" s="28"/>
+      <c r="AA4" s="28"/>
+      <c r="AB4" s="28"/>
+      <c r="AC4" s="28"/>
+      <c r="AD4" s="28"/>
+      <c r="AE4" s="28"/>
+      <c r="AF4" s="28"/>
+      <c r="AG4" s="28"/>
+      <c r="AH4" s="28"/>
+      <c r="AI4" s="28"/>
+      <c r="AJ4" s="28"/>
+      <c r="AK4" s="28"/>
+      <c r="AL4" s="28"/>
+      <c r="AM4" s="28"/>
+      <c r="AN4" s="28"/>
+      <c r="AO4" s="28"/>
+      <c r="AP4" s="28"/>
+      <c r="AQ4" s="28"/>
+      <c r="AR4" s="28"/>
+      <c r="AS4" s="28"/>
+      <c r="AT4" s="28"/>
+      <c r="AU4" s="28"/>
+      <c r="AV4" s="28"/>
+      <c r="AW4" s="28"/>
+      <c r="AX4" s="28"/>
+      <c r="AY4" s="28"/>
+      <c r="AZ4" s="28"/>
+      <c r="BA4" s="28"/>
+      <c r="BB4" s="28"/>
+      <c r="BC4" s="28"/>
+      <c r="BD4" s="28"/>
+      <c r="BE4" s="28"/>
+      <c r="BF4" s="28"/>
+      <c r="BG4" s="28"/>
+      <c r="BH4" s="28"/>
+      <c r="BI4" s="28"/>
+      <c r="BJ4" s="28"/>
+      <c r="BK4" s="28"/>
+      <c r="BL4" s="28"/>
+      <c r="BM4" s="28"/>
+      <c r="BN4" s="28"/>
+      <c r="BO4" s="28"/>
+      <c r="BP4" s="28"/>
+      <c r="BQ4" s="28"/>
+      <c r="BR4" s="28"/>
+      <c r="BS4" s="28"/>
+      <c r="BT4" s="28"/>
+      <c r="BU4" s="28"/>
+      <c r="BV4" s="28"/>
+      <c r="BW4" s="28"/>
+      <c r="BX4" s="28"/>
+      <c r="BY4" s="28"/>
+      <c r="BZ4" s="28"/>
+      <c r="CA4" s="28"/>
+      <c r="CB4" s="28"/>
+      <c r="CC4" s="28"/>
+      <c r="CD4" s="28"/>
+      <c r="CE4" s="28"/>
+      <c r="CF4" s="28"/>
+      <c r="CG4" s="28"/>
+      <c r="CH4" s="28"/>
+      <c r="CI4" s="28"/>
+      <c r="CJ4" s="28"/>
+      <c r="CK4" s="28"/>
+      <c r="CL4" s="29"/>
+    </row>
+    <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="33"/>
+      <c r="B5" s="34"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="34"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="34"/>
+      <c r="G5" s="65" t="s">
+        <v>209</v>
+      </c>
+      <c r="H5" s="36"/>
+      <c r="I5" s="36"/>
+      <c r="J5" s="36"/>
+      <c r="K5" s="36"/>
+      <c r="L5" s="36"/>
+      <c r="M5" s="36"/>
+      <c r="N5" s="36"/>
+      <c r="O5" s="36"/>
+      <c r="P5" s="36"/>
+      <c r="Q5" s="64" t="s">
+        <v>326</v>
+      </c>
+      <c r="R5" s="36"/>
+      <c r="S5" s="36"/>
+      <c r="T5" s="36"/>
+      <c r="U5" s="36"/>
+      <c r="V5" s="36"/>
+      <c r="W5" s="36"/>
+      <c r="X5" s="36"/>
+      <c r="Y5" s="36"/>
+      <c r="Z5" s="36"/>
+      <c r="AA5" s="36"/>
+      <c r="AB5" s="36"/>
+      <c r="AC5" s="36"/>
+      <c r="AD5" s="36"/>
+      <c r="AE5" s="36"/>
+      <c r="AF5" s="36"/>
+      <c r="AG5" s="36"/>
+      <c r="AH5" s="36"/>
+      <c r="AI5" s="36"/>
+      <c r="AJ5" s="36"/>
+      <c r="AK5" s="36"/>
+      <c r="AL5" s="36"/>
+      <c r="AM5" s="36"/>
+      <c r="AN5" s="36"/>
+      <c r="AO5" s="36"/>
+      <c r="AP5" s="36"/>
+      <c r="AQ5" s="36"/>
+      <c r="AR5" s="36"/>
+      <c r="AS5" s="36"/>
+      <c r="AT5" s="36"/>
+      <c r="AU5" s="36"/>
+      <c r="AV5" s="36"/>
+      <c r="AW5" s="36"/>
+      <c r="AX5" s="36"/>
+      <c r="AY5" s="36"/>
+      <c r="AZ5" s="36"/>
+      <c r="BA5" s="36"/>
+      <c r="BB5" s="36"/>
+      <c r="BC5" s="36"/>
+      <c r="BD5" s="36"/>
+      <c r="BE5" s="36"/>
+      <c r="BF5" s="36"/>
+      <c r="BG5" s="36"/>
+      <c r="BH5" s="36"/>
+      <c r="BI5" s="36"/>
+      <c r="BJ5" s="36"/>
+      <c r="BK5" s="36"/>
+      <c r="BL5" s="36"/>
+      <c r="BM5" s="36"/>
+      <c r="BN5" s="36"/>
+      <c r="BO5" s="36"/>
+      <c r="BP5" s="36"/>
+      <c r="BQ5" s="36"/>
+      <c r="BR5" s="36"/>
+      <c r="BS5" s="36"/>
+      <c r="BT5" s="36"/>
+      <c r="BU5" s="36"/>
+      <c r="BV5" s="36"/>
+      <c r="BW5" s="36"/>
+      <c r="BX5" s="36"/>
+      <c r="BY5" s="36"/>
+      <c r="BZ5" s="36"/>
+      <c r="CA5" s="36"/>
+      <c r="CB5" s="36"/>
+      <c r="CC5" s="36"/>
+      <c r="CD5" s="36"/>
+      <c r="CE5" s="36"/>
+      <c r="CF5" s="36"/>
+      <c r="CG5" s="36"/>
+      <c r="CH5" s="36"/>
+      <c r="CI5" s="36"/>
+      <c r="CJ5" s="36"/>
+      <c r="CK5" s="36"/>
+      <c r="CL5" s="37"/>
+    </row>
+    <row r="6" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
+      <c r="P6" s="1"/>
+      <c r="Q6" s="1"/>
+      <c r="R6" s="1"/>
+      <c r="S6" s="1"/>
+      <c r="T6" s="1"/>
+      <c r="U6" s="1"/>
+      <c r="V6" s="1"/>
+      <c r="W6" s="1"/>
+      <c r="X6" s="1"/>
+      <c r="Y6" s="1"/>
+      <c r="Z6" s="1"/>
+      <c r="AA6" s="1"/>
+      <c r="AB6" s="1"/>
+      <c r="AC6" s="1"/>
+      <c r="AD6" s="1"/>
+      <c r="AE6" s="1"/>
+      <c r="AF6" s="1"/>
+      <c r="AG6" s="1"/>
+      <c r="AH6" s="1"/>
+      <c r="AI6" s="1"/>
+      <c r="AJ6" s="1"/>
+      <c r="AK6" s="1"/>
+      <c r="AL6" s="1"/>
+      <c r="AM6" s="1"/>
+      <c r="AN6" s="1"/>
+      <c r="AO6" s="1"/>
+      <c r="AP6" s="1"/>
+      <c r="AQ6" s="1"/>
+      <c r="AR6" s="1"/>
+      <c r="AS6" s="1"/>
+      <c r="AT6" s="1"/>
+      <c r="AU6" s="1"/>
+      <c r="AV6" s="1"/>
+      <c r="AW6" s="1"/>
+      <c r="AX6" s="1"/>
+      <c r="AY6" s="1"/>
+      <c r="AZ6" s="1"/>
+      <c r="BA6" s="1"/>
+      <c r="BB6" s="1"/>
+      <c r="BC6" s="1"/>
+      <c r="BD6" s="1"/>
+      <c r="BE6" s="1"/>
+      <c r="BF6" s="1"/>
+      <c r="BG6" s="1"/>
+      <c r="BH6" s="1"/>
+      <c r="BI6" s="1"/>
+      <c r="BJ6" s="1"/>
+      <c r="BK6" s="1"/>
+      <c r="BL6" s="1"/>
+      <c r="BM6" s="1"/>
+      <c r="BN6" s="1"/>
+      <c r="BO6" s="1"/>
+      <c r="BP6" s="1"/>
+      <c r="BQ6" s="1"/>
+      <c r="BR6" s="1"/>
+      <c r="BS6" s="1"/>
+      <c r="BT6" s="1"/>
+      <c r="BU6" s="1"/>
+      <c r="BV6" s="1"/>
+      <c r="BW6" s="1"/>
+      <c r="BX6" s="1"/>
+      <c r="BY6" s="1"/>
+      <c r="BZ6" s="1"/>
+      <c r="CA6" s="1"/>
+      <c r="CB6" s="1"/>
+      <c r="CC6" s="1"/>
+      <c r="CD6" s="1"/>
+      <c r="CE6" s="1"/>
+      <c r="CF6" s="1"/>
+      <c r="CG6" s="1"/>
+      <c r="CH6" s="1"/>
+      <c r="CI6" s="1"/>
+      <c r="CJ6" s="1"/>
+      <c r="CK6" s="1"/>
+      <c r="CL6" s="1"/>
+    </row>
+    <row r="7" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="56" t="s">
+        <v>213</v>
+      </c>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="1"/>
+      <c r="R7" s="1"/>
+      <c r="S7" s="1"/>
+      <c r="T7" s="1"/>
+      <c r="U7" s="1"/>
+      <c r="V7" s="1"/>
+      <c r="W7" s="1"/>
+      <c r="X7" s="1"/>
+      <c r="Y7" s="1"/>
+      <c r="Z7" s="1"/>
+      <c r="AA7" s="1"/>
+      <c r="AB7" s="1"/>
+      <c r="AC7" s="1"/>
+      <c r="AD7" s="1"/>
+      <c r="AE7" s="1"/>
+      <c r="AF7" s="1"/>
+      <c r="AG7" s="1"/>
+      <c r="AH7" s="1"/>
+      <c r="AI7" s="1"/>
+      <c r="AJ7" s="1"/>
+      <c r="AK7" s="1"/>
+      <c r="AL7" s="1"/>
+      <c r="AM7" s="1"/>
+      <c r="AN7" s="1"/>
+      <c r="AO7" s="1"/>
+      <c r="AP7" s="1"/>
+      <c r="AQ7" s="1"/>
+      <c r="AR7" s="1"/>
+      <c r="AS7" s="1"/>
+      <c r="AT7" s="1"/>
+      <c r="AU7" s="1"/>
+      <c r="AV7" s="1"/>
+      <c r="AW7" s="1"/>
+      <c r="AX7" s="1"/>
+      <c r="AY7" s="1"/>
+      <c r="AZ7" s="1"/>
+      <c r="BA7" s="1"/>
+      <c r="BB7" s="1"/>
+      <c r="BC7" s="1"/>
+      <c r="BD7" s="1"/>
+      <c r="BE7" s="1"/>
+      <c r="BF7" s="1"/>
+      <c r="BG7" s="1"/>
+      <c r="BH7" s="1"/>
+      <c r="BI7" s="1"/>
+      <c r="BJ7" s="1"/>
+      <c r="BK7" s="1"/>
+      <c r="BL7" s="1"/>
+      <c r="BM7" s="1"/>
+      <c r="BN7" s="1"/>
+      <c r="BO7" s="1"/>
+      <c r="BP7" s="1"/>
+      <c r="BQ7" s="1"/>
+      <c r="BR7" s="1"/>
+      <c r="BS7" s="1"/>
+      <c r="BT7" s="1"/>
+      <c r="BU7" s="1"/>
+      <c r="BV7" s="1"/>
+      <c r="BW7" s="1"/>
+      <c r="BX7" s="1"/>
+      <c r="BY7" s="1"/>
+      <c r="BZ7" s="1"/>
+      <c r="CA7" s="1"/>
+      <c r="CB7" s="1"/>
+      <c r="CC7" s="1"/>
+      <c r="CD7" s="1"/>
+      <c r="CE7" s="1"/>
+      <c r="CF7" s="1"/>
+      <c r="CG7" s="1"/>
+      <c r="CH7" s="1"/>
+      <c r="CI7" s="1"/>
+      <c r="CJ7" s="1"/>
+      <c r="CK7" s="1"/>
+      <c r="CL7" s="1"/>
+    </row>
+    <row r="8" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="56" t="s">
+        <v>327</v>
+      </c>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="1"/>
+      <c r="P8" s="1"/>
+      <c r="Q8" s="1"/>
+      <c r="R8" s="1"/>
+      <c r="S8" s="1"/>
+      <c r="T8" s="1"/>
+      <c r="U8" s="1"/>
+      <c r="V8" s="1"/>
+      <c r="W8" s="1"/>
+      <c r="X8" s="1"/>
+      <c r="Y8" s="1"/>
+      <c r="Z8" s="1"/>
+      <c r="AA8" s="1"/>
+      <c r="AB8" s="1"/>
+      <c r="AC8" s="1"/>
+      <c r="AD8" s="1"/>
+      <c r="AE8" s="1"/>
+      <c r="AF8" s="1"/>
+      <c r="AG8" s="1"/>
+      <c r="AH8" s="1"/>
+      <c r="AI8" s="1"/>
+      <c r="AJ8" s="1"/>
+      <c r="AK8" s="1"/>
+      <c r="AL8" s="1"/>
+      <c r="AM8" s="1"/>
+      <c r="AN8" s="1"/>
+      <c r="AO8" s="1"/>
+      <c r="AP8" s="1"/>
+      <c r="AQ8" s="1"/>
+      <c r="AR8" s="1"/>
+      <c r="AS8" s="1"/>
+      <c r="AT8" s="1"/>
+      <c r="AU8" s="1"/>
+      <c r="AV8" s="1"/>
+      <c r="AW8" s="1"/>
+      <c r="AX8" s="1"/>
+      <c r="AY8" s="1"/>
+      <c r="AZ8" s="1"/>
+      <c r="BA8" s="1"/>
+      <c r="BB8" s="1"/>
+      <c r="BC8" s="1"/>
+      <c r="BD8" s="1"/>
+      <c r="BE8" s="1"/>
+      <c r="BF8" s="1"/>
+      <c r="BG8" s="1"/>
+      <c r="BH8" s="1"/>
+      <c r="BI8" s="1"/>
+      <c r="BJ8" s="1"/>
+      <c r="BK8" s="1"/>
+      <c r="BL8" s="1"/>
+      <c r="BM8" s="1"/>
+      <c r="BN8" s="1"/>
+      <c r="BO8" s="1"/>
+      <c r="BP8" s="1"/>
+      <c r="BQ8" s="1"/>
+      <c r="BR8" s="1"/>
+      <c r="BS8" s="1"/>
+      <c r="BT8" s="1"/>
+      <c r="BU8" s="1"/>
+      <c r="BV8" s="1"/>
+      <c r="BW8" s="1"/>
+      <c r="BX8" s="1"/>
+      <c r="BY8" s="1"/>
+      <c r="BZ8" s="1"/>
+      <c r="CA8" s="1"/>
+      <c r="CB8" s="1"/>
+      <c r="CC8" s="1"/>
+      <c r="CD8" s="1"/>
+      <c r="CE8" s="1"/>
+      <c r="CF8" s="1"/>
+      <c r="CG8" s="1"/>
+      <c r="CH8" s="1"/>
+      <c r="CI8" s="1"/>
+      <c r="CJ8" s="1"/>
+      <c r="CK8" s="1"/>
+      <c r="CL8" s="1"/>
+    </row>
+    <row r="9" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="62" t="s">
+        <v>214</v>
+      </c>
+      <c r="B9" s="39"/>
+      <c r="C9" s="39"/>
+      <c r="D9" s="39"/>
+      <c r="E9" s="39"/>
+      <c r="F9" s="39"/>
+      <c r="G9" s="39"/>
+      <c r="H9" s="39"/>
+      <c r="I9" s="39"/>
+      <c r="J9" s="39"/>
+      <c r="K9" s="39"/>
+      <c r="L9" s="39"/>
+      <c r="M9" s="39"/>
+      <c r="N9" s="39"/>
+      <c r="O9" s="39"/>
+      <c r="P9" s="39"/>
+      <c r="Q9" s="39"/>
+      <c r="R9" s="39"/>
+      <c r="S9" s="62" t="s">
+        <v>215</v>
+      </c>
+      <c r="T9" s="39"/>
+      <c r="U9" s="39"/>
+      <c r="V9" s="39"/>
+      <c r="W9" s="39"/>
+      <c r="X9" s="39"/>
+      <c r="Y9" s="39"/>
+      <c r="Z9" s="39"/>
+      <c r="AA9" s="39"/>
+      <c r="AB9" s="39"/>
+      <c r="AC9" s="39"/>
+      <c r="AD9" s="39"/>
+      <c r="AE9" s="39"/>
+      <c r="AF9" s="39"/>
+      <c r="AG9" s="39"/>
+      <c r="AH9" s="39"/>
+      <c r="AI9" s="39"/>
+      <c r="AJ9" s="39"/>
+      <c r="AK9" s="62" t="s">
+        <v>216</v>
+      </c>
+      <c r="AL9" s="39"/>
+      <c r="AM9" s="39"/>
+      <c r="AN9" s="39"/>
+      <c r="AO9" s="39"/>
+      <c r="AP9" s="39"/>
+      <c r="AQ9" s="39"/>
+      <c r="AR9" s="39"/>
+      <c r="AS9" s="39"/>
+      <c r="AT9" s="39"/>
+      <c r="AU9" s="39"/>
+      <c r="AV9" s="39"/>
+      <c r="AW9" s="39"/>
+      <c r="AX9" s="39"/>
+      <c r="AY9" s="39"/>
+      <c r="AZ9" s="39"/>
+      <c r="BA9" s="39"/>
+      <c r="BB9" s="39"/>
+      <c r="BC9" s="39"/>
+      <c r="BD9" s="39"/>
+      <c r="BE9" s="39"/>
+      <c r="BF9" s="39"/>
+      <c r="BG9" s="39"/>
+      <c r="BH9" s="39"/>
+      <c r="BI9" s="39"/>
+      <c r="BJ9" s="39"/>
+      <c r="BK9" s="39"/>
+      <c r="BL9" s="39"/>
+      <c r="BM9" s="39"/>
+      <c r="BN9" s="39"/>
+      <c r="BO9" s="39"/>
+      <c r="BP9" s="39"/>
+      <c r="BQ9" s="39"/>
+      <c r="BR9" s="39"/>
+      <c r="BS9" s="39"/>
+      <c r="BT9" s="39"/>
+      <c r="BU9" s="39"/>
+      <c r="BV9" s="39"/>
+      <c r="BW9" s="39"/>
+      <c r="BX9" s="39"/>
+      <c r="BY9" s="39"/>
+      <c r="BZ9" s="39"/>
+      <c r="CA9" s="39"/>
+      <c r="CB9" s="39"/>
+      <c r="CC9" s="39"/>
+      <c r="CD9" s="39"/>
+      <c r="CE9" s="39"/>
+      <c r="CF9" s="39"/>
+      <c r="CG9" s="39"/>
+      <c r="CH9" s="39"/>
+      <c r="CI9" s="39"/>
+      <c r="CJ9" s="39"/>
+      <c r="CK9" s="39"/>
+      <c r="CL9" s="49"/>
+    </row>
+    <row r="10" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="60" t="s">
+        <v>301</v>
+      </c>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="24"/>
+      <c r="J10" s="24"/>
+      <c r="K10" s="24"/>
+      <c r="L10" s="24"/>
+      <c r="M10" s="24"/>
+      <c r="N10" s="24"/>
+      <c r="O10" s="24"/>
+      <c r="P10" s="24"/>
+      <c r="Q10" s="24"/>
+      <c r="R10" s="24"/>
+      <c r="S10" s="31"/>
+      <c r="T10" s="24"/>
+      <c r="U10" s="24"/>
+      <c r="V10" s="24"/>
+      <c r="W10" s="24"/>
+      <c r="X10" s="24"/>
+      <c r="Y10" s="24"/>
+      <c r="Z10" s="24"/>
+      <c r="AA10" s="24"/>
+      <c r="AB10" s="24"/>
+      <c r="AC10" s="24"/>
+      <c r="AD10" s="24"/>
+      <c r="AE10" s="24"/>
+      <c r="AF10" s="24"/>
+      <c r="AG10" s="24"/>
+      <c r="AH10" s="24"/>
+      <c r="AI10" s="24"/>
+      <c r="AJ10" s="24"/>
+      <c r="AK10" s="68" t="s">
+        <v>328</v>
+      </c>
+      <c r="AL10" s="24"/>
+      <c r="AM10" s="24"/>
+      <c r="AN10" s="24"/>
+      <c r="AO10" s="24"/>
+      <c r="AP10" s="24"/>
+      <c r="AQ10" s="24"/>
+      <c r="AR10" s="24"/>
+      <c r="AS10" s="24"/>
+      <c r="AT10" s="24"/>
+      <c r="AU10" s="24"/>
+      <c r="AV10" s="24"/>
+      <c r="AW10" s="24"/>
+      <c r="AX10" s="24"/>
+      <c r="AY10" s="24"/>
+      <c r="AZ10" s="24"/>
+      <c r="BA10" s="24"/>
+      <c r="BB10" s="24"/>
+      <c r="BC10" s="24"/>
+      <c r="BD10" s="24"/>
+      <c r="BE10" s="24"/>
+      <c r="BF10" s="24"/>
+      <c r="BG10" s="24"/>
+      <c r="BH10" s="24"/>
+      <c r="BI10" s="24"/>
+      <c r="BJ10" s="24"/>
+      <c r="BK10" s="24"/>
+      <c r="BL10" s="24"/>
+      <c r="BM10" s="24"/>
+      <c r="BN10" s="24"/>
+      <c r="BO10" s="24"/>
+      <c r="BP10" s="24"/>
+      <c r="BQ10" s="24"/>
+      <c r="BR10" s="24"/>
+      <c r="BS10" s="24"/>
+      <c r="BT10" s="24"/>
+      <c r="BU10" s="24"/>
+      <c r="BV10" s="24"/>
+      <c r="BW10" s="24"/>
+      <c r="BX10" s="24"/>
+      <c r="BY10" s="24"/>
+      <c r="BZ10" s="24"/>
+      <c r="CA10" s="24"/>
+      <c r="CB10" s="24"/>
+      <c r="CC10" s="24"/>
+      <c r="CD10" s="24"/>
+      <c r="CE10" s="24"/>
+      <c r="CF10" s="24"/>
+      <c r="CG10" s="24"/>
+      <c r="CH10" s="24"/>
+      <c r="CI10" s="24"/>
+      <c r="CJ10" s="24"/>
+      <c r="CK10" s="24"/>
+      <c r="CL10" s="32"/>
+    </row>
+    <row r="11" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="62" t="s">
+        <v>113</v>
+      </c>
+      <c r="B11" s="39"/>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="39"/>
+      <c r="F11" s="39"/>
+      <c r="G11" s="40"/>
+      <c r="H11" s="41"/>
+      <c r="I11" s="41"/>
+      <c r="J11" s="41"/>
+      <c r="K11" s="41"/>
+      <c r="L11" s="41"/>
+      <c r="M11" s="41"/>
+      <c r="N11" s="41"/>
+      <c r="O11" s="41"/>
+      <c r="P11" s="41"/>
+      <c r="Q11" s="63" t="s">
+        <v>323</v>
+      </c>
+      <c r="R11" s="41"/>
+      <c r="S11" s="41"/>
+      <c r="T11" s="41"/>
+      <c r="U11" s="41"/>
+      <c r="V11" s="41"/>
+      <c r="W11" s="41"/>
+      <c r="X11" s="41"/>
+      <c r="Y11" s="41"/>
+      <c r="Z11" s="41"/>
+      <c r="AA11" s="41"/>
+      <c r="AB11" s="41"/>
+      <c r="AC11" s="41"/>
+      <c r="AD11" s="41"/>
+      <c r="AE11" s="41"/>
+      <c r="AF11" s="41"/>
+      <c r="AG11" s="41"/>
+      <c r="AH11" s="41"/>
+      <c r="AI11" s="41"/>
+      <c r="AJ11" s="41"/>
+      <c r="AK11" s="41"/>
+      <c r="AL11" s="41"/>
+      <c r="AM11" s="41"/>
+      <c r="AN11" s="41"/>
+      <c r="AO11" s="41"/>
+      <c r="AP11" s="41"/>
+      <c r="AQ11" s="41"/>
+      <c r="AR11" s="41"/>
+      <c r="AS11" s="41"/>
+      <c r="AT11" s="41"/>
+      <c r="AU11" s="41"/>
+      <c r="AV11" s="41"/>
+      <c r="AW11" s="41"/>
+      <c r="AX11" s="41"/>
+      <c r="AY11" s="41"/>
+      <c r="AZ11" s="41"/>
+      <c r="BA11" s="41"/>
+      <c r="BB11" s="41"/>
+      <c r="BC11" s="41"/>
+      <c r="BD11" s="41"/>
+      <c r="BE11" s="41"/>
+      <c r="BF11" s="41"/>
+      <c r="BG11" s="41"/>
+      <c r="BH11" s="41"/>
+      <c r="BI11" s="41"/>
+      <c r="BJ11" s="41"/>
+      <c r="BK11" s="41"/>
+      <c r="BL11" s="41"/>
+      <c r="BM11" s="41"/>
+      <c r="BN11" s="41"/>
+      <c r="BO11" s="41"/>
+      <c r="BP11" s="41"/>
+      <c r="BQ11" s="41"/>
+      <c r="BR11" s="41"/>
+      <c r="BS11" s="41"/>
+      <c r="BT11" s="41"/>
+      <c r="BU11" s="41"/>
+      <c r="BV11" s="41"/>
+      <c r="BW11" s="41"/>
+      <c r="BX11" s="41"/>
+      <c r="BY11" s="41"/>
+      <c r="BZ11" s="41"/>
+      <c r="CA11" s="41"/>
+      <c r="CB11" s="41"/>
+      <c r="CC11" s="41"/>
+      <c r="CD11" s="41"/>
+      <c r="CE11" s="41"/>
+      <c r="CF11" s="41"/>
+      <c r="CG11" s="41"/>
+      <c r="CH11" s="41"/>
+      <c r="CI11" s="41"/>
+      <c r="CJ11" s="41"/>
+      <c r="CK11" s="41"/>
+      <c r="CL11" s="42"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{177B7FDC-759C-4C00-BE29-1B3AB6C5E4C1}">
+  <dimension ref="A1:CL10"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="90" width="1.75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="56" t="s">
+        <v>202</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
+      <c r="AD1" s="1"/>
+      <c r="AE1" s="1"/>
+      <c r="AF1" s="1"/>
+      <c r="AG1" s="1"/>
+      <c r="AH1" s="1"/>
+      <c r="AI1" s="1"/>
+      <c r="AJ1" s="1"/>
+      <c r="AK1" s="1"/>
+      <c r="AL1" s="1"/>
+      <c r="AM1" s="1"/>
+      <c r="AN1" s="1"/>
+      <c r="AO1" s="1"/>
+      <c r="AP1" s="1"/>
+      <c r="AQ1" s="1"/>
+      <c r="AR1" s="1"/>
+      <c r="AS1" s="1"/>
+      <c r="AT1" s="1"/>
+      <c r="AU1" s="1"/>
+      <c r="AV1" s="1"/>
+      <c r="AW1" s="1"/>
+      <c r="AX1" s="1"/>
+      <c r="AY1" s="1"/>
+      <c r="AZ1" s="1"/>
+      <c r="BA1" s="1"/>
+      <c r="BB1" s="1"/>
+      <c r="BC1" s="1"/>
+      <c r="BD1" s="1"/>
+      <c r="BE1" s="1"/>
+      <c r="BF1" s="1"/>
+      <c r="BG1" s="1"/>
+      <c r="BH1" s="1"/>
+      <c r="BI1" s="1"/>
+      <c r="BJ1" s="1"/>
+      <c r="BK1" s="1"/>
+      <c r="BL1" s="1"/>
+      <c r="BM1" s="1"/>
+      <c r="BN1" s="1"/>
+      <c r="BO1" s="1"/>
+      <c r="BP1" s="1"/>
+      <c r="BQ1" s="1"/>
+      <c r="BR1" s="1"/>
+      <c r="BS1" s="1"/>
+      <c r="BT1" s="1"/>
+      <c r="BU1" s="1"/>
+      <c r="BV1" s="1"/>
+      <c r="BW1" s="1"/>
+      <c r="BX1" s="1"/>
+      <c r="BY1" s="1"/>
+      <c r="BZ1" s="1"/>
+      <c r="CA1" s="1"/>
+      <c r="CB1" s="1"/>
+      <c r="CC1" s="1"/>
+      <c r="CD1" s="1"/>
+      <c r="CE1" s="1"/>
+      <c r="CF1" s="1"/>
+      <c r="CG1" s="1"/>
+      <c r="CH1" s="1"/>
+      <c r="CI1" s="1"/>
+      <c r="CJ1" s="1"/>
+      <c r="CK1" s="1"/>
+      <c r="CL1" s="1"/>
+    </row>
+    <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="56" t="s">
+        <v>273</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1"/>
+      <c r="W2" s="1"/>
+      <c r="X2" s="1"/>
+      <c r="Y2" s="1"/>
+      <c r="Z2" s="1"/>
+      <c r="AA2" s="1"/>
+      <c r="AB2" s="1"/>
+      <c r="AC2" s="1"/>
+      <c r="AD2" s="1"/>
+      <c r="AE2" s="1"/>
+      <c r="AF2" s="1"/>
+      <c r="AG2" s="1"/>
+      <c r="AH2" s="1"/>
+      <c r="AI2" s="1"/>
+      <c r="AJ2" s="1"/>
+      <c r="AK2" s="1"/>
+      <c r="AL2" s="1"/>
+      <c r="AM2" s="1"/>
+      <c r="AN2" s="1"/>
+      <c r="AO2" s="1"/>
+      <c r="AP2" s="1"/>
+      <c r="AQ2" s="1"/>
+      <c r="AR2" s="1"/>
+      <c r="AS2" s="1"/>
+      <c r="AT2" s="1"/>
+      <c r="AU2" s="1"/>
+      <c r="AV2" s="1"/>
+      <c r="AW2" s="1"/>
+      <c r="AX2" s="1"/>
+      <c r="AY2" s="1"/>
+      <c r="AZ2" s="1"/>
+      <c r="BA2" s="1"/>
+      <c r="BB2" s="1"/>
+      <c r="BC2" s="1"/>
+      <c r="BD2" s="1"/>
+      <c r="BE2" s="1"/>
+      <c r="BF2" s="1"/>
+      <c r="BG2" s="1"/>
+      <c r="BH2" s="1"/>
+      <c r="BI2" s="1"/>
+      <c r="BJ2" s="1"/>
+      <c r="BK2" s="1"/>
+      <c r="BL2" s="1"/>
+      <c r="BM2" s="1"/>
+      <c r="BN2" s="1"/>
+      <c r="BO2" s="1"/>
+      <c r="BP2" s="1"/>
+      <c r="BQ2" s="1"/>
+      <c r="BR2" s="1"/>
+      <c r="BS2" s="1"/>
+      <c r="BT2" s="1"/>
+      <c r="BU2" s="1"/>
+      <c r="BV2" s="1"/>
+      <c r="BW2" s="1"/>
+      <c r="BX2" s="1"/>
+      <c r="BY2" s="1"/>
+      <c r="BZ2" s="1"/>
+      <c r="CA2" s="1"/>
+      <c r="CB2" s="1"/>
+      <c r="CC2" s="1"/>
+      <c r="CD2" s="1"/>
+      <c r="CE2" s="1"/>
+      <c r="CF2" s="1"/>
+      <c r="CG2" s="1"/>
+      <c r="CH2" s="1"/>
+      <c r="CI2" s="1"/>
+      <c r="CJ2" s="1"/>
+      <c r="CK2" s="1"/>
+      <c r="CL2" s="1"/>
+    </row>
+    <row r="3" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="57" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="58" t="s">
+        <v>57</v>
+      </c>
+      <c r="H3" s="28"/>
+      <c r="I3" s="28"/>
+      <c r="J3" s="28"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="28"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="28"/>
+      <c r="O3" s="59" t="s">
+        <v>58</v>
+      </c>
+      <c r="P3" s="28"/>
+      <c r="Q3" s="59" t="s">
+        <v>329</v>
+      </c>
+      <c r="R3" s="28"/>
+      <c r="S3" s="28"/>
+      <c r="T3" s="28"/>
+      <c r="U3" s="28"/>
+      <c r="V3" s="28"/>
+      <c r="W3" s="28"/>
+      <c r="X3" s="28"/>
+      <c r="Y3" s="28"/>
+      <c r="Z3" s="28"/>
+      <c r="AA3" s="28"/>
+      <c r="AB3" s="28"/>
+      <c r="AC3" s="28"/>
+      <c r="AD3" s="28"/>
+      <c r="AE3" s="59" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF3" s="59" t="s">
+        <v>330</v>
+      </c>
+      <c r="AG3" s="28"/>
+      <c r="AH3" s="28"/>
+      <c r="AI3" s="28"/>
+      <c r="AJ3" s="28"/>
+      <c r="AK3" s="28"/>
+      <c r="AL3" s="28"/>
+      <c r="AM3" s="28"/>
+      <c r="AN3" s="28"/>
+      <c r="AO3" s="28"/>
+      <c r="AP3" s="28"/>
+      <c r="AQ3" s="28"/>
+      <c r="AR3" s="28"/>
+      <c r="AS3" s="28"/>
+      <c r="AT3" s="28"/>
+      <c r="AU3" s="28"/>
+      <c r="AV3" s="28"/>
+      <c r="AW3" s="28"/>
+      <c r="AX3" s="28"/>
+      <c r="AY3" s="28"/>
+      <c r="AZ3" s="28"/>
+      <c r="BA3" s="28"/>
+      <c r="BB3" s="28"/>
+      <c r="BC3" s="28"/>
+      <c r="BD3" s="28"/>
+      <c r="BE3" s="28"/>
+      <c r="BF3" s="28"/>
+      <c r="BG3" s="28"/>
+      <c r="BH3" s="28"/>
+      <c r="BI3" s="28"/>
+      <c r="BJ3" s="28"/>
+      <c r="BK3" s="28"/>
+      <c r="BL3" s="28"/>
+      <c r="BM3" s="28"/>
+      <c r="BN3" s="28"/>
+      <c r="BO3" s="28"/>
+      <c r="BP3" s="28"/>
+      <c r="BQ3" s="28"/>
+      <c r="BR3" s="28"/>
+      <c r="BS3" s="28"/>
+      <c r="BT3" s="28"/>
+      <c r="BU3" s="28"/>
+      <c r="BV3" s="28"/>
+      <c r="BW3" s="28"/>
+      <c r="BX3" s="28"/>
+      <c r="BY3" s="28"/>
+      <c r="BZ3" s="28"/>
+      <c r="CA3" s="28"/>
+      <c r="CB3" s="28"/>
+      <c r="CC3" s="28"/>
+      <c r="CD3" s="28"/>
+      <c r="CE3" s="28"/>
+      <c r="CF3" s="28"/>
+      <c r="CG3" s="28"/>
+      <c r="CH3" s="28"/>
+      <c r="CI3" s="28"/>
+      <c r="CJ3" s="28"/>
+      <c r="CK3" s="28"/>
+      <c r="CL3" s="29"/>
+    </row>
+    <row r="4" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="62" t="s">
+        <v>113</v>
+      </c>
+      <c r="B4" s="39"/>
+      <c r="C4" s="39"/>
+      <c r="D4" s="39"/>
+      <c r="E4" s="39"/>
+      <c r="F4" s="39"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="41"/>
+      <c r="I4" s="41"/>
+      <c r="J4" s="41"/>
+      <c r="K4" s="41"/>
+      <c r="L4" s="41"/>
+      <c r="M4" s="41"/>
+      <c r="N4" s="41"/>
+      <c r="O4" s="41"/>
+      <c r="P4" s="41"/>
+      <c r="Q4" s="63" t="s">
+        <v>208</v>
+      </c>
+      <c r="R4" s="41"/>
+      <c r="S4" s="41"/>
+      <c r="T4" s="41"/>
+      <c r="U4" s="41"/>
+      <c r="V4" s="41"/>
+      <c r="W4" s="41"/>
+      <c r="X4" s="41"/>
+      <c r="Y4" s="41"/>
+      <c r="Z4" s="41"/>
+      <c r="AA4" s="41"/>
+      <c r="AB4" s="41"/>
+      <c r="AC4" s="41"/>
+      <c r="AD4" s="41"/>
+      <c r="AE4" s="41"/>
+      <c r="AF4" s="41"/>
+      <c r="AG4" s="41"/>
+      <c r="AH4" s="41"/>
+      <c r="AI4" s="41"/>
+      <c r="AJ4" s="41"/>
+      <c r="AK4" s="41"/>
+      <c r="AL4" s="41"/>
+      <c r="AM4" s="41"/>
+      <c r="AN4" s="41"/>
+      <c r="AO4" s="41"/>
+      <c r="AP4" s="41"/>
+      <c r="AQ4" s="41"/>
+      <c r="AR4" s="41"/>
+      <c r="AS4" s="41"/>
+      <c r="AT4" s="41"/>
+      <c r="AU4" s="41"/>
+      <c r="AV4" s="41"/>
+      <c r="AW4" s="41"/>
+      <c r="AX4" s="41"/>
+      <c r="AY4" s="41"/>
+      <c r="AZ4" s="41"/>
+      <c r="BA4" s="41"/>
+      <c r="BB4" s="41"/>
+      <c r="BC4" s="41"/>
+      <c r="BD4" s="41"/>
+      <c r="BE4" s="41"/>
+      <c r="BF4" s="41"/>
+      <c r="BG4" s="41"/>
+      <c r="BH4" s="41"/>
+      <c r="BI4" s="41"/>
+      <c r="BJ4" s="41"/>
+      <c r="BK4" s="41"/>
+      <c r="BL4" s="41"/>
+      <c r="BM4" s="41"/>
+      <c r="BN4" s="41"/>
+      <c r="BO4" s="41"/>
+      <c r="BP4" s="41"/>
+      <c r="BQ4" s="41"/>
+      <c r="BR4" s="41"/>
+      <c r="BS4" s="41"/>
+      <c r="BT4" s="41"/>
+      <c r="BU4" s="41"/>
+      <c r="BV4" s="41"/>
+      <c r="BW4" s="41"/>
+      <c r="BX4" s="41"/>
+      <c r="BY4" s="41"/>
+      <c r="BZ4" s="41"/>
+      <c r="CA4" s="41"/>
+      <c r="CB4" s="41"/>
+      <c r="CC4" s="41"/>
+      <c r="CD4" s="41"/>
+      <c r="CE4" s="41"/>
+      <c r="CF4" s="41"/>
+      <c r="CG4" s="41"/>
+      <c r="CH4" s="41"/>
+      <c r="CI4" s="41"/>
+      <c r="CJ4" s="41"/>
+      <c r="CK4" s="41"/>
+      <c r="CL4" s="42"/>
+    </row>
+    <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
+      <c r="P5" s="1"/>
+      <c r="Q5" s="1"/>
+      <c r="R5" s="1"/>
+      <c r="S5" s="1"/>
+      <c r="T5" s="1"/>
+      <c r="U5" s="1"/>
+      <c r="V5" s="1"/>
+      <c r="W5" s="1"/>
+      <c r="X5" s="1"/>
+      <c r="Y5" s="1"/>
+      <c r="Z5" s="1"/>
+      <c r="AA5" s="1"/>
+      <c r="AB5" s="1"/>
+      <c r="AC5" s="1"/>
+      <c r="AD5" s="1"/>
+      <c r="AE5" s="1"/>
+      <c r="AF5" s="1"/>
+      <c r="AG5" s="1"/>
+      <c r="AH5" s="1"/>
+      <c r="AI5" s="1"/>
+      <c r="AJ5" s="1"/>
+      <c r="AK5" s="1"/>
+      <c r="AL5" s="1"/>
+      <c r="AM5" s="1"/>
+      <c r="AN5" s="1"/>
+      <c r="AO5" s="1"/>
+      <c r="AP5" s="1"/>
+      <c r="AQ5" s="1"/>
+      <c r="AR5" s="1"/>
+      <c r="AS5" s="1"/>
+      <c r="AT5" s="1"/>
+      <c r="AU5" s="1"/>
+      <c r="AV5" s="1"/>
+      <c r="AW5" s="1"/>
+      <c r="AX5" s="1"/>
+      <c r="AY5" s="1"/>
+      <c r="AZ5" s="1"/>
+      <c r="BA5" s="1"/>
+      <c r="BB5" s="1"/>
+      <c r="BC5" s="1"/>
+      <c r="BD5" s="1"/>
+      <c r="BE5" s="1"/>
+      <c r="BF5" s="1"/>
+      <c r="BG5" s="1"/>
+      <c r="BH5" s="1"/>
+      <c r="BI5" s="1"/>
+      <c r="BJ5" s="1"/>
+      <c r="BK5" s="1"/>
+      <c r="BL5" s="1"/>
+      <c r="BM5" s="1"/>
+      <c r="BN5" s="1"/>
+      <c r="BO5" s="1"/>
+      <c r="BP5" s="1"/>
+      <c r="BQ5" s="1"/>
+      <c r="BR5" s="1"/>
+      <c r="BS5" s="1"/>
+      <c r="BT5" s="1"/>
+      <c r="BU5" s="1"/>
+      <c r="BV5" s="1"/>
+      <c r="BW5" s="1"/>
+      <c r="BX5" s="1"/>
+      <c r="BY5" s="1"/>
+      <c r="BZ5" s="1"/>
+      <c r="CA5" s="1"/>
+      <c r="CB5" s="1"/>
+      <c r="CC5" s="1"/>
+      <c r="CD5" s="1"/>
+      <c r="CE5" s="1"/>
+      <c r="CF5" s="1"/>
+      <c r="CG5" s="1"/>
+      <c r="CH5" s="1"/>
+      <c r="CI5" s="1"/>
+      <c r="CJ5" s="1"/>
+      <c r="CK5" s="1"/>
+      <c r="CL5" s="1"/>
+    </row>
+    <row r="6" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="56" t="s">
+        <v>213</v>
+      </c>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
+      <c r="P6" s="1"/>
+      <c r="Q6" s="1"/>
+      <c r="R6" s="1"/>
+      <c r="S6" s="1"/>
+      <c r="T6" s="1"/>
+      <c r="U6" s="1"/>
+      <c r="V6" s="1"/>
+      <c r="W6" s="1"/>
+      <c r="X6" s="1"/>
+      <c r="Y6" s="1"/>
+      <c r="Z6" s="1"/>
+      <c r="AA6" s="1"/>
+      <c r="AB6" s="1"/>
+      <c r="AC6" s="1"/>
+      <c r="AD6" s="1"/>
+      <c r="AE6" s="1"/>
+      <c r="AF6" s="1"/>
+      <c r="AG6" s="1"/>
+      <c r="AH6" s="1"/>
+      <c r="AI6" s="1"/>
+      <c r="AJ6" s="1"/>
+      <c r="AK6" s="1"/>
+      <c r="AL6" s="1"/>
+      <c r="AM6" s="1"/>
+      <c r="AN6" s="1"/>
+      <c r="AO6" s="1"/>
+      <c r="AP6" s="1"/>
+      <c r="AQ6" s="1"/>
+      <c r="AR6" s="1"/>
+      <c r="AS6" s="1"/>
+      <c r="AT6" s="1"/>
+      <c r="AU6" s="1"/>
+      <c r="AV6" s="1"/>
+      <c r="AW6" s="1"/>
+      <c r="AX6" s="1"/>
+      <c r="AY6" s="1"/>
+      <c r="AZ6" s="1"/>
+      <c r="BA6" s="1"/>
+      <c r="BB6" s="1"/>
+      <c r="BC6" s="1"/>
+      <c r="BD6" s="1"/>
+      <c r="BE6" s="1"/>
+      <c r="BF6" s="1"/>
+      <c r="BG6" s="1"/>
+      <c r="BH6" s="1"/>
+      <c r="BI6" s="1"/>
+      <c r="BJ6" s="1"/>
+      <c r="BK6" s="1"/>
+      <c r="BL6" s="1"/>
+      <c r="BM6" s="1"/>
+      <c r="BN6" s="1"/>
+      <c r="BO6" s="1"/>
+      <c r="BP6" s="1"/>
+      <c r="BQ6" s="1"/>
+      <c r="BR6" s="1"/>
+      <c r="BS6" s="1"/>
+      <c r="BT6" s="1"/>
+      <c r="BU6" s="1"/>
+      <c r="BV6" s="1"/>
+      <c r="BW6" s="1"/>
+      <c r="BX6" s="1"/>
+      <c r="BY6" s="1"/>
+      <c r="BZ6" s="1"/>
+      <c r="CA6" s="1"/>
+      <c r="CB6" s="1"/>
+      <c r="CC6" s="1"/>
+      <c r="CD6" s="1"/>
+      <c r="CE6" s="1"/>
+      <c r="CF6" s="1"/>
+      <c r="CG6" s="1"/>
+      <c r="CH6" s="1"/>
+      <c r="CI6" s="1"/>
+      <c r="CJ6" s="1"/>
+      <c r="CK6" s="1"/>
+      <c r="CL6" s="1"/>
+    </row>
+    <row r="7" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="56" t="s">
+        <v>311</v>
+      </c>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="1"/>
+      <c r="R7" s="1"/>
+      <c r="S7" s="1"/>
+      <c r="T7" s="1"/>
+      <c r="U7" s="1"/>
+      <c r="V7" s="1"/>
+      <c r="W7" s="1"/>
+      <c r="X7" s="1"/>
+      <c r="Y7" s="1"/>
+      <c r="Z7" s="1"/>
+      <c r="AA7" s="1"/>
+      <c r="AB7" s="1"/>
+      <c r="AC7" s="1"/>
+      <c r="AD7" s="1"/>
+      <c r="AE7" s="1"/>
+      <c r="AF7" s="1"/>
+      <c r="AG7" s="1"/>
+      <c r="AH7" s="1"/>
+      <c r="AI7" s="1"/>
+      <c r="AJ7" s="1"/>
+      <c r="AK7" s="1"/>
+      <c r="AL7" s="1"/>
+      <c r="AM7" s="1"/>
+      <c r="AN7" s="1"/>
+      <c r="AO7" s="1"/>
+      <c r="AP7" s="1"/>
+      <c r="AQ7" s="1"/>
+      <c r="AR7" s="1"/>
+      <c r="AS7" s="1"/>
+      <c r="AT7" s="1"/>
+      <c r="AU7" s="1"/>
+      <c r="AV7" s="1"/>
+      <c r="AW7" s="1"/>
+      <c r="AX7" s="1"/>
+      <c r="AY7" s="1"/>
+      <c r="AZ7" s="1"/>
+      <c r="BA7" s="1"/>
+      <c r="BB7" s="1"/>
+      <c r="BC7" s="1"/>
+      <c r="BD7" s="1"/>
+      <c r="BE7" s="1"/>
+      <c r="BF7" s="1"/>
+      <c r="BG7" s="1"/>
+      <c r="BH7" s="1"/>
+      <c r="BI7" s="1"/>
+      <c r="BJ7" s="1"/>
+      <c r="BK7" s="1"/>
+      <c r="BL7" s="1"/>
+      <c r="BM7" s="1"/>
+      <c r="BN7" s="1"/>
+      <c r="BO7" s="1"/>
+      <c r="BP7" s="1"/>
+      <c r="BQ7" s="1"/>
+      <c r="BR7" s="1"/>
+      <c r="BS7" s="1"/>
+      <c r="BT7" s="1"/>
+      <c r="BU7" s="1"/>
+      <c r="BV7" s="1"/>
+      <c r="BW7" s="1"/>
+      <c r="BX7" s="1"/>
+      <c r="BY7" s="1"/>
+      <c r="BZ7" s="1"/>
+      <c r="CA7" s="1"/>
+      <c r="CB7" s="1"/>
+      <c r="CC7" s="1"/>
+      <c r="CD7" s="1"/>
+      <c r="CE7" s="1"/>
+      <c r="CF7" s="1"/>
+      <c r="CG7" s="1"/>
+      <c r="CH7" s="1"/>
+      <c r="CI7" s="1"/>
+      <c r="CJ7" s="1"/>
+      <c r="CK7" s="1"/>
+      <c r="CL7" s="1"/>
+    </row>
+    <row r="8" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="62" t="s">
+        <v>214</v>
+      </c>
+      <c r="B8" s="39"/>
+      <c r="C8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="39"/>
+      <c r="I8" s="39"/>
+      <c r="J8" s="39"/>
+      <c r="K8" s="39"/>
+      <c r="L8" s="39"/>
+      <c r="M8" s="39"/>
+      <c r="N8" s="39"/>
+      <c r="O8" s="39"/>
+      <c r="P8" s="39"/>
+      <c r="Q8" s="39"/>
+      <c r="R8" s="39"/>
+      <c r="S8" s="62" t="s">
+        <v>215</v>
+      </c>
+      <c r="T8" s="39"/>
+      <c r="U8" s="39"/>
+      <c r="V8" s="39"/>
+      <c r="W8" s="39"/>
+      <c r="X8" s="39"/>
+      <c r="Y8" s="39"/>
+      <c r="Z8" s="39"/>
+      <c r="AA8" s="39"/>
+      <c r="AB8" s="39"/>
+      <c r="AC8" s="39"/>
+      <c r="AD8" s="39"/>
+      <c r="AE8" s="39"/>
+      <c r="AF8" s="39"/>
+      <c r="AG8" s="39"/>
+      <c r="AH8" s="39"/>
+      <c r="AI8" s="39"/>
+      <c r="AJ8" s="39"/>
+      <c r="AK8" s="62" t="s">
+        <v>216</v>
+      </c>
+      <c r="AL8" s="39"/>
+      <c r="AM8" s="39"/>
+      <c r="AN8" s="39"/>
+      <c r="AO8" s="39"/>
+      <c r="AP8" s="39"/>
+      <c r="AQ8" s="39"/>
+      <c r="AR8" s="39"/>
+      <c r="AS8" s="39"/>
+      <c r="AT8" s="39"/>
+      <c r="AU8" s="39"/>
+      <c r="AV8" s="39"/>
+      <c r="AW8" s="39"/>
+      <c r="AX8" s="39"/>
+      <c r="AY8" s="39"/>
+      <c r="AZ8" s="39"/>
+      <c r="BA8" s="39"/>
+      <c r="BB8" s="39"/>
+      <c r="BC8" s="39"/>
+      <c r="BD8" s="39"/>
+      <c r="BE8" s="39"/>
+      <c r="BF8" s="39"/>
+      <c r="BG8" s="39"/>
+      <c r="BH8" s="39"/>
+      <c r="BI8" s="39"/>
+      <c r="BJ8" s="39"/>
+      <c r="BK8" s="39"/>
+      <c r="BL8" s="39"/>
+      <c r="BM8" s="39"/>
+      <c r="BN8" s="39"/>
+      <c r="BO8" s="39"/>
+      <c r="BP8" s="39"/>
+      <c r="BQ8" s="39"/>
+      <c r="BR8" s="39"/>
+      <c r="BS8" s="39"/>
+      <c r="BT8" s="39"/>
+      <c r="BU8" s="39"/>
+      <c r="BV8" s="39"/>
+      <c r="BW8" s="39"/>
+      <c r="BX8" s="39"/>
+      <c r="BY8" s="39"/>
+      <c r="BZ8" s="39"/>
+      <c r="CA8" s="39"/>
+      <c r="CB8" s="39"/>
+      <c r="CC8" s="39"/>
+      <c r="CD8" s="39"/>
+      <c r="CE8" s="39"/>
+      <c r="CF8" s="39"/>
+      <c r="CG8" s="39"/>
+      <c r="CH8" s="39"/>
+      <c r="CI8" s="39"/>
+      <c r="CJ8" s="39"/>
+      <c r="CK8" s="39"/>
+      <c r="CL8" s="49"/>
+    </row>
+    <row r="9" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="60" t="s">
+        <v>301</v>
+      </c>
+      <c r="B9" s="24"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="24"/>
+      <c r="H9" s="24"/>
+      <c r="I9" s="24"/>
+      <c r="J9" s="24"/>
+      <c r="K9" s="24"/>
+      <c r="L9" s="24"/>
+      <c r="M9" s="24"/>
+      <c r="N9" s="24"/>
+      <c r="O9" s="24"/>
+      <c r="P9" s="24"/>
+      <c r="Q9" s="24"/>
+      <c r="R9" s="24"/>
+      <c r="S9" s="31"/>
+      <c r="T9" s="24"/>
+      <c r="U9" s="24"/>
+      <c r="V9" s="24"/>
+      <c r="W9" s="24"/>
+      <c r="X9" s="24"/>
+      <c r="Y9" s="24"/>
+      <c r="Z9" s="24"/>
+      <c r="AA9" s="24"/>
+      <c r="AB9" s="24"/>
+      <c r="AC9" s="24"/>
+      <c r="AD9" s="24"/>
+      <c r="AE9" s="24"/>
+      <c r="AF9" s="24"/>
+      <c r="AG9" s="24"/>
+      <c r="AH9" s="24"/>
+      <c r="AI9" s="24"/>
+      <c r="AJ9" s="24"/>
+      <c r="AK9" s="68" t="s">
+        <v>331</v>
+      </c>
+      <c r="AL9" s="24"/>
+      <c r="AM9" s="24"/>
+      <c r="AN9" s="24"/>
+      <c r="AO9" s="24"/>
+      <c r="AP9" s="24"/>
+      <c r="AQ9" s="24"/>
+      <c r="AR9" s="24"/>
+      <c r="AS9" s="24"/>
+      <c r="AT9" s="24"/>
+      <c r="AU9" s="24"/>
+      <c r="AV9" s="24"/>
+      <c r="AW9" s="24"/>
+      <c r="AX9" s="24"/>
+      <c r="AY9" s="24"/>
+      <c r="AZ9" s="24"/>
+      <c r="BA9" s="24"/>
+      <c r="BB9" s="24"/>
+      <c r="BC9" s="24"/>
+      <c r="BD9" s="24"/>
+      <c r="BE9" s="24"/>
+      <c r="BF9" s="24"/>
+      <c r="BG9" s="24"/>
+      <c r="BH9" s="24"/>
+      <c r="BI9" s="24"/>
+      <c r="BJ9" s="24"/>
+      <c r="BK9" s="24"/>
+      <c r="BL9" s="24"/>
+      <c r="BM9" s="24"/>
+      <c r="BN9" s="24"/>
+      <c r="BO9" s="24"/>
+      <c r="BP9" s="24"/>
+      <c r="BQ9" s="24"/>
+      <c r="BR9" s="24"/>
+      <c r="BS9" s="24"/>
+      <c r="BT9" s="24"/>
+      <c r="BU9" s="24"/>
+      <c r="BV9" s="24"/>
+      <c r="BW9" s="24"/>
+      <c r="BX9" s="24"/>
+      <c r="BY9" s="24"/>
+      <c r="BZ9" s="24"/>
+      <c r="CA9" s="24"/>
+      <c r="CB9" s="24"/>
+      <c r="CC9" s="24"/>
+      <c r="CD9" s="24"/>
+      <c r="CE9" s="24"/>
+      <c r="CF9" s="24"/>
+      <c r="CG9" s="24"/>
+      <c r="CH9" s="24"/>
+      <c r="CI9" s="24"/>
+      <c r="CJ9" s="24"/>
+      <c r="CK9" s="24"/>
+      <c r="CL9" s="32"/>
+    </row>
+    <row r="10" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="62" t="s">
+        <v>113</v>
+      </c>
+      <c r="B10" s="39"/>
+      <c r="C10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="39"/>
+      <c r="F10" s="39"/>
+      <c r="G10" s="40"/>
+      <c r="H10" s="41"/>
+      <c r="I10" s="41"/>
+      <c r="J10" s="41"/>
+      <c r="K10" s="41"/>
+      <c r="L10" s="41"/>
+      <c r="M10" s="41"/>
+      <c r="N10" s="41"/>
+      <c r="O10" s="41"/>
+      <c r="P10" s="41"/>
+      <c r="Q10" s="63" t="s">
+        <v>332</v>
+      </c>
+      <c r="R10" s="41"/>
+      <c r="S10" s="41"/>
+      <c r="T10" s="41"/>
+      <c r="U10" s="41"/>
+      <c r="V10" s="41"/>
+      <c r="W10" s="41"/>
+      <c r="X10" s="41"/>
+      <c r="Y10" s="41"/>
+      <c r="Z10" s="41"/>
+      <c r="AA10" s="41"/>
+      <c r="AB10" s="41"/>
+      <c r="AC10" s="41"/>
+      <c r="AD10" s="41"/>
+      <c r="AE10" s="41"/>
+      <c r="AF10" s="41"/>
+      <c r="AG10" s="41"/>
+      <c r="AH10" s="41"/>
+      <c r="AI10" s="41"/>
+      <c r="AJ10" s="41"/>
+      <c r="AK10" s="41"/>
+      <c r="AL10" s="41"/>
+      <c r="AM10" s="41"/>
+      <c r="AN10" s="41"/>
+      <c r="AO10" s="41"/>
+      <c r="AP10" s="41"/>
+      <c r="AQ10" s="41"/>
+      <c r="AR10" s="41"/>
+      <c r="AS10" s="41"/>
+      <c r="AT10" s="41"/>
+      <c r="AU10" s="41"/>
+      <c r="AV10" s="41"/>
+      <c r="AW10" s="41"/>
+      <c r="AX10" s="41"/>
+      <c r="AY10" s="41"/>
+      <c r="AZ10" s="41"/>
+      <c r="BA10" s="41"/>
+      <c r="BB10" s="41"/>
+      <c r="BC10" s="41"/>
+      <c r="BD10" s="41"/>
+      <c r="BE10" s="41"/>
+      <c r="BF10" s="41"/>
+      <c r="BG10" s="41"/>
+      <c r="BH10" s="41"/>
+      <c r="BI10" s="41"/>
+      <c r="BJ10" s="41"/>
+      <c r="BK10" s="41"/>
+      <c r="BL10" s="41"/>
+      <c r="BM10" s="41"/>
+      <c r="BN10" s="41"/>
+      <c r="BO10" s="41"/>
+      <c r="BP10" s="41"/>
+      <c r="BQ10" s="41"/>
+      <c r="BR10" s="41"/>
+      <c r="BS10" s="41"/>
+      <c r="BT10" s="41"/>
+      <c r="BU10" s="41"/>
+      <c r="BV10" s="41"/>
+      <c r="BW10" s="41"/>
+      <c r="BX10" s="41"/>
+      <c r="BY10" s="41"/>
+      <c r="BZ10" s="41"/>
+      <c r="CA10" s="41"/>
+      <c r="CB10" s="41"/>
+      <c r="CC10" s="41"/>
+      <c r="CD10" s="41"/>
+      <c r="CE10" s="41"/>
+      <c r="CF10" s="41"/>
+      <c r="CG10" s="41"/>
+      <c r="CH10" s="41"/>
+      <c r="CI10" s="41"/>
+      <c r="CJ10" s="41"/>
+      <c r="CK10" s="41"/>
+      <c r="CL10" s="42"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{999AD117-9C89-46B1-8101-80FE48E37FB4}">
+  <dimension ref="A1:CL10"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="90" width="1.75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="56" t="s">
+        <v>202</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
+      <c r="AD1" s="1"/>
+      <c r="AE1" s="1"/>
+      <c r="AF1" s="1"/>
+      <c r="AG1" s="1"/>
+      <c r="AH1" s="1"/>
+      <c r="AI1" s="1"/>
+      <c r="AJ1" s="1"/>
+      <c r="AK1" s="1"/>
+      <c r="AL1" s="1"/>
+      <c r="AM1" s="1"/>
+      <c r="AN1" s="1"/>
+      <c r="AO1" s="1"/>
+      <c r="AP1" s="1"/>
+      <c r="AQ1" s="1"/>
+      <c r="AR1" s="1"/>
+      <c r="AS1" s="1"/>
+      <c r="AT1" s="1"/>
+      <c r="AU1" s="1"/>
+      <c r="AV1" s="1"/>
+      <c r="AW1" s="1"/>
+      <c r="AX1" s="1"/>
+      <c r="AY1" s="1"/>
+      <c r="AZ1" s="1"/>
+      <c r="BA1" s="1"/>
+      <c r="BB1" s="1"/>
+      <c r="BC1" s="1"/>
+      <c r="BD1" s="1"/>
+      <c r="BE1" s="1"/>
+      <c r="BF1" s="1"/>
+      <c r="BG1" s="1"/>
+      <c r="BH1" s="1"/>
+      <c r="BI1" s="1"/>
+      <c r="BJ1" s="1"/>
+      <c r="BK1" s="1"/>
+      <c r="BL1" s="1"/>
+      <c r="BM1" s="1"/>
+      <c r="BN1" s="1"/>
+      <c r="BO1" s="1"/>
+      <c r="BP1" s="1"/>
+      <c r="BQ1" s="1"/>
+      <c r="BR1" s="1"/>
+      <c r="BS1" s="1"/>
+      <c r="BT1" s="1"/>
+      <c r="BU1" s="1"/>
+      <c r="BV1" s="1"/>
+      <c r="BW1" s="1"/>
+      <c r="BX1" s="1"/>
+      <c r="BY1" s="1"/>
+      <c r="BZ1" s="1"/>
+      <c r="CA1" s="1"/>
+      <c r="CB1" s="1"/>
+      <c r="CC1" s="1"/>
+      <c r="CD1" s="1"/>
+      <c r="CE1" s="1"/>
+      <c r="CF1" s="1"/>
+      <c r="CG1" s="1"/>
+      <c r="CH1" s="1"/>
+      <c r="CI1" s="1"/>
+      <c r="CJ1" s="1"/>
+      <c r="CK1" s="1"/>
+      <c r="CL1" s="1"/>
+    </row>
+    <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="56" t="s">
+        <v>333</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1"/>
+      <c r="W2" s="1"/>
+      <c r="X2" s="1"/>
+      <c r="Y2" s="1"/>
+      <c r="Z2" s="1"/>
+      <c r="AA2" s="1"/>
+      <c r="AB2" s="1"/>
+      <c r="AC2" s="1"/>
+      <c r="AD2" s="1"/>
+      <c r="AE2" s="1"/>
+      <c r="AF2" s="1"/>
+      <c r="AG2" s="1"/>
+      <c r="AH2" s="1"/>
+      <c r="AI2" s="1"/>
+      <c r="AJ2" s="1"/>
+      <c r="AK2" s="1"/>
+      <c r="AL2" s="1"/>
+      <c r="AM2" s="1"/>
+      <c r="AN2" s="1"/>
+      <c r="AO2" s="1"/>
+      <c r="AP2" s="1"/>
+      <c r="AQ2" s="1"/>
+      <c r="AR2" s="1"/>
+      <c r="AS2" s="1"/>
+      <c r="AT2" s="1"/>
+      <c r="AU2" s="1"/>
+      <c r="AV2" s="1"/>
+      <c r="AW2" s="1"/>
+      <c r="AX2" s="1"/>
+      <c r="AY2" s="1"/>
+      <c r="AZ2" s="1"/>
+      <c r="BA2" s="1"/>
+      <c r="BB2" s="1"/>
+      <c r="BC2" s="1"/>
+      <c r="BD2" s="1"/>
+      <c r="BE2" s="1"/>
+      <c r="BF2" s="1"/>
+      <c r="BG2" s="1"/>
+      <c r="BH2" s="1"/>
+      <c r="BI2" s="1"/>
+      <c r="BJ2" s="1"/>
+      <c r="BK2" s="1"/>
+      <c r="BL2" s="1"/>
+      <c r="BM2" s="1"/>
+      <c r="BN2" s="1"/>
+      <c r="BO2" s="1"/>
+      <c r="BP2" s="1"/>
+      <c r="BQ2" s="1"/>
+      <c r="BR2" s="1"/>
+      <c r="BS2" s="1"/>
+      <c r="BT2" s="1"/>
+      <c r="BU2" s="1"/>
+      <c r="BV2" s="1"/>
+      <c r="BW2" s="1"/>
+      <c r="BX2" s="1"/>
+      <c r="BY2" s="1"/>
+      <c r="BZ2" s="1"/>
+      <c r="CA2" s="1"/>
+      <c r="CB2" s="1"/>
+      <c r="CC2" s="1"/>
+      <c r="CD2" s="1"/>
+      <c r="CE2" s="1"/>
+      <c r="CF2" s="1"/>
+      <c r="CG2" s="1"/>
+      <c r="CH2" s="1"/>
+      <c r="CI2" s="1"/>
+      <c r="CJ2" s="1"/>
+      <c r="CK2" s="1"/>
+      <c r="CL2" s="1"/>
+    </row>
+    <row r="3" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="57" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="58" t="s">
+        <v>57</v>
+      </c>
+      <c r="H3" s="28"/>
+      <c r="I3" s="28"/>
+      <c r="J3" s="28"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="28"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="28"/>
+      <c r="O3" s="59" t="s">
+        <v>58</v>
+      </c>
+      <c r="P3" s="28"/>
+      <c r="Q3" s="59" t="s">
+        <v>316</v>
+      </c>
+      <c r="R3" s="28"/>
+      <c r="S3" s="28"/>
+      <c r="T3" s="28"/>
+      <c r="U3" s="28"/>
+      <c r="V3" s="28"/>
+      <c r="W3" s="28"/>
+      <c r="X3" s="28"/>
+      <c r="Y3" s="28"/>
+      <c r="Z3" s="28"/>
+      <c r="AA3" s="28"/>
+      <c r="AB3" s="28"/>
+      <c r="AC3" s="28"/>
+      <c r="AD3" s="28"/>
+      <c r="AE3" s="28"/>
+      <c r="AF3" s="28"/>
+      <c r="AG3" s="28"/>
+      <c r="AH3" s="28"/>
+      <c r="AI3" s="28"/>
+      <c r="AJ3" s="28"/>
+      <c r="AK3" s="28"/>
+      <c r="AL3" s="28"/>
+      <c r="AM3" s="28"/>
+      <c r="AN3" s="28"/>
+      <c r="AO3" s="28"/>
+      <c r="AP3" s="28"/>
+      <c r="AQ3" s="28"/>
+      <c r="AR3" s="28"/>
+      <c r="AS3" s="28"/>
+      <c r="AT3" s="28"/>
+      <c r="AU3" s="28"/>
+      <c r="AV3" s="28"/>
+      <c r="AW3" s="28"/>
+      <c r="AX3" s="28"/>
+      <c r="AY3" s="28"/>
+      <c r="AZ3" s="28"/>
+      <c r="BA3" s="28"/>
+      <c r="BB3" s="28"/>
+      <c r="BC3" s="28"/>
+      <c r="BD3" s="28"/>
+      <c r="BE3" s="28"/>
+      <c r="BF3" s="28"/>
+      <c r="BG3" s="28"/>
+      <c r="BH3" s="28"/>
+      <c r="BI3" s="28"/>
+      <c r="BJ3" s="28"/>
+      <c r="BK3" s="28"/>
+      <c r="BL3" s="28"/>
+      <c r="BM3" s="28"/>
+      <c r="BN3" s="28"/>
+      <c r="BO3" s="28"/>
+      <c r="BP3" s="28"/>
+      <c r="BQ3" s="28"/>
+      <c r="BR3" s="28"/>
+      <c r="BS3" s="28"/>
+      <c r="BT3" s="28"/>
+      <c r="BU3" s="28"/>
+      <c r="BV3" s="28"/>
+      <c r="BW3" s="28"/>
+      <c r="BX3" s="28"/>
+      <c r="BY3" s="28"/>
+      <c r="BZ3" s="28"/>
+      <c r="CA3" s="28"/>
+      <c r="CB3" s="28"/>
+      <c r="CC3" s="28"/>
+      <c r="CD3" s="28"/>
+      <c r="CE3" s="28"/>
+      <c r="CF3" s="28"/>
+      <c r="CG3" s="28"/>
+      <c r="CH3" s="28"/>
+      <c r="CI3" s="28"/>
+      <c r="CJ3" s="28"/>
+      <c r="CK3" s="28"/>
+      <c r="CL3" s="29"/>
+    </row>
+    <row r="4" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="62" t="s">
+        <v>113</v>
+      </c>
+      <c r="B4" s="39"/>
+      <c r="C4" s="39"/>
+      <c r="D4" s="39"/>
+      <c r="E4" s="39"/>
+      <c r="F4" s="39"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="41"/>
+      <c r="I4" s="41"/>
+      <c r="J4" s="41"/>
+      <c r="K4" s="41"/>
+      <c r="L4" s="41"/>
+      <c r="M4" s="41"/>
+      <c r="N4" s="41"/>
+      <c r="O4" s="41"/>
+      <c r="P4" s="41"/>
+      <c r="Q4" s="63" t="s">
+        <v>334</v>
+      </c>
+      <c r="R4" s="41"/>
+      <c r="S4" s="41"/>
+      <c r="T4" s="41"/>
+      <c r="U4" s="41"/>
+      <c r="V4" s="41"/>
+      <c r="W4" s="41"/>
+      <c r="X4" s="41"/>
+      <c r="Y4" s="41"/>
+      <c r="Z4" s="41"/>
+      <c r="AA4" s="41"/>
+      <c r="AB4" s="41"/>
+      <c r="AC4" s="41"/>
+      <c r="AD4" s="41"/>
+      <c r="AE4" s="41"/>
+      <c r="AF4" s="41"/>
+      <c r="AG4" s="41"/>
+      <c r="AH4" s="41"/>
+      <c r="AI4" s="41"/>
+      <c r="AJ4" s="41"/>
+      <c r="AK4" s="41"/>
+      <c r="AL4" s="41"/>
+      <c r="AM4" s="41"/>
+      <c r="AN4" s="41"/>
+      <c r="AO4" s="41"/>
+      <c r="AP4" s="41"/>
+      <c r="AQ4" s="41"/>
+      <c r="AR4" s="41"/>
+      <c r="AS4" s="41"/>
+      <c r="AT4" s="41"/>
+      <c r="AU4" s="41"/>
+      <c r="AV4" s="41"/>
+      <c r="AW4" s="41"/>
+      <c r="AX4" s="41"/>
+      <c r="AY4" s="41"/>
+      <c r="AZ4" s="41"/>
+      <c r="BA4" s="41"/>
+      <c r="BB4" s="41"/>
+      <c r="BC4" s="41"/>
+      <c r="BD4" s="41"/>
+      <c r="BE4" s="41"/>
+      <c r="BF4" s="41"/>
+      <c r="BG4" s="41"/>
+      <c r="BH4" s="41"/>
+      <c r="BI4" s="41"/>
+      <c r="BJ4" s="41"/>
+      <c r="BK4" s="41"/>
+      <c r="BL4" s="41"/>
+      <c r="BM4" s="41"/>
+      <c r="BN4" s="41"/>
+      <c r="BO4" s="41"/>
+      <c r="BP4" s="41"/>
+      <c r="BQ4" s="41"/>
+      <c r="BR4" s="41"/>
+      <c r="BS4" s="41"/>
+      <c r="BT4" s="41"/>
+      <c r="BU4" s="41"/>
+      <c r="BV4" s="41"/>
+      <c r="BW4" s="41"/>
+      <c r="BX4" s="41"/>
+      <c r="BY4" s="41"/>
+      <c r="BZ4" s="41"/>
+      <c r="CA4" s="41"/>
+      <c r="CB4" s="41"/>
+      <c r="CC4" s="41"/>
+      <c r="CD4" s="41"/>
+      <c r="CE4" s="41"/>
+      <c r="CF4" s="41"/>
+      <c r="CG4" s="41"/>
+      <c r="CH4" s="41"/>
+      <c r="CI4" s="41"/>
+      <c r="CJ4" s="41"/>
+      <c r="CK4" s="41"/>
+      <c r="CL4" s="42"/>
+    </row>
+    <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
+      <c r="P5" s="1"/>
+      <c r="Q5" s="1"/>
+      <c r="R5" s="1"/>
+      <c r="S5" s="1"/>
+      <c r="T5" s="1"/>
+      <c r="U5" s="1"/>
+      <c r="V5" s="1"/>
+      <c r="W5" s="1"/>
+      <c r="X5" s="1"/>
+      <c r="Y5" s="1"/>
+      <c r="Z5" s="1"/>
+      <c r="AA5" s="1"/>
+      <c r="AB5" s="1"/>
+      <c r="AC5" s="1"/>
+      <c r="AD5" s="1"/>
+      <c r="AE5" s="1"/>
+      <c r="AF5" s="1"/>
+      <c r="AG5" s="1"/>
+      <c r="AH5" s="1"/>
+      <c r="AI5" s="1"/>
+      <c r="AJ5" s="1"/>
+      <c r="AK5" s="1"/>
+      <c r="AL5" s="1"/>
+      <c r="AM5" s="1"/>
+      <c r="AN5" s="1"/>
+      <c r="AO5" s="1"/>
+      <c r="AP5" s="1"/>
+      <c r="AQ5" s="1"/>
+      <c r="AR5" s="1"/>
+      <c r="AS5" s="1"/>
+      <c r="AT5" s="1"/>
+      <c r="AU5" s="1"/>
+      <c r="AV5" s="1"/>
+      <c r="AW5" s="1"/>
+      <c r="AX5" s="1"/>
+      <c r="AY5" s="1"/>
+      <c r="AZ5" s="1"/>
+      <c r="BA5" s="1"/>
+      <c r="BB5" s="1"/>
+      <c r="BC5" s="1"/>
+      <c r="BD5" s="1"/>
+      <c r="BE5" s="1"/>
+      <c r="BF5" s="1"/>
+      <c r="BG5" s="1"/>
+      <c r="BH5" s="1"/>
+      <c r="BI5" s="1"/>
+      <c r="BJ5" s="1"/>
+      <c r="BK5" s="1"/>
+      <c r="BL5" s="1"/>
+      <c r="BM5" s="1"/>
+      <c r="BN5" s="1"/>
+      <c r="BO5" s="1"/>
+      <c r="BP5" s="1"/>
+      <c r="BQ5" s="1"/>
+      <c r="BR5" s="1"/>
+      <c r="BS5" s="1"/>
+      <c r="BT5" s="1"/>
+      <c r="BU5" s="1"/>
+      <c r="BV5" s="1"/>
+      <c r="BW5" s="1"/>
+      <c r="BX5" s="1"/>
+      <c r="BY5" s="1"/>
+      <c r="BZ5" s="1"/>
+      <c r="CA5" s="1"/>
+      <c r="CB5" s="1"/>
+      <c r="CC5" s="1"/>
+      <c r="CD5" s="1"/>
+      <c r="CE5" s="1"/>
+      <c r="CF5" s="1"/>
+      <c r="CG5" s="1"/>
+      <c r="CH5" s="1"/>
+      <c r="CI5" s="1"/>
+      <c r="CJ5" s="1"/>
+      <c r="CK5" s="1"/>
+      <c r="CL5" s="1"/>
+    </row>
+    <row r="6" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="56" t="s">
+        <v>213</v>
+      </c>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
+      <c r="P6" s="1"/>
+      <c r="Q6" s="1"/>
+      <c r="R6" s="1"/>
+      <c r="S6" s="1"/>
+      <c r="T6" s="1"/>
+      <c r="U6" s="1"/>
+      <c r="V6" s="1"/>
+      <c r="W6" s="1"/>
+      <c r="X6" s="1"/>
+      <c r="Y6" s="1"/>
+      <c r="Z6" s="1"/>
+      <c r="AA6" s="1"/>
+      <c r="AB6" s="1"/>
+      <c r="AC6" s="1"/>
+      <c r="AD6" s="1"/>
+      <c r="AE6" s="1"/>
+      <c r="AF6" s="1"/>
+      <c r="AG6" s="1"/>
+      <c r="AH6" s="1"/>
+      <c r="AI6" s="1"/>
+      <c r="AJ6" s="1"/>
+      <c r="AK6" s="1"/>
+      <c r="AL6" s="1"/>
+      <c r="AM6" s="1"/>
+      <c r="AN6" s="1"/>
+      <c r="AO6" s="1"/>
+      <c r="AP6" s="1"/>
+      <c r="AQ6" s="1"/>
+      <c r="AR6" s="1"/>
+      <c r="AS6" s="1"/>
+      <c r="AT6" s="1"/>
+      <c r="AU6" s="1"/>
+      <c r="AV6" s="1"/>
+      <c r="AW6" s="1"/>
+      <c r="AX6" s="1"/>
+      <c r="AY6" s="1"/>
+      <c r="AZ6" s="1"/>
+      <c r="BA6" s="1"/>
+      <c r="BB6" s="1"/>
+      <c r="BC6" s="1"/>
+      <c r="BD6" s="1"/>
+      <c r="BE6" s="1"/>
+      <c r="BF6" s="1"/>
+      <c r="BG6" s="1"/>
+      <c r="BH6" s="1"/>
+      <c r="BI6" s="1"/>
+      <c r="BJ6" s="1"/>
+      <c r="BK6" s="1"/>
+      <c r="BL6" s="1"/>
+      <c r="BM6" s="1"/>
+      <c r="BN6" s="1"/>
+      <c r="BO6" s="1"/>
+      <c r="BP6" s="1"/>
+      <c r="BQ6" s="1"/>
+      <c r="BR6" s="1"/>
+      <c r="BS6" s="1"/>
+      <c r="BT6" s="1"/>
+      <c r="BU6" s="1"/>
+      <c r="BV6" s="1"/>
+      <c r="BW6" s="1"/>
+      <c r="BX6" s="1"/>
+      <c r="BY6" s="1"/>
+      <c r="BZ6" s="1"/>
+      <c r="CA6" s="1"/>
+      <c r="CB6" s="1"/>
+      <c r="CC6" s="1"/>
+      <c r="CD6" s="1"/>
+      <c r="CE6" s="1"/>
+      <c r="CF6" s="1"/>
+      <c r="CG6" s="1"/>
+      <c r="CH6" s="1"/>
+      <c r="CI6" s="1"/>
+      <c r="CJ6" s="1"/>
+      <c r="CK6" s="1"/>
+      <c r="CL6" s="1"/>
+    </row>
+    <row r="7" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="56" t="s">
+        <v>311</v>
+      </c>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="1"/>
+      <c r="R7" s="1"/>
+      <c r="S7" s="1"/>
+      <c r="T7" s="1"/>
+      <c r="U7" s="1"/>
+      <c r="V7" s="1"/>
+      <c r="W7" s="1"/>
+      <c r="X7" s="1"/>
+      <c r="Y7" s="1"/>
+      <c r="Z7" s="1"/>
+      <c r="AA7" s="1"/>
+      <c r="AB7" s="1"/>
+      <c r="AC7" s="1"/>
+      <c r="AD7" s="1"/>
+      <c r="AE7" s="1"/>
+      <c r="AF7" s="1"/>
+      <c r="AG7" s="1"/>
+      <c r="AH7" s="1"/>
+      <c r="AI7" s="1"/>
+      <c r="AJ7" s="1"/>
+      <c r="AK7" s="1"/>
+      <c r="AL7" s="1"/>
+      <c r="AM7" s="1"/>
+      <c r="AN7" s="1"/>
+      <c r="AO7" s="1"/>
+      <c r="AP7" s="1"/>
+      <c r="AQ7" s="1"/>
+      <c r="AR7" s="1"/>
+      <c r="AS7" s="1"/>
+      <c r="AT7" s="1"/>
+      <c r="AU7" s="1"/>
+      <c r="AV7" s="1"/>
+      <c r="AW7" s="1"/>
+      <c r="AX7" s="1"/>
+      <c r="AY7" s="1"/>
+      <c r="AZ7" s="1"/>
+      <c r="BA7" s="1"/>
+      <c r="BB7" s="1"/>
+      <c r="BC7" s="1"/>
+      <c r="BD7" s="1"/>
+      <c r="BE7" s="1"/>
+      <c r="BF7" s="1"/>
+      <c r="BG7" s="1"/>
+      <c r="BH7" s="1"/>
+      <c r="BI7" s="1"/>
+      <c r="BJ7" s="1"/>
+      <c r="BK7" s="1"/>
+      <c r="BL7" s="1"/>
+      <c r="BM7" s="1"/>
+      <c r="BN7" s="1"/>
+      <c r="BO7" s="1"/>
+      <c r="BP7" s="1"/>
+      <c r="BQ7" s="1"/>
+      <c r="BR7" s="1"/>
+      <c r="BS7" s="1"/>
+      <c r="BT7" s="1"/>
+      <c r="BU7" s="1"/>
+      <c r="BV7" s="1"/>
+      <c r="BW7" s="1"/>
+      <c r="BX7" s="1"/>
+      <c r="BY7" s="1"/>
+      <c r="BZ7" s="1"/>
+      <c r="CA7" s="1"/>
+      <c r="CB7" s="1"/>
+      <c r="CC7" s="1"/>
+      <c r="CD7" s="1"/>
+      <c r="CE7" s="1"/>
+      <c r="CF7" s="1"/>
+      <c r="CG7" s="1"/>
+      <c r="CH7" s="1"/>
+      <c r="CI7" s="1"/>
+      <c r="CJ7" s="1"/>
+      <c r="CK7" s="1"/>
+      <c r="CL7" s="1"/>
+    </row>
+    <row r="8" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="62" t="s">
+        <v>214</v>
+      </c>
+      <c r="B8" s="39"/>
+      <c r="C8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="39"/>
+      <c r="I8" s="39"/>
+      <c r="J8" s="39"/>
+      <c r="K8" s="39"/>
+      <c r="L8" s="39"/>
+      <c r="M8" s="39"/>
+      <c r="N8" s="39"/>
+      <c r="O8" s="39"/>
+      <c r="P8" s="39"/>
+      <c r="Q8" s="39"/>
+      <c r="R8" s="39"/>
+      <c r="S8" s="62" t="s">
+        <v>215</v>
+      </c>
+      <c r="T8" s="39"/>
+      <c r="U8" s="39"/>
+      <c r="V8" s="39"/>
+      <c r="W8" s="39"/>
+      <c r="X8" s="39"/>
+      <c r="Y8" s="39"/>
+      <c r="Z8" s="39"/>
+      <c r="AA8" s="39"/>
+      <c r="AB8" s="39"/>
+      <c r="AC8" s="39"/>
+      <c r="AD8" s="39"/>
+      <c r="AE8" s="39"/>
+      <c r="AF8" s="39"/>
+      <c r="AG8" s="39"/>
+      <c r="AH8" s="39"/>
+      <c r="AI8" s="39"/>
+      <c r="AJ8" s="39"/>
+      <c r="AK8" s="62" t="s">
+        <v>216</v>
+      </c>
+      <c r="AL8" s="39"/>
+      <c r="AM8" s="39"/>
+      <c r="AN8" s="39"/>
+      <c r="AO8" s="39"/>
+      <c r="AP8" s="39"/>
+      <c r="AQ8" s="39"/>
+      <c r="AR8" s="39"/>
+      <c r="AS8" s="39"/>
+      <c r="AT8" s="39"/>
+      <c r="AU8" s="39"/>
+      <c r="AV8" s="39"/>
+      <c r="AW8" s="39"/>
+      <c r="AX8" s="39"/>
+      <c r="AY8" s="39"/>
+      <c r="AZ8" s="39"/>
+      <c r="BA8" s="39"/>
+      <c r="BB8" s="39"/>
+      <c r="BC8" s="39"/>
+      <c r="BD8" s="39"/>
+      <c r="BE8" s="39"/>
+      <c r="BF8" s="39"/>
+      <c r="BG8" s="39"/>
+      <c r="BH8" s="39"/>
+      <c r="BI8" s="39"/>
+      <c r="BJ8" s="39"/>
+      <c r="BK8" s="39"/>
+      <c r="BL8" s="39"/>
+      <c r="BM8" s="39"/>
+      <c r="BN8" s="39"/>
+      <c r="BO8" s="39"/>
+      <c r="BP8" s="39"/>
+      <c r="BQ8" s="39"/>
+      <c r="BR8" s="39"/>
+      <c r="BS8" s="39"/>
+      <c r="BT8" s="39"/>
+      <c r="BU8" s="39"/>
+      <c r="BV8" s="39"/>
+      <c r="BW8" s="39"/>
+      <c r="BX8" s="39"/>
+      <c r="BY8" s="39"/>
+      <c r="BZ8" s="39"/>
+      <c r="CA8" s="39"/>
+      <c r="CB8" s="39"/>
+      <c r="CC8" s="39"/>
+      <c r="CD8" s="39"/>
+      <c r="CE8" s="39"/>
+      <c r="CF8" s="39"/>
+      <c r="CG8" s="39"/>
+      <c r="CH8" s="39"/>
+      <c r="CI8" s="39"/>
+      <c r="CJ8" s="39"/>
+      <c r="CK8" s="39"/>
+      <c r="CL8" s="49"/>
+    </row>
+    <row r="9" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="60" t="s">
+        <v>301</v>
+      </c>
+      <c r="B9" s="24"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="24"/>
+      <c r="H9" s="24"/>
+      <c r="I9" s="24"/>
+      <c r="J9" s="24"/>
+      <c r="K9" s="24"/>
+      <c r="L9" s="24"/>
+      <c r="M9" s="24"/>
+      <c r="N9" s="24"/>
+      <c r="O9" s="24"/>
+      <c r="P9" s="24"/>
+      <c r="Q9" s="24"/>
+      <c r="R9" s="24"/>
+      <c r="S9" s="31"/>
+      <c r="T9" s="24"/>
+      <c r="U9" s="24"/>
+      <c r="V9" s="24"/>
+      <c r="W9" s="24"/>
+      <c r="X9" s="24"/>
+      <c r="Y9" s="24"/>
+      <c r="Z9" s="24"/>
+      <c r="AA9" s="24"/>
+      <c r="AB9" s="24"/>
+      <c r="AC9" s="24"/>
+      <c r="AD9" s="24"/>
+      <c r="AE9" s="24"/>
+      <c r="AF9" s="24"/>
+      <c r="AG9" s="24"/>
+      <c r="AH9" s="24"/>
+      <c r="AI9" s="24"/>
+      <c r="AJ9" s="24"/>
+      <c r="AK9" s="68" t="s">
+        <v>335</v>
+      </c>
+      <c r="AL9" s="24"/>
+      <c r="AM9" s="24"/>
+      <c r="AN9" s="24"/>
+      <c r="AO9" s="24"/>
+      <c r="AP9" s="24"/>
+      <c r="AQ9" s="24"/>
+      <c r="AR9" s="24"/>
+      <c r="AS9" s="24"/>
+      <c r="AT9" s="24"/>
+      <c r="AU9" s="24"/>
+      <c r="AV9" s="24"/>
+      <c r="AW9" s="24"/>
+      <c r="AX9" s="24"/>
+      <c r="AY9" s="24"/>
+      <c r="AZ9" s="24"/>
+      <c r="BA9" s="24"/>
+      <c r="BB9" s="24"/>
+      <c r="BC9" s="24"/>
+      <c r="BD9" s="24"/>
+      <c r="BE9" s="24"/>
+      <c r="BF9" s="24"/>
+      <c r="BG9" s="24"/>
+      <c r="BH9" s="24"/>
+      <c r="BI9" s="24"/>
+      <c r="BJ9" s="24"/>
+      <c r="BK9" s="24"/>
+      <c r="BL9" s="24"/>
+      <c r="BM9" s="24"/>
+      <c r="BN9" s="24"/>
+      <c r="BO9" s="24"/>
+      <c r="BP9" s="24"/>
+      <c r="BQ9" s="24"/>
+      <c r="BR9" s="24"/>
+      <c r="BS9" s="24"/>
+      <c r="BT9" s="24"/>
+      <c r="BU9" s="24"/>
+      <c r="BV9" s="24"/>
+      <c r="BW9" s="24"/>
+      <c r="BX9" s="24"/>
+      <c r="BY9" s="24"/>
+      <c r="BZ9" s="24"/>
+      <c r="CA9" s="24"/>
+      <c r="CB9" s="24"/>
+      <c r="CC9" s="24"/>
+      <c r="CD9" s="24"/>
+      <c r="CE9" s="24"/>
+      <c r="CF9" s="24"/>
+      <c r="CG9" s="24"/>
+      <c r="CH9" s="24"/>
+      <c r="CI9" s="24"/>
+      <c r="CJ9" s="24"/>
+      <c r="CK9" s="24"/>
+      <c r="CL9" s="32"/>
+    </row>
+    <row r="10" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="62" t="s">
+        <v>113</v>
+      </c>
+      <c r="B10" s="39"/>
+      <c r="C10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="39"/>
+      <c r="F10" s="39"/>
+      <c r="G10" s="40"/>
+      <c r="H10" s="41"/>
+      <c r="I10" s="41"/>
+      <c r="J10" s="41"/>
+      <c r="K10" s="41"/>
+      <c r="L10" s="41"/>
+      <c r="M10" s="41"/>
+      <c r="N10" s="41"/>
+      <c r="O10" s="41"/>
+      <c r="P10" s="41"/>
+      <c r="Q10" s="63" t="s">
+        <v>336</v>
+      </c>
+      <c r="R10" s="41"/>
+      <c r="S10" s="41"/>
+      <c r="T10" s="41"/>
+      <c r="U10" s="41"/>
+      <c r="V10" s="41"/>
+      <c r="W10" s="41"/>
+      <c r="X10" s="41"/>
+      <c r="Y10" s="41"/>
+      <c r="Z10" s="41"/>
+      <c r="AA10" s="41"/>
+      <c r="AB10" s="41"/>
+      <c r="AC10" s="41"/>
+      <c r="AD10" s="41"/>
+      <c r="AE10" s="41"/>
+      <c r="AF10" s="41"/>
+      <c r="AG10" s="41"/>
+      <c r="AH10" s="41"/>
+      <c r="AI10" s="41"/>
+      <c r="AJ10" s="41"/>
+      <c r="AK10" s="41"/>
+      <c r="AL10" s="41"/>
+      <c r="AM10" s="41"/>
+      <c r="AN10" s="41"/>
+      <c r="AO10" s="41"/>
+      <c r="AP10" s="41"/>
+      <c r="AQ10" s="41"/>
+      <c r="AR10" s="41"/>
+      <c r="AS10" s="41"/>
+      <c r="AT10" s="41"/>
+      <c r="AU10" s="41"/>
+      <c r="AV10" s="41"/>
+      <c r="AW10" s="41"/>
+      <c r="AX10" s="41"/>
+      <c r="AY10" s="41"/>
+      <c r="AZ10" s="41"/>
+      <c r="BA10" s="41"/>
+      <c r="BB10" s="41"/>
+      <c r="BC10" s="41"/>
+      <c r="BD10" s="41"/>
+      <c r="BE10" s="41"/>
+      <c r="BF10" s="41"/>
+      <c r="BG10" s="41"/>
+      <c r="BH10" s="41"/>
+      <c r="BI10" s="41"/>
+      <c r="BJ10" s="41"/>
+      <c r="BK10" s="41"/>
+      <c r="BL10" s="41"/>
+      <c r="BM10" s="41"/>
+      <c r="BN10" s="41"/>
+      <c r="BO10" s="41"/>
+      <c r="BP10" s="41"/>
+      <c r="BQ10" s="41"/>
+      <c r="BR10" s="41"/>
+      <c r="BS10" s="41"/>
+      <c r="BT10" s="41"/>
+      <c r="BU10" s="41"/>
+      <c r="BV10" s="41"/>
+      <c r="BW10" s="41"/>
+      <c r="BX10" s="41"/>
+      <c r="BY10" s="41"/>
+      <c r="BZ10" s="41"/>
+      <c r="CA10" s="41"/>
+      <c r="CB10" s="41"/>
+      <c r="CC10" s="41"/>
+      <c r="CD10" s="41"/>
+      <c r="CE10" s="41"/>
+      <c r="CF10" s="41"/>
+      <c r="CG10" s="41"/>
+      <c r="CH10" s="41"/>
+      <c r="CI10" s="41"/>
+      <c r="CJ10" s="41"/>
+      <c r="CK10" s="41"/>
+      <c r="CL10" s="42"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF9898D0-97E7-4BA1-9234-259483827CA2}">
   <sheetPr codeName="Sheet1"/>

</xml_diff>

<commit_message>
test: add CASE placement golden expectations
</commit_message>
<xml_diff>
--- a/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
+++ b/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\Macro\SqlAnalyzerFormatter-feature\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E5C72A-2503-4A5D-82D1-23E55461E8E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47C06EDD-BFC2-4AE0-978A-2B3EB4587545}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="63" activeTab="69" xr2:uid="{41A826B0-B2A2-4DC8-9B04-8EFBE807DC37}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="67" activeTab="73" xr2:uid="{41A826B0-B2A2-4DC8-9B04-8EFBE807DC37}"/>
   </bookViews>
   <sheets>
     <sheet name="SEL-064" sheetId="66" r:id="rId1"/>
@@ -83,6 +83,11 @@
     <sheet name="SEL-068" sheetId="71" r:id="rId68"/>
     <sheet name="SEL-069" sheetId="72" r:id="rId69"/>
     <sheet name="SEL-070" sheetId="73" r:id="rId70"/>
+    <sheet name="SEL-071" sheetId="74" r:id="rId71"/>
+    <sheet name="SEL-072" sheetId="75" r:id="rId72"/>
+    <sheet name="SEL-073" sheetId="76" r:id="rId73"/>
+    <sheet name="SEL-075" sheetId="78" r:id="rId74"/>
+    <sheet name="SEL-074" sheetId="77" r:id="rId75"/>
   </sheets>
   <calcPr calcId="191029" calcMode="manual"/>
   <extLst>
@@ -94,7 +99,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1244" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1300" uniqueCount="355">
   <si>
     <t>＜DB入出力項目定義＞</t>
     <rPh sb="3" eb="10">
@@ -1465,6 +1470,33 @@
   <si>
     <t>eligible_flag</t>
   </si>
+  <si>
+    <t>tb1.削除日時 IS NULL</t>
+  </si>
+  <si>
+    <t>AND tb1.有効区分 = 1 → 'ACTIVE'</t>
+  </si>
+  <si>
+    <t>それ以外 → 'INACTIVE'</t>
+  </si>
+  <si>
+    <t>@active = 1 → 'ACTIVE'</t>
+  </si>
+  <si>
+    <t>@all_rows = 1 → 100</t>
+  </si>
+  <si>
+    <t>それ以外 → 10</t>
+  </si>
+  <si>
+    <t>offset (CASE結果) rows fetch next 20 rows only</t>
+  </si>
+  <si>
+    <t>@skip_rows = 1 → 10</t>
+  </si>
+  <si>
+    <t>tb1.状態 = 'ACTIVE' → 1</t>
+  </si>
 </sst>
 </file>
 
@@ -2327,6 +2359,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8342C69F-C45D-427C-B3AA-1E8F3561DA3F}">
+  <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:CL8"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
@@ -13185,6 +13218,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7594DDE4-F031-431B-9740-0D95F5F84FA4}">
+  <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:CL13"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
@@ -21267,6 +21301,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C83768B-411E-4F12-B21D-9496B5CFD80D}">
+  <sheetPr codeName="Sheet16"/>
   <dimension ref="A1:CL12"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
@@ -27441,6 +27476,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B8EFC88-B32B-464F-B271-9A0BD6A61532}">
+  <sheetPr codeName="Sheet61"/>
   <dimension ref="A1:CL7"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
@@ -32999,6 +33035,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A45D62D-68F5-47F4-82BD-406753D82392}">
+  <sheetPr codeName="Sheet62"/>
   <dimension ref="A1:CL24"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
@@ -41089,6 +41126,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B4E52F0-775C-4BA3-8E6B-04DBE455867D}">
+  <sheetPr codeName="Sheet63"/>
   <dimension ref="A1:CL13"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
@@ -44341,6 +44379,7 @@
 
 <file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{125A3CC4-F32F-4AFC-B49F-2EB086F762F7}">
+  <sheetPr codeName="Sheet64"/>
   <dimension ref="A1:CL11"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
@@ -45405,6 +45444,7 @@
 
 <file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{177B7FDC-759C-4C00-BE29-1B3AB6C5E4C1}">
+  <sheetPr codeName="Sheet65"/>
   <dimension ref="A1:CL10"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
@@ -46377,6 +46417,7 @@
 
 <file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{999AD117-9C89-46B1-8101-80FE48E37FB4}">
+  <sheetPr codeName="Sheet66"/>
   <dimension ref="A1:CL10"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
@@ -47345,6 +47386,7 @@
 
 <file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB0D1930-9AB8-4E8B-A69C-E8A464241E29}">
+  <sheetPr codeName="Sheet67"/>
   <dimension ref="A1:CL10"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
@@ -48319,6 +48361,7 @@
 
 <file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98123E36-DEC7-4BA3-914F-651666C56468}">
+  <sheetPr codeName="Sheet68"/>
   <dimension ref="A1:CL4"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
@@ -48721,6 +48764,7 @@
 
 <file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7D2694E-D810-4A8F-9E88-6BF6AE47836A}">
+  <sheetPr codeName="Sheet69"/>
   <dimension ref="A1:CL6"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
@@ -50758,6 +50802,7 @@
 
 <file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13E13F0B-BD68-436F-AC4B-0DE79A71FA29}">
+  <sheetPr codeName="Sheet70"/>
   <dimension ref="A1:CL5"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
@@ -51243,6 +51288,2584 @@
       <c r="CJ5" s="36"/>
       <c r="CK5" s="36"/>
       <c r="CL5" s="37"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30AB51C2-4CAF-40D2-90C0-05BD312EBAB8}">
+  <sheetPr codeName="Sheet71"/>
+  <dimension ref="A1:CL6"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="90" width="1.75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="56" t="s">
+        <v>213</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
+      <c r="AD1" s="1"/>
+      <c r="AE1" s="1"/>
+      <c r="AF1" s="1"/>
+      <c r="AG1" s="1"/>
+      <c r="AH1" s="1"/>
+      <c r="AI1" s="1"/>
+      <c r="AJ1" s="1"/>
+      <c r="AK1" s="1"/>
+      <c r="AL1" s="1"/>
+      <c r="AM1" s="1"/>
+      <c r="AN1" s="1"/>
+      <c r="AO1" s="1"/>
+      <c r="AP1" s="1"/>
+      <c r="AQ1" s="1"/>
+      <c r="AR1" s="1"/>
+      <c r="AS1" s="1"/>
+      <c r="AT1" s="1"/>
+      <c r="AU1" s="1"/>
+      <c r="AV1" s="1"/>
+      <c r="AW1" s="1"/>
+      <c r="AX1" s="1"/>
+      <c r="AY1" s="1"/>
+      <c r="AZ1" s="1"/>
+      <c r="BA1" s="1"/>
+      <c r="BB1" s="1"/>
+      <c r="BC1" s="1"/>
+      <c r="BD1" s="1"/>
+      <c r="BE1" s="1"/>
+      <c r="BF1" s="1"/>
+      <c r="BG1" s="1"/>
+      <c r="BH1" s="1"/>
+      <c r="BI1" s="1"/>
+      <c r="BJ1" s="1"/>
+      <c r="BK1" s="1"/>
+      <c r="BL1" s="1"/>
+      <c r="BM1" s="1"/>
+      <c r="BN1" s="1"/>
+      <c r="BO1" s="1"/>
+      <c r="BP1" s="1"/>
+      <c r="BQ1" s="1"/>
+      <c r="BR1" s="1"/>
+      <c r="BS1" s="1"/>
+      <c r="BT1" s="1"/>
+      <c r="BU1" s="1"/>
+      <c r="BV1" s="1"/>
+      <c r="BW1" s="1"/>
+      <c r="BX1" s="1"/>
+      <c r="BY1" s="1"/>
+      <c r="BZ1" s="1"/>
+      <c r="CA1" s="1"/>
+      <c r="CB1" s="1"/>
+      <c r="CC1" s="1"/>
+      <c r="CD1" s="1"/>
+      <c r="CE1" s="1"/>
+      <c r="CF1" s="1"/>
+      <c r="CG1" s="1"/>
+      <c r="CH1" s="1"/>
+      <c r="CI1" s="1"/>
+      <c r="CJ1" s="1"/>
+      <c r="CK1" s="1"/>
+      <c r="CL1" s="1"/>
+    </row>
+    <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="56" t="s">
+        <v>74</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1"/>
+      <c r="W2" s="1"/>
+      <c r="X2" s="1"/>
+      <c r="Y2" s="1"/>
+      <c r="Z2" s="1"/>
+      <c r="AA2" s="1"/>
+      <c r="AB2" s="1"/>
+      <c r="AC2" s="1"/>
+      <c r="AD2" s="1"/>
+      <c r="AE2" s="1"/>
+      <c r="AF2" s="1"/>
+      <c r="AG2" s="1"/>
+      <c r="AH2" s="1"/>
+      <c r="AI2" s="1"/>
+      <c r="AJ2" s="1"/>
+      <c r="AK2" s="1"/>
+      <c r="AL2" s="1"/>
+      <c r="AM2" s="1"/>
+      <c r="AN2" s="1"/>
+      <c r="AO2" s="1"/>
+      <c r="AP2" s="1"/>
+      <c r="AQ2" s="1"/>
+      <c r="AR2" s="1"/>
+      <c r="AS2" s="1"/>
+      <c r="AT2" s="1"/>
+      <c r="AU2" s="1"/>
+      <c r="AV2" s="1"/>
+      <c r="AW2" s="1"/>
+      <c r="AX2" s="1"/>
+      <c r="AY2" s="1"/>
+      <c r="AZ2" s="1"/>
+      <c r="BA2" s="1"/>
+      <c r="BB2" s="1"/>
+      <c r="BC2" s="1"/>
+      <c r="BD2" s="1"/>
+      <c r="BE2" s="1"/>
+      <c r="BF2" s="1"/>
+      <c r="BG2" s="1"/>
+      <c r="BH2" s="1"/>
+      <c r="BI2" s="1"/>
+      <c r="BJ2" s="1"/>
+      <c r="BK2" s="1"/>
+      <c r="BL2" s="1"/>
+      <c r="BM2" s="1"/>
+      <c r="BN2" s="1"/>
+      <c r="BO2" s="1"/>
+      <c r="BP2" s="1"/>
+      <c r="BQ2" s="1"/>
+      <c r="BR2" s="1"/>
+      <c r="BS2" s="1"/>
+      <c r="BT2" s="1"/>
+      <c r="BU2" s="1"/>
+      <c r="BV2" s="1"/>
+      <c r="BW2" s="1"/>
+      <c r="BX2" s="1"/>
+      <c r="BY2" s="1"/>
+      <c r="BZ2" s="1"/>
+      <c r="CA2" s="1"/>
+      <c r="CB2" s="1"/>
+      <c r="CC2" s="1"/>
+      <c r="CD2" s="1"/>
+      <c r="CE2" s="1"/>
+      <c r="CF2" s="1"/>
+      <c r="CG2" s="1"/>
+      <c r="CH2" s="1"/>
+      <c r="CI2" s="1"/>
+      <c r="CJ2" s="1"/>
+      <c r="CK2" s="1"/>
+      <c r="CL2" s="1"/>
+    </row>
+    <row r="3" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="62" t="s">
+        <v>214</v>
+      </c>
+      <c r="B3" s="39"/>
+      <c r="C3" s="39"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="39"/>
+      <c r="J3" s="39"/>
+      <c r="K3" s="39"/>
+      <c r="L3" s="39"/>
+      <c r="M3" s="39"/>
+      <c r="N3" s="39"/>
+      <c r="O3" s="39"/>
+      <c r="P3" s="39"/>
+      <c r="Q3" s="39"/>
+      <c r="R3" s="39"/>
+      <c r="S3" s="62" t="s">
+        <v>215</v>
+      </c>
+      <c r="T3" s="39"/>
+      <c r="U3" s="39"/>
+      <c r="V3" s="39"/>
+      <c r="W3" s="39"/>
+      <c r="X3" s="39"/>
+      <c r="Y3" s="39"/>
+      <c r="Z3" s="39"/>
+      <c r="AA3" s="39"/>
+      <c r="AB3" s="39"/>
+      <c r="AC3" s="39"/>
+      <c r="AD3" s="39"/>
+      <c r="AE3" s="39"/>
+      <c r="AF3" s="39"/>
+      <c r="AG3" s="39"/>
+      <c r="AH3" s="39"/>
+      <c r="AI3" s="39"/>
+      <c r="AJ3" s="39"/>
+      <c r="AK3" s="62" t="s">
+        <v>216</v>
+      </c>
+      <c r="AL3" s="39"/>
+      <c r="AM3" s="39"/>
+      <c r="AN3" s="39"/>
+      <c r="AO3" s="39"/>
+      <c r="AP3" s="39"/>
+      <c r="AQ3" s="39"/>
+      <c r="AR3" s="39"/>
+      <c r="AS3" s="39"/>
+      <c r="AT3" s="39"/>
+      <c r="AU3" s="39"/>
+      <c r="AV3" s="39"/>
+      <c r="AW3" s="39"/>
+      <c r="AX3" s="39"/>
+      <c r="AY3" s="39"/>
+      <c r="AZ3" s="39"/>
+      <c r="BA3" s="39"/>
+      <c r="BB3" s="39"/>
+      <c r="BC3" s="39"/>
+      <c r="BD3" s="39"/>
+      <c r="BE3" s="39"/>
+      <c r="BF3" s="39"/>
+      <c r="BG3" s="39"/>
+      <c r="BH3" s="39"/>
+      <c r="BI3" s="39"/>
+      <c r="BJ3" s="39"/>
+      <c r="BK3" s="39"/>
+      <c r="BL3" s="39"/>
+      <c r="BM3" s="39"/>
+      <c r="BN3" s="39"/>
+      <c r="BO3" s="39"/>
+      <c r="BP3" s="39"/>
+      <c r="BQ3" s="39"/>
+      <c r="BR3" s="39"/>
+      <c r="BS3" s="39"/>
+      <c r="BT3" s="39"/>
+      <c r="BU3" s="39"/>
+      <c r="BV3" s="39"/>
+      <c r="BW3" s="39"/>
+      <c r="BX3" s="39"/>
+      <c r="BY3" s="39"/>
+      <c r="BZ3" s="39"/>
+      <c r="CA3" s="39"/>
+      <c r="CB3" s="39"/>
+      <c r="CC3" s="39"/>
+      <c r="CD3" s="39"/>
+      <c r="CE3" s="39"/>
+      <c r="CF3" s="39"/>
+      <c r="CG3" s="39"/>
+      <c r="CH3" s="39"/>
+      <c r="CI3" s="39"/>
+      <c r="CJ3" s="39"/>
+      <c r="CK3" s="39"/>
+      <c r="CL3" s="49"/>
+    </row>
+    <row r="4" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="65" t="s">
+        <v>299</v>
+      </c>
+      <c r="B4" s="36"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="36"/>
+      <c r="F4" s="36"/>
+      <c r="G4" s="36"/>
+      <c r="H4" s="36"/>
+      <c r="I4" s="36"/>
+      <c r="J4" s="36"/>
+      <c r="K4" s="36"/>
+      <c r="L4" s="36"/>
+      <c r="M4" s="36"/>
+      <c r="N4" s="36"/>
+      <c r="O4" s="36"/>
+      <c r="P4" s="36"/>
+      <c r="Q4" s="36"/>
+      <c r="R4" s="36"/>
+      <c r="S4" s="65" t="s">
+        <v>249</v>
+      </c>
+      <c r="T4" s="36"/>
+      <c r="U4" s="36"/>
+      <c r="V4" s="36"/>
+      <c r="W4" s="36"/>
+      <c r="X4" s="36"/>
+      <c r="Y4" s="36"/>
+      <c r="Z4" s="36"/>
+      <c r="AA4" s="36"/>
+      <c r="AB4" s="36"/>
+      <c r="AC4" s="36"/>
+      <c r="AD4" s="36"/>
+      <c r="AE4" s="36"/>
+      <c r="AF4" s="36"/>
+      <c r="AG4" s="36"/>
+      <c r="AH4" s="36"/>
+      <c r="AI4" s="64" t="s">
+        <v>60</v>
+      </c>
+      <c r="AJ4" s="36"/>
+      <c r="AK4" s="65" t="s">
+        <v>346</v>
+      </c>
+      <c r="AL4" s="36"/>
+      <c r="AM4" s="36"/>
+      <c r="AN4" s="36"/>
+      <c r="AO4" s="36"/>
+      <c r="AP4" s="36"/>
+      <c r="AQ4" s="36"/>
+      <c r="AR4" s="36"/>
+      <c r="AS4" s="36"/>
+      <c r="AT4" s="36"/>
+      <c r="AU4" s="36"/>
+      <c r="AV4" s="36"/>
+      <c r="AW4" s="36"/>
+      <c r="AX4" s="36"/>
+      <c r="AY4" s="36"/>
+      <c r="AZ4" s="36"/>
+      <c r="BA4" s="36"/>
+      <c r="BB4" s="36"/>
+      <c r="BC4" s="36"/>
+      <c r="BD4" s="36"/>
+      <c r="BE4" s="36"/>
+      <c r="BF4" s="36"/>
+      <c r="BG4" s="36"/>
+      <c r="BH4" s="36"/>
+      <c r="BI4" s="36"/>
+      <c r="BJ4" s="36"/>
+      <c r="BK4" s="36"/>
+      <c r="BL4" s="36"/>
+      <c r="BM4" s="36"/>
+      <c r="BN4" s="36"/>
+      <c r="BO4" s="36"/>
+      <c r="BP4" s="36"/>
+      <c r="BQ4" s="36"/>
+      <c r="BR4" s="36"/>
+      <c r="BS4" s="36"/>
+      <c r="BT4" s="36"/>
+      <c r="BU4" s="36"/>
+      <c r="BV4" s="36"/>
+      <c r="BW4" s="36"/>
+      <c r="BX4" s="36"/>
+      <c r="BY4" s="36"/>
+      <c r="BZ4" s="36"/>
+      <c r="CA4" s="36"/>
+      <c r="CB4" s="36"/>
+      <c r="CC4" s="36"/>
+      <c r="CD4" s="36"/>
+      <c r="CE4" s="36"/>
+      <c r="CF4" s="36"/>
+      <c r="CG4" s="36"/>
+      <c r="CH4" s="36"/>
+      <c r="CI4" s="36"/>
+      <c r="CJ4" s="36"/>
+      <c r="CK4" s="36"/>
+      <c r="CL4" s="37"/>
+    </row>
+    <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="40"/>
+      <c r="B5" s="41"/>
+      <c r="C5" s="41"/>
+      <c r="D5" s="41"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="41"/>
+      <c r="G5" s="41"/>
+      <c r="H5" s="41"/>
+      <c r="I5" s="41"/>
+      <c r="J5" s="41"/>
+      <c r="K5" s="41"/>
+      <c r="L5" s="41"/>
+      <c r="M5" s="41"/>
+      <c r="N5" s="41"/>
+      <c r="O5" s="41"/>
+      <c r="P5" s="41"/>
+      <c r="Q5" s="41"/>
+      <c r="R5" s="41"/>
+      <c r="S5" s="40"/>
+      <c r="T5" s="41"/>
+      <c r="U5" s="41"/>
+      <c r="V5" s="41"/>
+      <c r="W5" s="41"/>
+      <c r="X5" s="41"/>
+      <c r="Y5" s="41"/>
+      <c r="Z5" s="41"/>
+      <c r="AA5" s="41"/>
+      <c r="AB5" s="41"/>
+      <c r="AC5" s="41"/>
+      <c r="AD5" s="41"/>
+      <c r="AE5" s="41"/>
+      <c r="AF5" s="41"/>
+      <c r="AG5" s="41"/>
+      <c r="AH5" s="41"/>
+      <c r="AI5" s="41"/>
+      <c r="AJ5" s="41"/>
+      <c r="AK5" s="43" t="s">
+        <v>347</v>
+      </c>
+      <c r="AL5" s="41"/>
+      <c r="AM5" s="41"/>
+      <c r="AN5" s="41"/>
+      <c r="AO5" s="41"/>
+      <c r="AP5" s="41"/>
+      <c r="AQ5" s="41"/>
+      <c r="AR5" s="41"/>
+      <c r="AS5" s="41"/>
+      <c r="AT5" s="41"/>
+      <c r="AU5" s="41"/>
+      <c r="AV5" s="41"/>
+      <c r="AW5" s="41"/>
+      <c r="AX5" s="41"/>
+      <c r="AY5" s="41"/>
+      <c r="AZ5" s="41"/>
+      <c r="BA5" s="41"/>
+      <c r="BB5" s="41"/>
+      <c r="BC5" s="41"/>
+      <c r="BD5" s="41"/>
+      <c r="BE5" s="41"/>
+      <c r="BF5" s="41"/>
+      <c r="BG5" s="41"/>
+      <c r="BH5" s="41"/>
+      <c r="BI5" s="41"/>
+      <c r="BJ5" s="41"/>
+      <c r="BK5" s="41"/>
+      <c r="BL5" s="41"/>
+      <c r="BM5" s="41"/>
+      <c r="BN5" s="41"/>
+      <c r="BO5" s="41"/>
+      <c r="BP5" s="41"/>
+      <c r="BQ5" s="41"/>
+      <c r="BR5" s="41"/>
+      <c r="BS5" s="41"/>
+      <c r="BT5" s="41"/>
+      <c r="BU5" s="41"/>
+      <c r="BV5" s="41"/>
+      <c r="BW5" s="41"/>
+      <c r="BX5" s="41"/>
+      <c r="BY5" s="41"/>
+      <c r="BZ5" s="41"/>
+      <c r="CA5" s="41"/>
+      <c r="CB5" s="41"/>
+      <c r="CC5" s="41"/>
+      <c r="CD5" s="41"/>
+      <c r="CE5" s="41"/>
+      <c r="CF5" s="41"/>
+      <c r="CG5" s="41"/>
+      <c r="CH5" s="41"/>
+      <c r="CI5" s="41"/>
+      <c r="CJ5" s="41"/>
+      <c r="CK5" s="41"/>
+      <c r="CL5" s="42"/>
+    </row>
+    <row r="6" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="40"/>
+      <c r="B6" s="41"/>
+      <c r="C6" s="41"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="41"/>
+      <c r="H6" s="41"/>
+      <c r="I6" s="41"/>
+      <c r="J6" s="41"/>
+      <c r="K6" s="41"/>
+      <c r="L6" s="41"/>
+      <c r="M6" s="41"/>
+      <c r="N6" s="41"/>
+      <c r="O6" s="41"/>
+      <c r="P6" s="41"/>
+      <c r="Q6" s="41"/>
+      <c r="R6" s="41"/>
+      <c r="S6" s="40"/>
+      <c r="T6" s="41"/>
+      <c r="U6" s="41"/>
+      <c r="V6" s="41"/>
+      <c r="W6" s="41"/>
+      <c r="X6" s="41"/>
+      <c r="Y6" s="41"/>
+      <c r="Z6" s="41"/>
+      <c r="AA6" s="41"/>
+      <c r="AB6" s="41"/>
+      <c r="AC6" s="41"/>
+      <c r="AD6" s="41"/>
+      <c r="AE6" s="41"/>
+      <c r="AF6" s="41"/>
+      <c r="AG6" s="41"/>
+      <c r="AH6" s="41"/>
+      <c r="AI6" s="41"/>
+      <c r="AJ6" s="41"/>
+      <c r="AK6" s="43" t="s">
+        <v>348</v>
+      </c>
+      <c r="AL6" s="41"/>
+      <c r="AM6" s="41"/>
+      <c r="AN6" s="41"/>
+      <c r="AO6" s="41"/>
+      <c r="AP6" s="41"/>
+      <c r="AQ6" s="41"/>
+      <c r="AR6" s="41"/>
+      <c r="AS6" s="41"/>
+      <c r="AT6" s="41"/>
+      <c r="AU6" s="41"/>
+      <c r="AV6" s="41"/>
+      <c r="AW6" s="41"/>
+      <c r="AX6" s="41"/>
+      <c r="AY6" s="41"/>
+      <c r="AZ6" s="41"/>
+      <c r="BA6" s="41"/>
+      <c r="BB6" s="41"/>
+      <c r="BC6" s="41"/>
+      <c r="BD6" s="41"/>
+      <c r="BE6" s="41"/>
+      <c r="BF6" s="41"/>
+      <c r="BG6" s="41"/>
+      <c r="BH6" s="41"/>
+      <c r="BI6" s="41"/>
+      <c r="BJ6" s="41"/>
+      <c r="BK6" s="41"/>
+      <c r="BL6" s="41"/>
+      <c r="BM6" s="41"/>
+      <c r="BN6" s="41"/>
+      <c r="BO6" s="41"/>
+      <c r="BP6" s="41"/>
+      <c r="BQ6" s="41"/>
+      <c r="BR6" s="41"/>
+      <c r="BS6" s="41"/>
+      <c r="BT6" s="41"/>
+      <c r="BU6" s="41"/>
+      <c r="BV6" s="41"/>
+      <c r="BW6" s="41"/>
+      <c r="BX6" s="41"/>
+      <c r="BY6" s="41"/>
+      <c r="BZ6" s="41"/>
+      <c r="CA6" s="41"/>
+      <c r="CB6" s="41"/>
+      <c r="CC6" s="41"/>
+      <c r="CD6" s="41"/>
+      <c r="CE6" s="41"/>
+      <c r="CF6" s="41"/>
+      <c r="CG6" s="41"/>
+      <c r="CH6" s="41"/>
+      <c r="CI6" s="41"/>
+      <c r="CJ6" s="41"/>
+      <c r="CK6" s="41"/>
+      <c r="CL6" s="42"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A2358E7-8911-407D-AA94-1AF2EC7340FC}">
+  <sheetPr codeName="Sheet72"/>
+  <dimension ref="A1:CL5"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="90" width="1.75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="56" t="s">
+        <v>213</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
+      <c r="AD1" s="1"/>
+      <c r="AE1" s="1"/>
+      <c r="AF1" s="1"/>
+      <c r="AG1" s="1"/>
+      <c r="AH1" s="1"/>
+      <c r="AI1" s="1"/>
+      <c r="AJ1" s="1"/>
+      <c r="AK1" s="1"/>
+      <c r="AL1" s="1"/>
+      <c r="AM1" s="1"/>
+      <c r="AN1" s="1"/>
+      <c r="AO1" s="1"/>
+      <c r="AP1" s="1"/>
+      <c r="AQ1" s="1"/>
+      <c r="AR1" s="1"/>
+      <c r="AS1" s="1"/>
+      <c r="AT1" s="1"/>
+      <c r="AU1" s="1"/>
+      <c r="AV1" s="1"/>
+      <c r="AW1" s="1"/>
+      <c r="AX1" s="1"/>
+      <c r="AY1" s="1"/>
+      <c r="AZ1" s="1"/>
+      <c r="BA1" s="1"/>
+      <c r="BB1" s="1"/>
+      <c r="BC1" s="1"/>
+      <c r="BD1" s="1"/>
+      <c r="BE1" s="1"/>
+      <c r="BF1" s="1"/>
+      <c r="BG1" s="1"/>
+      <c r="BH1" s="1"/>
+      <c r="BI1" s="1"/>
+      <c r="BJ1" s="1"/>
+      <c r="BK1" s="1"/>
+      <c r="BL1" s="1"/>
+      <c r="BM1" s="1"/>
+      <c r="BN1" s="1"/>
+      <c r="BO1" s="1"/>
+      <c r="BP1" s="1"/>
+      <c r="BQ1" s="1"/>
+      <c r="BR1" s="1"/>
+      <c r="BS1" s="1"/>
+      <c r="BT1" s="1"/>
+      <c r="BU1" s="1"/>
+      <c r="BV1" s="1"/>
+      <c r="BW1" s="1"/>
+      <c r="BX1" s="1"/>
+      <c r="BY1" s="1"/>
+      <c r="BZ1" s="1"/>
+      <c r="CA1" s="1"/>
+      <c r="CB1" s="1"/>
+      <c r="CC1" s="1"/>
+      <c r="CD1" s="1"/>
+      <c r="CE1" s="1"/>
+      <c r="CF1" s="1"/>
+      <c r="CG1" s="1"/>
+      <c r="CH1" s="1"/>
+      <c r="CI1" s="1"/>
+      <c r="CJ1" s="1"/>
+      <c r="CK1" s="1"/>
+      <c r="CL1" s="1"/>
+    </row>
+    <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="56" t="s">
+        <v>302</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1"/>
+      <c r="W2" s="1"/>
+      <c r="X2" s="1"/>
+      <c r="Y2" s="1"/>
+      <c r="Z2" s="1"/>
+      <c r="AA2" s="1"/>
+      <c r="AB2" s="1"/>
+      <c r="AC2" s="1"/>
+      <c r="AD2" s="1"/>
+      <c r="AE2" s="1"/>
+      <c r="AF2" s="1"/>
+      <c r="AG2" s="1"/>
+      <c r="AH2" s="1"/>
+      <c r="AI2" s="1"/>
+      <c r="AJ2" s="1"/>
+      <c r="AK2" s="1"/>
+      <c r="AL2" s="1"/>
+      <c r="AM2" s="1"/>
+      <c r="AN2" s="1"/>
+      <c r="AO2" s="1"/>
+      <c r="AP2" s="1"/>
+      <c r="AQ2" s="1"/>
+      <c r="AR2" s="1"/>
+      <c r="AS2" s="1"/>
+      <c r="AT2" s="1"/>
+      <c r="AU2" s="1"/>
+      <c r="AV2" s="1"/>
+      <c r="AW2" s="1"/>
+      <c r="AX2" s="1"/>
+      <c r="AY2" s="1"/>
+      <c r="AZ2" s="1"/>
+      <c r="BA2" s="1"/>
+      <c r="BB2" s="1"/>
+      <c r="BC2" s="1"/>
+      <c r="BD2" s="1"/>
+      <c r="BE2" s="1"/>
+      <c r="BF2" s="1"/>
+      <c r="BG2" s="1"/>
+      <c r="BH2" s="1"/>
+      <c r="BI2" s="1"/>
+      <c r="BJ2" s="1"/>
+      <c r="BK2" s="1"/>
+      <c r="BL2" s="1"/>
+      <c r="BM2" s="1"/>
+      <c r="BN2" s="1"/>
+      <c r="BO2" s="1"/>
+      <c r="BP2" s="1"/>
+      <c r="BQ2" s="1"/>
+      <c r="BR2" s="1"/>
+      <c r="BS2" s="1"/>
+      <c r="BT2" s="1"/>
+      <c r="BU2" s="1"/>
+      <c r="BV2" s="1"/>
+      <c r="BW2" s="1"/>
+      <c r="BX2" s="1"/>
+      <c r="BY2" s="1"/>
+      <c r="BZ2" s="1"/>
+      <c r="CA2" s="1"/>
+      <c r="CB2" s="1"/>
+      <c r="CC2" s="1"/>
+      <c r="CD2" s="1"/>
+      <c r="CE2" s="1"/>
+      <c r="CF2" s="1"/>
+      <c r="CG2" s="1"/>
+      <c r="CH2" s="1"/>
+      <c r="CI2" s="1"/>
+      <c r="CJ2" s="1"/>
+      <c r="CK2" s="1"/>
+      <c r="CL2" s="1"/>
+    </row>
+    <row r="3" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="62" t="s">
+        <v>214</v>
+      </c>
+      <c r="B3" s="39"/>
+      <c r="C3" s="39"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="39"/>
+      <c r="J3" s="39"/>
+      <c r="K3" s="39"/>
+      <c r="L3" s="39"/>
+      <c r="M3" s="39"/>
+      <c r="N3" s="39"/>
+      <c r="O3" s="39"/>
+      <c r="P3" s="39"/>
+      <c r="Q3" s="39"/>
+      <c r="R3" s="39"/>
+      <c r="S3" s="62" t="s">
+        <v>215</v>
+      </c>
+      <c r="T3" s="39"/>
+      <c r="U3" s="39"/>
+      <c r="V3" s="39"/>
+      <c r="W3" s="39"/>
+      <c r="X3" s="39"/>
+      <c r="Y3" s="39"/>
+      <c r="Z3" s="39"/>
+      <c r="AA3" s="39"/>
+      <c r="AB3" s="39"/>
+      <c r="AC3" s="39"/>
+      <c r="AD3" s="39"/>
+      <c r="AE3" s="39"/>
+      <c r="AF3" s="39"/>
+      <c r="AG3" s="39"/>
+      <c r="AH3" s="39"/>
+      <c r="AI3" s="39"/>
+      <c r="AJ3" s="39"/>
+      <c r="AK3" s="62" t="s">
+        <v>216</v>
+      </c>
+      <c r="AL3" s="39"/>
+      <c r="AM3" s="39"/>
+      <c r="AN3" s="39"/>
+      <c r="AO3" s="39"/>
+      <c r="AP3" s="39"/>
+      <c r="AQ3" s="39"/>
+      <c r="AR3" s="39"/>
+      <c r="AS3" s="39"/>
+      <c r="AT3" s="39"/>
+      <c r="AU3" s="39"/>
+      <c r="AV3" s="39"/>
+      <c r="AW3" s="39"/>
+      <c r="AX3" s="39"/>
+      <c r="AY3" s="39"/>
+      <c r="AZ3" s="39"/>
+      <c r="BA3" s="39"/>
+      <c r="BB3" s="39"/>
+      <c r="BC3" s="39"/>
+      <c r="BD3" s="39"/>
+      <c r="BE3" s="39"/>
+      <c r="BF3" s="39"/>
+      <c r="BG3" s="39"/>
+      <c r="BH3" s="39"/>
+      <c r="BI3" s="39"/>
+      <c r="BJ3" s="39"/>
+      <c r="BK3" s="39"/>
+      <c r="BL3" s="39"/>
+      <c r="BM3" s="39"/>
+      <c r="BN3" s="39"/>
+      <c r="BO3" s="39"/>
+      <c r="BP3" s="39"/>
+      <c r="BQ3" s="39"/>
+      <c r="BR3" s="39"/>
+      <c r="BS3" s="39"/>
+      <c r="BT3" s="39"/>
+      <c r="BU3" s="39"/>
+      <c r="BV3" s="39"/>
+      <c r="BW3" s="39"/>
+      <c r="BX3" s="39"/>
+      <c r="BY3" s="39"/>
+      <c r="BZ3" s="39"/>
+      <c r="CA3" s="39"/>
+      <c r="CB3" s="39"/>
+      <c r="CC3" s="39"/>
+      <c r="CD3" s="39"/>
+      <c r="CE3" s="39"/>
+      <c r="CF3" s="39"/>
+      <c r="CG3" s="39"/>
+      <c r="CH3" s="39"/>
+      <c r="CI3" s="39"/>
+      <c r="CJ3" s="39"/>
+      <c r="CK3" s="39"/>
+      <c r="CL3" s="49"/>
+    </row>
+    <row r="4" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="65" t="s">
+        <v>299</v>
+      </c>
+      <c r="B4" s="36"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="36"/>
+      <c r="F4" s="36"/>
+      <c r="G4" s="36"/>
+      <c r="H4" s="36"/>
+      <c r="I4" s="36"/>
+      <c r="J4" s="36"/>
+      <c r="K4" s="36"/>
+      <c r="L4" s="36"/>
+      <c r="M4" s="36"/>
+      <c r="N4" s="36"/>
+      <c r="O4" s="36"/>
+      <c r="P4" s="36"/>
+      <c r="Q4" s="36"/>
+      <c r="R4" s="36"/>
+      <c r="S4" s="65" t="s">
+        <v>249</v>
+      </c>
+      <c r="T4" s="36"/>
+      <c r="U4" s="36"/>
+      <c r="V4" s="36"/>
+      <c r="W4" s="36"/>
+      <c r="X4" s="36"/>
+      <c r="Y4" s="36"/>
+      <c r="Z4" s="36"/>
+      <c r="AA4" s="36"/>
+      <c r="AB4" s="36"/>
+      <c r="AC4" s="36"/>
+      <c r="AD4" s="36"/>
+      <c r="AE4" s="36"/>
+      <c r="AF4" s="36"/>
+      <c r="AG4" s="36"/>
+      <c r="AH4" s="36"/>
+      <c r="AI4" s="64" t="s">
+        <v>60</v>
+      </c>
+      <c r="AJ4" s="36"/>
+      <c r="AK4" s="65" t="s">
+        <v>349</v>
+      </c>
+      <c r="AL4" s="36"/>
+      <c r="AM4" s="36"/>
+      <c r="AN4" s="36"/>
+      <c r="AO4" s="36"/>
+      <c r="AP4" s="36"/>
+      <c r="AQ4" s="36"/>
+      <c r="AR4" s="36"/>
+      <c r="AS4" s="36"/>
+      <c r="AT4" s="36"/>
+      <c r="AU4" s="36"/>
+      <c r="AV4" s="36"/>
+      <c r="AW4" s="36"/>
+      <c r="AX4" s="36"/>
+      <c r="AY4" s="36"/>
+      <c r="AZ4" s="36"/>
+      <c r="BA4" s="36"/>
+      <c r="BB4" s="36"/>
+      <c r="BC4" s="36"/>
+      <c r="BD4" s="36"/>
+      <c r="BE4" s="36"/>
+      <c r="BF4" s="36"/>
+      <c r="BG4" s="36"/>
+      <c r="BH4" s="36"/>
+      <c r="BI4" s="36"/>
+      <c r="BJ4" s="36"/>
+      <c r="BK4" s="36"/>
+      <c r="BL4" s="36"/>
+      <c r="BM4" s="36"/>
+      <c r="BN4" s="36"/>
+      <c r="BO4" s="36"/>
+      <c r="BP4" s="36"/>
+      <c r="BQ4" s="36"/>
+      <c r="BR4" s="36"/>
+      <c r="BS4" s="36"/>
+      <c r="BT4" s="36"/>
+      <c r="BU4" s="36"/>
+      <c r="BV4" s="36"/>
+      <c r="BW4" s="36"/>
+      <c r="BX4" s="36"/>
+      <c r="BY4" s="36"/>
+      <c r="BZ4" s="36"/>
+      <c r="CA4" s="36"/>
+      <c r="CB4" s="36"/>
+      <c r="CC4" s="36"/>
+      <c r="CD4" s="36"/>
+      <c r="CE4" s="36"/>
+      <c r="CF4" s="36"/>
+      <c r="CG4" s="36"/>
+      <c r="CH4" s="36"/>
+      <c r="CI4" s="36"/>
+      <c r="CJ4" s="36"/>
+      <c r="CK4" s="36"/>
+      <c r="CL4" s="37"/>
+    </row>
+    <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="40"/>
+      <c r="B5" s="41"/>
+      <c r="C5" s="41"/>
+      <c r="D5" s="41"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="41"/>
+      <c r="G5" s="41"/>
+      <c r="H5" s="41"/>
+      <c r="I5" s="41"/>
+      <c r="J5" s="41"/>
+      <c r="K5" s="41"/>
+      <c r="L5" s="41"/>
+      <c r="M5" s="41"/>
+      <c r="N5" s="41"/>
+      <c r="O5" s="41"/>
+      <c r="P5" s="41"/>
+      <c r="Q5" s="41"/>
+      <c r="R5" s="41"/>
+      <c r="S5" s="40"/>
+      <c r="T5" s="41"/>
+      <c r="U5" s="41"/>
+      <c r="V5" s="41"/>
+      <c r="W5" s="41"/>
+      <c r="X5" s="41"/>
+      <c r="Y5" s="41"/>
+      <c r="Z5" s="41"/>
+      <c r="AA5" s="41"/>
+      <c r="AB5" s="41"/>
+      <c r="AC5" s="41"/>
+      <c r="AD5" s="41"/>
+      <c r="AE5" s="41"/>
+      <c r="AF5" s="41"/>
+      <c r="AG5" s="41"/>
+      <c r="AH5" s="41"/>
+      <c r="AI5" s="41"/>
+      <c r="AJ5" s="41"/>
+      <c r="AK5" s="43" t="s">
+        <v>348</v>
+      </c>
+      <c r="AL5" s="41"/>
+      <c r="AM5" s="41"/>
+      <c r="AN5" s="41"/>
+      <c r="AO5" s="41"/>
+      <c r="AP5" s="41"/>
+      <c r="AQ5" s="41"/>
+      <c r="AR5" s="41"/>
+      <c r="AS5" s="41"/>
+      <c r="AT5" s="41"/>
+      <c r="AU5" s="41"/>
+      <c r="AV5" s="41"/>
+      <c r="AW5" s="41"/>
+      <c r="AX5" s="41"/>
+      <c r="AY5" s="41"/>
+      <c r="AZ5" s="41"/>
+      <c r="BA5" s="41"/>
+      <c r="BB5" s="41"/>
+      <c r="BC5" s="41"/>
+      <c r="BD5" s="41"/>
+      <c r="BE5" s="41"/>
+      <c r="BF5" s="41"/>
+      <c r="BG5" s="41"/>
+      <c r="BH5" s="41"/>
+      <c r="BI5" s="41"/>
+      <c r="BJ5" s="41"/>
+      <c r="BK5" s="41"/>
+      <c r="BL5" s="41"/>
+      <c r="BM5" s="41"/>
+      <c r="BN5" s="41"/>
+      <c r="BO5" s="41"/>
+      <c r="BP5" s="41"/>
+      <c r="BQ5" s="41"/>
+      <c r="BR5" s="41"/>
+      <c r="BS5" s="41"/>
+      <c r="BT5" s="41"/>
+      <c r="BU5" s="41"/>
+      <c r="BV5" s="41"/>
+      <c r="BW5" s="41"/>
+      <c r="BX5" s="41"/>
+      <c r="BY5" s="41"/>
+      <c r="BZ5" s="41"/>
+      <c r="CA5" s="41"/>
+      <c r="CB5" s="41"/>
+      <c r="CC5" s="41"/>
+      <c r="CD5" s="41"/>
+      <c r="CE5" s="41"/>
+      <c r="CF5" s="41"/>
+      <c r="CG5" s="41"/>
+      <c r="CH5" s="41"/>
+      <c r="CI5" s="41"/>
+      <c r="CJ5" s="41"/>
+      <c r="CK5" s="41"/>
+      <c r="CL5" s="42"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{956EFD9A-0444-473E-BD83-6FED68498CDD}">
+  <sheetPr codeName="Sheet73"/>
+  <dimension ref="A1:CL5"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="90" width="1.75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="56" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
+      <c r="AD1" s="1"/>
+      <c r="AE1" s="1"/>
+      <c r="AF1" s="1"/>
+      <c r="AG1" s="1"/>
+      <c r="AH1" s="1"/>
+      <c r="AI1" s="1"/>
+      <c r="AJ1" s="1"/>
+      <c r="AK1" s="1"/>
+      <c r="AL1" s="1"/>
+      <c r="AM1" s="1"/>
+      <c r="AN1" s="1"/>
+      <c r="AO1" s="1"/>
+      <c r="AP1" s="1"/>
+      <c r="AQ1" s="1"/>
+      <c r="AR1" s="1"/>
+      <c r="AS1" s="1"/>
+      <c r="AT1" s="1"/>
+      <c r="AU1" s="1"/>
+      <c r="AV1" s="1"/>
+      <c r="AW1" s="1"/>
+      <c r="AX1" s="1"/>
+      <c r="AY1" s="1"/>
+      <c r="AZ1" s="1"/>
+      <c r="BA1" s="1"/>
+      <c r="BB1" s="1"/>
+      <c r="BC1" s="1"/>
+      <c r="BD1" s="1"/>
+      <c r="BE1" s="1"/>
+      <c r="BF1" s="1"/>
+      <c r="BG1" s="1"/>
+      <c r="BH1" s="1"/>
+      <c r="BI1" s="1"/>
+      <c r="BJ1" s="1"/>
+      <c r="BK1" s="1"/>
+      <c r="BL1" s="1"/>
+      <c r="BM1" s="1"/>
+      <c r="BN1" s="1"/>
+      <c r="BO1" s="1"/>
+      <c r="BP1" s="1"/>
+      <c r="BQ1" s="1"/>
+      <c r="BR1" s="1"/>
+      <c r="BS1" s="1"/>
+      <c r="BT1" s="1"/>
+      <c r="BU1" s="1"/>
+      <c r="BV1" s="1"/>
+      <c r="BW1" s="1"/>
+      <c r="BX1" s="1"/>
+      <c r="BY1" s="1"/>
+      <c r="BZ1" s="1"/>
+      <c r="CA1" s="1"/>
+      <c r="CB1" s="1"/>
+      <c r="CC1" s="1"/>
+      <c r="CD1" s="1"/>
+      <c r="CE1" s="1"/>
+      <c r="CF1" s="1"/>
+      <c r="CG1" s="1"/>
+      <c r="CH1" s="1"/>
+      <c r="CI1" s="1"/>
+      <c r="CJ1" s="1"/>
+      <c r="CK1" s="1"/>
+      <c r="CL1" s="1"/>
+    </row>
+    <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="56" t="s">
+        <v>74</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1"/>
+      <c r="W2" s="1"/>
+      <c r="X2" s="1"/>
+      <c r="Y2" s="1"/>
+      <c r="Z2" s="1"/>
+      <c r="AA2" s="1"/>
+      <c r="AB2" s="1"/>
+      <c r="AC2" s="1"/>
+      <c r="AD2" s="1"/>
+      <c r="AE2" s="1"/>
+      <c r="AF2" s="1"/>
+      <c r="AG2" s="1"/>
+      <c r="AH2" s="1"/>
+      <c r="AI2" s="1"/>
+      <c r="AJ2" s="1"/>
+      <c r="AK2" s="1"/>
+      <c r="AL2" s="1"/>
+      <c r="AM2" s="1"/>
+      <c r="AN2" s="1"/>
+      <c r="AO2" s="1"/>
+      <c r="AP2" s="1"/>
+      <c r="AQ2" s="1"/>
+      <c r="AR2" s="1"/>
+      <c r="AS2" s="1"/>
+      <c r="AT2" s="1"/>
+      <c r="AU2" s="1"/>
+      <c r="AV2" s="1"/>
+      <c r="AW2" s="1"/>
+      <c r="AX2" s="1"/>
+      <c r="AY2" s="1"/>
+      <c r="AZ2" s="1"/>
+      <c r="BA2" s="1"/>
+      <c r="BB2" s="1"/>
+      <c r="BC2" s="1"/>
+      <c r="BD2" s="1"/>
+      <c r="BE2" s="1"/>
+      <c r="BF2" s="1"/>
+      <c r="BG2" s="1"/>
+      <c r="BH2" s="1"/>
+      <c r="BI2" s="1"/>
+      <c r="BJ2" s="1"/>
+      <c r="BK2" s="1"/>
+      <c r="BL2" s="1"/>
+      <c r="BM2" s="1"/>
+      <c r="BN2" s="1"/>
+      <c r="BO2" s="1"/>
+      <c r="BP2" s="1"/>
+      <c r="BQ2" s="1"/>
+      <c r="BR2" s="1"/>
+      <c r="BS2" s="1"/>
+      <c r="BT2" s="1"/>
+      <c r="BU2" s="1"/>
+      <c r="BV2" s="1"/>
+      <c r="BW2" s="1"/>
+      <c r="BX2" s="1"/>
+      <c r="BY2" s="1"/>
+      <c r="BZ2" s="1"/>
+      <c r="CA2" s="1"/>
+      <c r="CB2" s="1"/>
+      <c r="CC2" s="1"/>
+      <c r="CD2" s="1"/>
+      <c r="CE2" s="1"/>
+      <c r="CF2" s="1"/>
+      <c r="CG2" s="1"/>
+      <c r="CH2" s="1"/>
+      <c r="CI2" s="1"/>
+      <c r="CJ2" s="1"/>
+      <c r="CK2" s="1"/>
+      <c r="CL2" s="1"/>
+    </row>
+    <row r="3" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="57" t="s">
+        <v>120</v>
+      </c>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="58" t="s">
+        <v>249</v>
+      </c>
+      <c r="H3" s="28"/>
+      <c r="I3" s="28"/>
+      <c r="J3" s="28"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="28"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="28"/>
+      <c r="O3" s="59" t="s">
+        <v>60</v>
+      </c>
+      <c r="P3" s="28"/>
+      <c r="Q3" s="59" t="s">
+        <v>350</v>
+      </c>
+      <c r="R3" s="28"/>
+      <c r="S3" s="28"/>
+      <c r="T3" s="28"/>
+      <c r="U3" s="28"/>
+      <c r="V3" s="28"/>
+      <c r="W3" s="28"/>
+      <c r="X3" s="28"/>
+      <c r="Y3" s="28"/>
+      <c r="Z3" s="28"/>
+      <c r="AA3" s="28"/>
+      <c r="AB3" s="28"/>
+      <c r="AC3" s="28"/>
+      <c r="AD3" s="28"/>
+      <c r="AE3" s="28"/>
+      <c r="AF3" s="28"/>
+      <c r="AG3" s="28"/>
+      <c r="AH3" s="28"/>
+      <c r="AI3" s="28"/>
+      <c r="AJ3" s="28"/>
+      <c r="AK3" s="28"/>
+      <c r="AL3" s="28"/>
+      <c r="AM3" s="28"/>
+      <c r="AN3" s="28"/>
+      <c r="AO3" s="28"/>
+      <c r="AP3" s="28"/>
+      <c r="AQ3" s="28"/>
+      <c r="AR3" s="28"/>
+      <c r="AS3" s="28"/>
+      <c r="AT3" s="28"/>
+      <c r="AU3" s="28"/>
+      <c r="AV3" s="28"/>
+      <c r="AW3" s="28"/>
+      <c r="AX3" s="28"/>
+      <c r="AY3" s="28"/>
+      <c r="AZ3" s="28"/>
+      <c r="BA3" s="28"/>
+      <c r="BB3" s="28"/>
+      <c r="BC3" s="28"/>
+      <c r="BD3" s="28"/>
+      <c r="BE3" s="28"/>
+      <c r="BF3" s="28"/>
+      <c r="BG3" s="28"/>
+      <c r="BH3" s="28"/>
+      <c r="BI3" s="28"/>
+      <c r="BJ3" s="28"/>
+      <c r="BK3" s="28"/>
+      <c r="BL3" s="28"/>
+      <c r="BM3" s="28"/>
+      <c r="BN3" s="28"/>
+      <c r="BO3" s="28"/>
+      <c r="BP3" s="28"/>
+      <c r="BQ3" s="28"/>
+      <c r="BR3" s="28"/>
+      <c r="BS3" s="28"/>
+      <c r="BT3" s="28"/>
+      <c r="BU3" s="28"/>
+      <c r="BV3" s="28"/>
+      <c r="BW3" s="28"/>
+      <c r="BX3" s="28"/>
+      <c r="BY3" s="28"/>
+      <c r="BZ3" s="28"/>
+      <c r="CA3" s="28"/>
+      <c r="CB3" s="28"/>
+      <c r="CC3" s="28"/>
+      <c r="CD3" s="28"/>
+      <c r="CE3" s="28"/>
+      <c r="CF3" s="28"/>
+      <c r="CG3" s="28"/>
+      <c r="CH3" s="28"/>
+      <c r="CI3" s="28"/>
+      <c r="CJ3" s="28"/>
+      <c r="CK3" s="28"/>
+      <c r="CL3" s="29"/>
+    </row>
+    <row r="4" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="30"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="31"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="24"/>
+      <c r="K4" s="24"/>
+      <c r="L4" s="24"/>
+      <c r="M4" s="24"/>
+      <c r="N4" s="24"/>
+      <c r="O4" s="24"/>
+      <c r="P4" s="24"/>
+      <c r="Q4" s="61" t="s">
+        <v>351</v>
+      </c>
+      <c r="R4" s="24"/>
+      <c r="S4" s="24"/>
+      <c r="T4" s="24"/>
+      <c r="U4" s="24"/>
+      <c r="V4" s="24"/>
+      <c r="W4" s="24"/>
+      <c r="X4" s="24"/>
+      <c r="Y4" s="24"/>
+      <c r="Z4" s="24"/>
+      <c r="AA4" s="24"/>
+      <c r="AB4" s="24"/>
+      <c r="AC4" s="24"/>
+      <c r="AD4" s="24"/>
+      <c r="AE4" s="24"/>
+      <c r="AF4" s="24"/>
+      <c r="AG4" s="24"/>
+      <c r="AH4" s="24"/>
+      <c r="AI4" s="24"/>
+      <c r="AJ4" s="24"/>
+      <c r="AK4" s="24"/>
+      <c r="AL4" s="24"/>
+      <c r="AM4" s="24"/>
+      <c r="AN4" s="24"/>
+      <c r="AO4" s="24"/>
+      <c r="AP4" s="24"/>
+      <c r="AQ4" s="24"/>
+      <c r="AR4" s="24"/>
+      <c r="AS4" s="24"/>
+      <c r="AT4" s="24"/>
+      <c r="AU4" s="24"/>
+      <c r="AV4" s="24"/>
+      <c r="AW4" s="24"/>
+      <c r="AX4" s="24"/>
+      <c r="AY4" s="24"/>
+      <c r="AZ4" s="24"/>
+      <c r="BA4" s="24"/>
+      <c r="BB4" s="24"/>
+      <c r="BC4" s="24"/>
+      <c r="BD4" s="24"/>
+      <c r="BE4" s="24"/>
+      <c r="BF4" s="24"/>
+      <c r="BG4" s="24"/>
+      <c r="BH4" s="24"/>
+      <c r="BI4" s="24"/>
+      <c r="BJ4" s="24"/>
+      <c r="BK4" s="24"/>
+      <c r="BL4" s="24"/>
+      <c r="BM4" s="24"/>
+      <c r="BN4" s="24"/>
+      <c r="BO4" s="24"/>
+      <c r="BP4" s="24"/>
+      <c r="BQ4" s="24"/>
+      <c r="BR4" s="24"/>
+      <c r="BS4" s="24"/>
+      <c r="BT4" s="24"/>
+      <c r="BU4" s="24"/>
+      <c r="BV4" s="24"/>
+      <c r="BW4" s="24"/>
+      <c r="BX4" s="24"/>
+      <c r="BY4" s="24"/>
+      <c r="BZ4" s="24"/>
+      <c r="CA4" s="24"/>
+      <c r="CB4" s="24"/>
+      <c r="CC4" s="24"/>
+      <c r="CD4" s="24"/>
+      <c r="CE4" s="24"/>
+      <c r="CF4" s="24"/>
+      <c r="CG4" s="24"/>
+      <c r="CH4" s="24"/>
+      <c r="CI4" s="24"/>
+      <c r="CJ4" s="24"/>
+      <c r="CK4" s="24"/>
+      <c r="CL4" s="32"/>
+    </row>
+    <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="62" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" s="39"/>
+      <c r="C5" s="39"/>
+      <c r="D5" s="39"/>
+      <c r="E5" s="39"/>
+      <c r="F5" s="39"/>
+      <c r="G5" s="43" t="s">
+        <v>57</v>
+      </c>
+      <c r="H5" s="41"/>
+      <c r="I5" s="41"/>
+      <c r="J5" s="41"/>
+      <c r="K5" s="41"/>
+      <c r="L5" s="41"/>
+      <c r="M5" s="41"/>
+      <c r="N5" s="41"/>
+      <c r="O5" s="63" t="s">
+        <v>58</v>
+      </c>
+      <c r="P5" s="41"/>
+      <c r="Q5" s="63" t="s">
+        <v>75</v>
+      </c>
+      <c r="R5" s="41"/>
+      <c r="S5" s="41"/>
+      <c r="T5" s="41"/>
+      <c r="U5" s="41"/>
+      <c r="V5" s="41"/>
+      <c r="W5" s="41"/>
+      <c r="X5" s="41"/>
+      <c r="Y5" s="41"/>
+      <c r="Z5" s="41"/>
+      <c r="AA5" s="41"/>
+      <c r="AB5" s="41"/>
+      <c r="AC5" s="41"/>
+      <c r="AD5" s="41"/>
+      <c r="AE5" s="41"/>
+      <c r="AF5" s="41"/>
+      <c r="AG5" s="41"/>
+      <c r="AH5" s="41"/>
+      <c r="AI5" s="41"/>
+      <c r="AJ5" s="41"/>
+      <c r="AK5" s="41"/>
+      <c r="AL5" s="41"/>
+      <c r="AM5" s="41"/>
+      <c r="AN5" s="41"/>
+      <c r="AO5" s="41"/>
+      <c r="AP5" s="41"/>
+      <c r="AQ5" s="41"/>
+      <c r="AR5" s="41"/>
+      <c r="AS5" s="41"/>
+      <c r="AT5" s="41"/>
+      <c r="AU5" s="41"/>
+      <c r="AV5" s="41"/>
+      <c r="AW5" s="41"/>
+      <c r="AX5" s="41"/>
+      <c r="AY5" s="41"/>
+      <c r="AZ5" s="41"/>
+      <c r="BA5" s="41"/>
+      <c r="BB5" s="41"/>
+      <c r="BC5" s="41"/>
+      <c r="BD5" s="41"/>
+      <c r="BE5" s="41"/>
+      <c r="BF5" s="41"/>
+      <c r="BG5" s="41"/>
+      <c r="BH5" s="41"/>
+      <c r="BI5" s="41"/>
+      <c r="BJ5" s="41"/>
+      <c r="BK5" s="41"/>
+      <c r="BL5" s="41"/>
+      <c r="BM5" s="41"/>
+      <c r="BN5" s="41"/>
+      <c r="BO5" s="41"/>
+      <c r="BP5" s="41"/>
+      <c r="BQ5" s="41"/>
+      <c r="BR5" s="41"/>
+      <c r="BS5" s="41"/>
+      <c r="BT5" s="41"/>
+      <c r="BU5" s="41"/>
+      <c r="BV5" s="41"/>
+      <c r="BW5" s="41"/>
+      <c r="BX5" s="41"/>
+      <c r="BY5" s="41"/>
+      <c r="BZ5" s="41"/>
+      <c r="CA5" s="41"/>
+      <c r="CB5" s="41"/>
+      <c r="CC5" s="41"/>
+      <c r="CD5" s="41"/>
+      <c r="CE5" s="41"/>
+      <c r="CF5" s="41"/>
+      <c r="CG5" s="41"/>
+      <c r="CH5" s="41"/>
+      <c r="CI5" s="41"/>
+      <c r="CJ5" s="41"/>
+      <c r="CK5" s="41"/>
+      <c r="CL5" s="42"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55C79228-10C5-406A-9C26-30FF8F9FEFED}">
+  <dimension ref="A1:CL4"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="90" width="1.75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="56" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
+      <c r="AD1" s="1"/>
+      <c r="AE1" s="1"/>
+      <c r="AF1" s="1"/>
+      <c r="AG1" s="1"/>
+      <c r="AH1" s="1"/>
+      <c r="AI1" s="1"/>
+      <c r="AJ1" s="1"/>
+      <c r="AK1" s="1"/>
+      <c r="AL1" s="1"/>
+      <c r="AM1" s="1"/>
+      <c r="AN1" s="1"/>
+      <c r="AO1" s="1"/>
+      <c r="AP1" s="1"/>
+      <c r="AQ1" s="1"/>
+      <c r="AR1" s="1"/>
+      <c r="AS1" s="1"/>
+      <c r="AT1" s="1"/>
+      <c r="AU1" s="1"/>
+      <c r="AV1" s="1"/>
+      <c r="AW1" s="1"/>
+      <c r="AX1" s="1"/>
+      <c r="AY1" s="1"/>
+      <c r="AZ1" s="1"/>
+      <c r="BA1" s="1"/>
+      <c r="BB1" s="1"/>
+      <c r="BC1" s="1"/>
+      <c r="BD1" s="1"/>
+      <c r="BE1" s="1"/>
+      <c r="BF1" s="1"/>
+      <c r="BG1" s="1"/>
+      <c r="BH1" s="1"/>
+      <c r="BI1" s="1"/>
+      <c r="BJ1" s="1"/>
+      <c r="BK1" s="1"/>
+      <c r="BL1" s="1"/>
+      <c r="BM1" s="1"/>
+      <c r="BN1" s="1"/>
+      <c r="BO1" s="1"/>
+      <c r="BP1" s="1"/>
+      <c r="BQ1" s="1"/>
+      <c r="BR1" s="1"/>
+      <c r="BS1" s="1"/>
+      <c r="BT1" s="1"/>
+      <c r="BU1" s="1"/>
+      <c r="BV1" s="1"/>
+      <c r="BW1" s="1"/>
+      <c r="BX1" s="1"/>
+      <c r="BY1" s="1"/>
+      <c r="BZ1" s="1"/>
+      <c r="CA1" s="1"/>
+      <c r="CB1" s="1"/>
+      <c r="CC1" s="1"/>
+      <c r="CD1" s="1"/>
+      <c r="CE1" s="1"/>
+      <c r="CF1" s="1"/>
+      <c r="CG1" s="1"/>
+      <c r="CH1" s="1"/>
+      <c r="CI1" s="1"/>
+      <c r="CJ1" s="1"/>
+      <c r="CK1" s="1"/>
+      <c r="CL1" s="1"/>
+    </row>
+    <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="56" t="s">
+        <v>74</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1"/>
+      <c r="W2" s="1"/>
+      <c r="X2" s="1"/>
+      <c r="Y2" s="1"/>
+      <c r="Z2" s="1"/>
+      <c r="AA2" s="1"/>
+      <c r="AB2" s="1"/>
+      <c r="AC2" s="1"/>
+      <c r="AD2" s="1"/>
+      <c r="AE2" s="1"/>
+      <c r="AF2" s="1"/>
+      <c r="AG2" s="1"/>
+      <c r="AH2" s="1"/>
+      <c r="AI2" s="1"/>
+      <c r="AJ2" s="1"/>
+      <c r="AK2" s="1"/>
+      <c r="AL2" s="1"/>
+      <c r="AM2" s="1"/>
+      <c r="AN2" s="1"/>
+      <c r="AO2" s="1"/>
+      <c r="AP2" s="1"/>
+      <c r="AQ2" s="1"/>
+      <c r="AR2" s="1"/>
+      <c r="AS2" s="1"/>
+      <c r="AT2" s="1"/>
+      <c r="AU2" s="1"/>
+      <c r="AV2" s="1"/>
+      <c r="AW2" s="1"/>
+      <c r="AX2" s="1"/>
+      <c r="AY2" s="1"/>
+      <c r="AZ2" s="1"/>
+      <c r="BA2" s="1"/>
+      <c r="BB2" s="1"/>
+      <c r="BC2" s="1"/>
+      <c r="BD2" s="1"/>
+      <c r="BE2" s="1"/>
+      <c r="BF2" s="1"/>
+      <c r="BG2" s="1"/>
+      <c r="BH2" s="1"/>
+      <c r="BI2" s="1"/>
+      <c r="BJ2" s="1"/>
+      <c r="BK2" s="1"/>
+      <c r="BL2" s="1"/>
+      <c r="BM2" s="1"/>
+      <c r="BN2" s="1"/>
+      <c r="BO2" s="1"/>
+      <c r="BP2" s="1"/>
+      <c r="BQ2" s="1"/>
+      <c r="BR2" s="1"/>
+      <c r="BS2" s="1"/>
+      <c r="BT2" s="1"/>
+      <c r="BU2" s="1"/>
+      <c r="BV2" s="1"/>
+      <c r="BW2" s="1"/>
+      <c r="BX2" s="1"/>
+      <c r="BY2" s="1"/>
+      <c r="BZ2" s="1"/>
+      <c r="CA2" s="1"/>
+      <c r="CB2" s="1"/>
+      <c r="CC2" s="1"/>
+      <c r="CD2" s="1"/>
+      <c r="CE2" s="1"/>
+      <c r="CF2" s="1"/>
+      <c r="CG2" s="1"/>
+      <c r="CH2" s="1"/>
+      <c r="CI2" s="1"/>
+      <c r="CJ2" s="1"/>
+      <c r="CK2" s="1"/>
+      <c r="CL2" s="1"/>
+    </row>
+    <row r="3" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="57" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="58" t="s">
+        <v>57</v>
+      </c>
+      <c r="H3" s="28"/>
+      <c r="I3" s="28"/>
+      <c r="J3" s="28"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="28"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="28"/>
+      <c r="O3" s="59" t="s">
+        <v>58</v>
+      </c>
+      <c r="P3" s="28"/>
+      <c r="Q3" s="59" t="s">
+        <v>249</v>
+      </c>
+      <c r="R3" s="28"/>
+      <c r="S3" s="28"/>
+      <c r="T3" s="28"/>
+      <c r="U3" s="28"/>
+      <c r="V3" s="28"/>
+      <c r="W3" s="28"/>
+      <c r="X3" s="28"/>
+      <c r="Y3" s="28"/>
+      <c r="Z3" s="28"/>
+      <c r="AA3" s="28"/>
+      <c r="AB3" s="28"/>
+      <c r="AC3" s="28"/>
+      <c r="AD3" s="28"/>
+      <c r="AE3" s="59" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF3" s="59" t="s">
+        <v>354</v>
+      </c>
+      <c r="AG3" s="28"/>
+      <c r="AH3" s="28"/>
+      <c r="AI3" s="28"/>
+      <c r="AJ3" s="28"/>
+      <c r="AK3" s="28"/>
+      <c r="AL3" s="28"/>
+      <c r="AM3" s="28"/>
+      <c r="AN3" s="28"/>
+      <c r="AO3" s="28"/>
+      <c r="AP3" s="28"/>
+      <c r="AQ3" s="28"/>
+      <c r="AR3" s="28"/>
+      <c r="AS3" s="28"/>
+      <c r="AT3" s="28"/>
+      <c r="AU3" s="28"/>
+      <c r="AV3" s="28"/>
+      <c r="AW3" s="28"/>
+      <c r="AX3" s="28"/>
+      <c r="AY3" s="28"/>
+      <c r="AZ3" s="28"/>
+      <c r="BA3" s="28"/>
+      <c r="BB3" s="28"/>
+      <c r="BC3" s="28"/>
+      <c r="BD3" s="28"/>
+      <c r="BE3" s="28"/>
+      <c r="BF3" s="28"/>
+      <c r="BG3" s="28"/>
+      <c r="BH3" s="28"/>
+      <c r="BI3" s="28"/>
+      <c r="BJ3" s="28"/>
+      <c r="BK3" s="28"/>
+      <c r="BL3" s="28"/>
+      <c r="BM3" s="28"/>
+      <c r="BN3" s="28"/>
+      <c r="BO3" s="28"/>
+      <c r="BP3" s="28"/>
+      <c r="BQ3" s="28"/>
+      <c r="BR3" s="28"/>
+      <c r="BS3" s="28"/>
+      <c r="BT3" s="28"/>
+      <c r="BU3" s="28"/>
+      <c r="BV3" s="28"/>
+      <c r="BW3" s="28"/>
+      <c r="BX3" s="28"/>
+      <c r="BY3" s="28"/>
+      <c r="BZ3" s="28"/>
+      <c r="CA3" s="28"/>
+      <c r="CB3" s="28"/>
+      <c r="CC3" s="28"/>
+      <c r="CD3" s="28"/>
+      <c r="CE3" s="28"/>
+      <c r="CF3" s="28"/>
+      <c r="CG3" s="28"/>
+      <c r="CH3" s="28"/>
+      <c r="CI3" s="28"/>
+      <c r="CJ3" s="28"/>
+      <c r="CK3" s="28"/>
+      <c r="CL3" s="29"/>
+    </row>
+    <row r="4" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="33"/>
+      <c r="B4" s="34"/>
+      <c r="C4" s="34"/>
+      <c r="D4" s="34"/>
+      <c r="E4" s="34"/>
+      <c r="F4" s="34"/>
+      <c r="G4" s="35"/>
+      <c r="H4" s="36"/>
+      <c r="I4" s="36"/>
+      <c r="J4" s="36"/>
+      <c r="K4" s="36"/>
+      <c r="L4" s="36"/>
+      <c r="M4" s="36"/>
+      <c r="N4" s="36"/>
+      <c r="O4" s="36"/>
+      <c r="P4" s="36"/>
+      <c r="Q4" s="36"/>
+      <c r="R4" s="36"/>
+      <c r="S4" s="36"/>
+      <c r="T4" s="36"/>
+      <c r="U4" s="36"/>
+      <c r="V4" s="36"/>
+      <c r="W4" s="36"/>
+      <c r="X4" s="36"/>
+      <c r="Y4" s="36"/>
+      <c r="Z4" s="36"/>
+      <c r="AA4" s="36"/>
+      <c r="AB4" s="36"/>
+      <c r="AC4" s="36"/>
+      <c r="AD4" s="36"/>
+      <c r="AE4" s="36"/>
+      <c r="AF4" s="64" t="s">
+        <v>236</v>
+      </c>
+      <c r="AG4" s="36"/>
+      <c r="AH4" s="36"/>
+      <c r="AI4" s="36"/>
+      <c r="AJ4" s="36"/>
+      <c r="AK4" s="36"/>
+      <c r="AL4" s="36"/>
+      <c r="AM4" s="36"/>
+      <c r="AN4" s="36"/>
+      <c r="AO4" s="36"/>
+      <c r="AP4" s="36"/>
+      <c r="AQ4" s="36"/>
+      <c r="AR4" s="36"/>
+      <c r="AS4" s="36"/>
+      <c r="AT4" s="36"/>
+      <c r="AU4" s="36"/>
+      <c r="AV4" s="36"/>
+      <c r="AW4" s="36"/>
+      <c r="AX4" s="36"/>
+      <c r="AY4" s="36"/>
+      <c r="AZ4" s="36"/>
+      <c r="BA4" s="36"/>
+      <c r="BB4" s="36"/>
+      <c r="BC4" s="36"/>
+      <c r="BD4" s="36"/>
+      <c r="BE4" s="36"/>
+      <c r="BF4" s="36"/>
+      <c r="BG4" s="36"/>
+      <c r="BH4" s="36"/>
+      <c r="BI4" s="36"/>
+      <c r="BJ4" s="36"/>
+      <c r="BK4" s="36"/>
+      <c r="BL4" s="36"/>
+      <c r="BM4" s="36"/>
+      <c r="BN4" s="36"/>
+      <c r="BO4" s="36"/>
+      <c r="BP4" s="36"/>
+      <c r="BQ4" s="36"/>
+      <c r="BR4" s="36"/>
+      <c r="BS4" s="36"/>
+      <c r="BT4" s="36"/>
+      <c r="BU4" s="36"/>
+      <c r="BV4" s="36"/>
+      <c r="BW4" s="36"/>
+      <c r="BX4" s="36"/>
+      <c r="BY4" s="36"/>
+      <c r="BZ4" s="36"/>
+      <c r="CA4" s="36"/>
+      <c r="CB4" s="36"/>
+      <c r="CC4" s="36"/>
+      <c r="CD4" s="36"/>
+      <c r="CE4" s="36"/>
+      <c r="CF4" s="36"/>
+      <c r="CG4" s="36"/>
+      <c r="CH4" s="36"/>
+      <c r="CI4" s="36"/>
+      <c r="CJ4" s="36"/>
+      <c r="CK4" s="36"/>
+      <c r="CL4" s="37"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{274F91F3-4FA3-4162-9351-46CAD6674E97}">
+  <sheetPr codeName="Sheet74"/>
+  <dimension ref="A1:CL6"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="90" width="1.75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="56" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
+      <c r="AD1" s="1"/>
+      <c r="AE1" s="1"/>
+      <c r="AF1" s="1"/>
+      <c r="AG1" s="1"/>
+      <c r="AH1" s="1"/>
+      <c r="AI1" s="1"/>
+      <c r="AJ1" s="1"/>
+      <c r="AK1" s="1"/>
+      <c r="AL1" s="1"/>
+      <c r="AM1" s="1"/>
+      <c r="AN1" s="1"/>
+      <c r="AO1" s="1"/>
+      <c r="AP1" s="1"/>
+      <c r="AQ1" s="1"/>
+      <c r="AR1" s="1"/>
+      <c r="AS1" s="1"/>
+      <c r="AT1" s="1"/>
+      <c r="AU1" s="1"/>
+      <c r="AV1" s="1"/>
+      <c r="AW1" s="1"/>
+      <c r="AX1" s="1"/>
+      <c r="AY1" s="1"/>
+      <c r="AZ1" s="1"/>
+      <c r="BA1" s="1"/>
+      <c r="BB1" s="1"/>
+      <c r="BC1" s="1"/>
+      <c r="BD1" s="1"/>
+      <c r="BE1" s="1"/>
+      <c r="BF1" s="1"/>
+      <c r="BG1" s="1"/>
+      <c r="BH1" s="1"/>
+      <c r="BI1" s="1"/>
+      <c r="BJ1" s="1"/>
+      <c r="BK1" s="1"/>
+      <c r="BL1" s="1"/>
+      <c r="BM1" s="1"/>
+      <c r="BN1" s="1"/>
+      <c r="BO1" s="1"/>
+      <c r="BP1" s="1"/>
+      <c r="BQ1" s="1"/>
+      <c r="BR1" s="1"/>
+      <c r="BS1" s="1"/>
+      <c r="BT1" s="1"/>
+      <c r="BU1" s="1"/>
+      <c r="BV1" s="1"/>
+      <c r="BW1" s="1"/>
+      <c r="BX1" s="1"/>
+      <c r="BY1" s="1"/>
+      <c r="BZ1" s="1"/>
+      <c r="CA1" s="1"/>
+      <c r="CB1" s="1"/>
+      <c r="CC1" s="1"/>
+      <c r="CD1" s="1"/>
+      <c r="CE1" s="1"/>
+      <c r="CF1" s="1"/>
+      <c r="CG1" s="1"/>
+      <c r="CH1" s="1"/>
+      <c r="CI1" s="1"/>
+      <c r="CJ1" s="1"/>
+      <c r="CK1" s="1"/>
+      <c r="CL1" s="1"/>
+    </row>
+    <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="56" t="s">
+        <v>74</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1"/>
+      <c r="W2" s="1"/>
+      <c r="X2" s="1"/>
+      <c r="Y2" s="1"/>
+      <c r="Z2" s="1"/>
+      <c r="AA2" s="1"/>
+      <c r="AB2" s="1"/>
+      <c r="AC2" s="1"/>
+      <c r="AD2" s="1"/>
+      <c r="AE2" s="1"/>
+      <c r="AF2" s="1"/>
+      <c r="AG2" s="1"/>
+      <c r="AH2" s="1"/>
+      <c r="AI2" s="1"/>
+      <c r="AJ2" s="1"/>
+      <c r="AK2" s="1"/>
+      <c r="AL2" s="1"/>
+      <c r="AM2" s="1"/>
+      <c r="AN2" s="1"/>
+      <c r="AO2" s="1"/>
+      <c r="AP2" s="1"/>
+      <c r="AQ2" s="1"/>
+      <c r="AR2" s="1"/>
+      <c r="AS2" s="1"/>
+      <c r="AT2" s="1"/>
+      <c r="AU2" s="1"/>
+      <c r="AV2" s="1"/>
+      <c r="AW2" s="1"/>
+      <c r="AX2" s="1"/>
+      <c r="AY2" s="1"/>
+      <c r="AZ2" s="1"/>
+      <c r="BA2" s="1"/>
+      <c r="BB2" s="1"/>
+      <c r="BC2" s="1"/>
+      <c r="BD2" s="1"/>
+      <c r="BE2" s="1"/>
+      <c r="BF2" s="1"/>
+      <c r="BG2" s="1"/>
+      <c r="BH2" s="1"/>
+      <c r="BI2" s="1"/>
+      <c r="BJ2" s="1"/>
+      <c r="BK2" s="1"/>
+      <c r="BL2" s="1"/>
+      <c r="BM2" s="1"/>
+      <c r="BN2" s="1"/>
+      <c r="BO2" s="1"/>
+      <c r="BP2" s="1"/>
+      <c r="BQ2" s="1"/>
+      <c r="BR2" s="1"/>
+      <c r="BS2" s="1"/>
+      <c r="BT2" s="1"/>
+      <c r="BU2" s="1"/>
+      <c r="BV2" s="1"/>
+      <c r="BW2" s="1"/>
+      <c r="BX2" s="1"/>
+      <c r="BY2" s="1"/>
+      <c r="BZ2" s="1"/>
+      <c r="CA2" s="1"/>
+      <c r="CB2" s="1"/>
+      <c r="CC2" s="1"/>
+      <c r="CD2" s="1"/>
+      <c r="CE2" s="1"/>
+      <c r="CF2" s="1"/>
+      <c r="CG2" s="1"/>
+      <c r="CH2" s="1"/>
+      <c r="CI2" s="1"/>
+      <c r="CJ2" s="1"/>
+      <c r="CK2" s="1"/>
+      <c r="CL2" s="1"/>
+    </row>
+    <row r="3" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="57" t="s">
+        <v>118</v>
+      </c>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="58" t="s">
+        <v>352</v>
+      </c>
+      <c r="H3" s="28"/>
+      <c r="I3" s="28"/>
+      <c r="J3" s="28"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="28"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="28"/>
+      <c r="O3" s="59" t="s">
+        <v>60</v>
+      </c>
+      <c r="P3" s="28"/>
+      <c r="Q3" s="59" t="s">
+        <v>353</v>
+      </c>
+      <c r="R3" s="28"/>
+      <c r="S3" s="28"/>
+      <c r="T3" s="28"/>
+      <c r="U3" s="28"/>
+      <c r="V3" s="28"/>
+      <c r="W3" s="28"/>
+      <c r="X3" s="28"/>
+      <c r="Y3" s="28"/>
+      <c r="Z3" s="28"/>
+      <c r="AA3" s="28"/>
+      <c r="AB3" s="28"/>
+      <c r="AC3" s="28"/>
+      <c r="AD3" s="28"/>
+      <c r="AE3" s="28"/>
+      <c r="AF3" s="28"/>
+      <c r="AG3" s="28"/>
+      <c r="AH3" s="28"/>
+      <c r="AI3" s="28"/>
+      <c r="AJ3" s="28"/>
+      <c r="AK3" s="28"/>
+      <c r="AL3" s="28"/>
+      <c r="AM3" s="28"/>
+      <c r="AN3" s="28"/>
+      <c r="AO3" s="28"/>
+      <c r="AP3" s="28"/>
+      <c r="AQ3" s="28"/>
+      <c r="AR3" s="28"/>
+      <c r="AS3" s="28"/>
+      <c r="AT3" s="28"/>
+      <c r="AU3" s="28"/>
+      <c r="AV3" s="28"/>
+      <c r="AW3" s="28"/>
+      <c r="AX3" s="28"/>
+      <c r="AY3" s="28"/>
+      <c r="AZ3" s="28"/>
+      <c r="BA3" s="28"/>
+      <c r="BB3" s="28"/>
+      <c r="BC3" s="28"/>
+      <c r="BD3" s="28"/>
+      <c r="BE3" s="28"/>
+      <c r="BF3" s="28"/>
+      <c r="BG3" s="28"/>
+      <c r="BH3" s="28"/>
+      <c r="BI3" s="28"/>
+      <c r="BJ3" s="28"/>
+      <c r="BK3" s="28"/>
+      <c r="BL3" s="28"/>
+      <c r="BM3" s="28"/>
+      <c r="BN3" s="28"/>
+      <c r="BO3" s="28"/>
+      <c r="BP3" s="28"/>
+      <c r="BQ3" s="28"/>
+      <c r="BR3" s="28"/>
+      <c r="BS3" s="28"/>
+      <c r="BT3" s="28"/>
+      <c r="BU3" s="28"/>
+      <c r="BV3" s="28"/>
+      <c r="BW3" s="28"/>
+      <c r="BX3" s="28"/>
+      <c r="BY3" s="28"/>
+      <c r="BZ3" s="28"/>
+      <c r="CA3" s="28"/>
+      <c r="CB3" s="28"/>
+      <c r="CC3" s="28"/>
+      <c r="CD3" s="28"/>
+      <c r="CE3" s="28"/>
+      <c r="CF3" s="28"/>
+      <c r="CG3" s="28"/>
+      <c r="CH3" s="28"/>
+      <c r="CI3" s="28"/>
+      <c r="CJ3" s="28"/>
+      <c r="CK3" s="28"/>
+      <c r="CL3" s="29"/>
+    </row>
+    <row r="4" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="30"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="31"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="24"/>
+      <c r="K4" s="24"/>
+      <c r="L4" s="24"/>
+      <c r="M4" s="24"/>
+      <c r="N4" s="24"/>
+      <c r="O4" s="24"/>
+      <c r="P4" s="24"/>
+      <c r="Q4" s="61" t="s">
+        <v>236</v>
+      </c>
+      <c r="R4" s="24"/>
+      <c r="S4" s="24"/>
+      <c r="T4" s="24"/>
+      <c r="U4" s="24"/>
+      <c r="V4" s="24"/>
+      <c r="W4" s="24"/>
+      <c r="X4" s="24"/>
+      <c r="Y4" s="24"/>
+      <c r="Z4" s="24"/>
+      <c r="AA4" s="24"/>
+      <c r="AB4" s="24"/>
+      <c r="AC4" s="24"/>
+      <c r="AD4" s="24"/>
+      <c r="AE4" s="24"/>
+      <c r="AF4" s="24"/>
+      <c r="AG4" s="24"/>
+      <c r="AH4" s="24"/>
+      <c r="AI4" s="24"/>
+      <c r="AJ4" s="24"/>
+      <c r="AK4" s="24"/>
+      <c r="AL4" s="24"/>
+      <c r="AM4" s="24"/>
+      <c r="AN4" s="24"/>
+      <c r="AO4" s="24"/>
+      <c r="AP4" s="24"/>
+      <c r="AQ4" s="24"/>
+      <c r="AR4" s="24"/>
+      <c r="AS4" s="24"/>
+      <c r="AT4" s="24"/>
+      <c r="AU4" s="24"/>
+      <c r="AV4" s="24"/>
+      <c r="AW4" s="24"/>
+      <c r="AX4" s="24"/>
+      <c r="AY4" s="24"/>
+      <c r="AZ4" s="24"/>
+      <c r="BA4" s="24"/>
+      <c r="BB4" s="24"/>
+      <c r="BC4" s="24"/>
+      <c r="BD4" s="24"/>
+      <c r="BE4" s="24"/>
+      <c r="BF4" s="24"/>
+      <c r="BG4" s="24"/>
+      <c r="BH4" s="24"/>
+      <c r="BI4" s="24"/>
+      <c r="BJ4" s="24"/>
+      <c r="BK4" s="24"/>
+      <c r="BL4" s="24"/>
+      <c r="BM4" s="24"/>
+      <c r="BN4" s="24"/>
+      <c r="BO4" s="24"/>
+      <c r="BP4" s="24"/>
+      <c r="BQ4" s="24"/>
+      <c r="BR4" s="24"/>
+      <c r="BS4" s="24"/>
+      <c r="BT4" s="24"/>
+      <c r="BU4" s="24"/>
+      <c r="BV4" s="24"/>
+      <c r="BW4" s="24"/>
+      <c r="BX4" s="24"/>
+      <c r="BY4" s="24"/>
+      <c r="BZ4" s="24"/>
+      <c r="CA4" s="24"/>
+      <c r="CB4" s="24"/>
+      <c r="CC4" s="24"/>
+      <c r="CD4" s="24"/>
+      <c r="CE4" s="24"/>
+      <c r="CF4" s="24"/>
+      <c r="CG4" s="24"/>
+      <c r="CH4" s="24"/>
+      <c r="CI4" s="24"/>
+      <c r="CJ4" s="24"/>
+      <c r="CK4" s="24"/>
+      <c r="CL4" s="32"/>
+    </row>
+    <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="57" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" s="26"/>
+      <c r="C5" s="26"/>
+      <c r="D5" s="26"/>
+      <c r="E5" s="26"/>
+      <c r="F5" s="26"/>
+      <c r="G5" s="58" t="s">
+        <v>57</v>
+      </c>
+      <c r="H5" s="28"/>
+      <c r="I5" s="28"/>
+      <c r="J5" s="28"/>
+      <c r="K5" s="28"/>
+      <c r="L5" s="28"/>
+      <c r="M5" s="28"/>
+      <c r="N5" s="28"/>
+      <c r="O5" s="59" t="s">
+        <v>58</v>
+      </c>
+      <c r="P5" s="28"/>
+      <c r="Q5" s="59" t="s">
+        <v>75</v>
+      </c>
+      <c r="R5" s="28"/>
+      <c r="S5" s="28"/>
+      <c r="T5" s="28"/>
+      <c r="U5" s="28"/>
+      <c r="V5" s="28"/>
+      <c r="W5" s="28"/>
+      <c r="X5" s="28"/>
+      <c r="Y5" s="28"/>
+      <c r="Z5" s="28"/>
+      <c r="AA5" s="28"/>
+      <c r="AB5" s="28"/>
+      <c r="AC5" s="28"/>
+      <c r="AD5" s="28"/>
+      <c r="AE5" s="28"/>
+      <c r="AF5" s="28"/>
+      <c r="AG5" s="28"/>
+      <c r="AH5" s="28"/>
+      <c r="AI5" s="28"/>
+      <c r="AJ5" s="28"/>
+      <c r="AK5" s="28"/>
+      <c r="AL5" s="28"/>
+      <c r="AM5" s="28"/>
+      <c r="AN5" s="28"/>
+      <c r="AO5" s="28"/>
+      <c r="AP5" s="28"/>
+      <c r="AQ5" s="28"/>
+      <c r="AR5" s="28"/>
+      <c r="AS5" s="28"/>
+      <c r="AT5" s="28"/>
+      <c r="AU5" s="28"/>
+      <c r="AV5" s="28"/>
+      <c r="AW5" s="28"/>
+      <c r="AX5" s="28"/>
+      <c r="AY5" s="28"/>
+      <c r="AZ5" s="28"/>
+      <c r="BA5" s="28"/>
+      <c r="BB5" s="28"/>
+      <c r="BC5" s="28"/>
+      <c r="BD5" s="28"/>
+      <c r="BE5" s="28"/>
+      <c r="BF5" s="28"/>
+      <c r="BG5" s="28"/>
+      <c r="BH5" s="28"/>
+      <c r="BI5" s="28"/>
+      <c r="BJ5" s="28"/>
+      <c r="BK5" s="28"/>
+      <c r="BL5" s="28"/>
+      <c r="BM5" s="28"/>
+      <c r="BN5" s="28"/>
+      <c r="BO5" s="28"/>
+      <c r="BP5" s="28"/>
+      <c r="BQ5" s="28"/>
+      <c r="BR5" s="28"/>
+      <c r="BS5" s="28"/>
+      <c r="BT5" s="28"/>
+      <c r="BU5" s="28"/>
+      <c r="BV5" s="28"/>
+      <c r="BW5" s="28"/>
+      <c r="BX5" s="28"/>
+      <c r="BY5" s="28"/>
+      <c r="BZ5" s="28"/>
+      <c r="CA5" s="28"/>
+      <c r="CB5" s="28"/>
+      <c r="CC5" s="28"/>
+      <c r="CD5" s="28"/>
+      <c r="CE5" s="28"/>
+      <c r="CF5" s="28"/>
+      <c r="CG5" s="28"/>
+      <c r="CH5" s="28"/>
+      <c r="CI5" s="28"/>
+      <c r="CJ5" s="28"/>
+      <c r="CK5" s="28"/>
+      <c r="CL5" s="29"/>
+    </row>
+    <row r="6" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="62" t="s">
+        <v>116</v>
+      </c>
+      <c r="B6" s="39"/>
+      <c r="C6" s="39"/>
+      <c r="D6" s="39"/>
+      <c r="E6" s="39"/>
+      <c r="F6" s="39"/>
+      <c r="G6" s="43" t="s">
+        <v>117</v>
+      </c>
+      <c r="H6" s="41"/>
+      <c r="I6" s="41"/>
+      <c r="J6" s="41"/>
+      <c r="K6" s="41"/>
+      <c r="L6" s="41"/>
+      <c r="M6" s="41"/>
+      <c r="N6" s="41"/>
+      <c r="O6" s="63" t="s">
+        <v>58</v>
+      </c>
+      <c r="P6" s="41"/>
+      <c r="Q6" s="63" t="s">
+        <v>75</v>
+      </c>
+      <c r="R6" s="41"/>
+      <c r="S6" s="41"/>
+      <c r="T6" s="41"/>
+      <c r="U6" s="41"/>
+      <c r="V6" s="41"/>
+      <c r="W6" s="41"/>
+      <c r="X6" s="41"/>
+      <c r="Y6" s="41"/>
+      <c r="Z6" s="41"/>
+      <c r="AA6" s="41"/>
+      <c r="AB6" s="41"/>
+      <c r="AC6" s="41"/>
+      <c r="AD6" s="41"/>
+      <c r="AE6" s="41"/>
+      <c r="AF6" s="41"/>
+      <c r="AG6" s="41"/>
+      <c r="AH6" s="41"/>
+      <c r="AI6" s="41"/>
+      <c r="AJ6" s="41"/>
+      <c r="AK6" s="41"/>
+      <c r="AL6" s="41"/>
+      <c r="AM6" s="41"/>
+      <c r="AN6" s="41"/>
+      <c r="AO6" s="41"/>
+      <c r="AP6" s="41"/>
+      <c r="AQ6" s="41"/>
+      <c r="AR6" s="41"/>
+      <c r="AS6" s="41"/>
+      <c r="AT6" s="41"/>
+      <c r="AU6" s="41"/>
+      <c r="AV6" s="41"/>
+      <c r="AW6" s="41"/>
+      <c r="AX6" s="41"/>
+      <c r="AY6" s="41"/>
+      <c r="AZ6" s="41"/>
+      <c r="BA6" s="41"/>
+      <c r="BB6" s="41"/>
+      <c r="BC6" s="41"/>
+      <c r="BD6" s="41"/>
+      <c r="BE6" s="41"/>
+      <c r="BF6" s="41"/>
+      <c r="BG6" s="41"/>
+      <c r="BH6" s="41"/>
+      <c r="BI6" s="41"/>
+      <c r="BJ6" s="41"/>
+      <c r="BK6" s="41"/>
+      <c r="BL6" s="41"/>
+      <c r="BM6" s="41"/>
+      <c r="BN6" s="41"/>
+      <c r="BO6" s="41"/>
+      <c r="BP6" s="41"/>
+      <c r="BQ6" s="41"/>
+      <c r="BR6" s="41"/>
+      <c r="BS6" s="41"/>
+      <c r="BT6" s="41"/>
+      <c r="BU6" s="41"/>
+      <c r="BV6" s="41"/>
+      <c r="BW6" s="41"/>
+      <c r="BX6" s="41"/>
+      <c r="BY6" s="41"/>
+      <c r="BZ6" s="41"/>
+      <c r="CA6" s="41"/>
+      <c r="CB6" s="41"/>
+      <c r="CC6" s="41"/>
+      <c r="CD6" s="41"/>
+      <c r="CE6" s="41"/>
+      <c r="CF6" s="41"/>
+      <c r="CG6" s="41"/>
+      <c r="CH6" s="41"/>
+      <c r="CI6" s="41"/>
+      <c r="CJ6" s="41"/>
+      <c r="CK6" s="41"/>
+      <c r="CL6" s="42"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>

</xml_diff>

<commit_message>
fix: separate transfer expressions from source columns
</commit_message>
<xml_diff>
--- a/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
+++ b/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
@@ -2,81 +2,81 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-001" sheetId="1" r:id="Re3d60d232002441c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-002" sheetId="2" r:id="Reaff004d4fb54bad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-003" sheetId="3" r:id="R8838b10aed8a4616"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-004" sheetId="4" r:id="R31dceb04a79b41d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-005" sheetId="5" r:id="R45a8515e4def4173"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-006" sheetId="6" r:id="R6de82e3aa9e74108"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-007" sheetId="7" r:id="R45efd9e865d14a0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-008" sheetId="8" r:id="Rc51e5a0284ce4359"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-009" sheetId="9" r:id="Rca106a0fa9f04f82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-010" sheetId="10" r:id="R2ef531694d804715"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-011" sheetId="11" r:id="Rd376e3bc62464cdb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-012" sheetId="12" r:id="R11e36c15d7c24576"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-013" sheetId="13" r:id="Rc0840a5829504498"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-014" sheetId="14" r:id="R92491fb6435f4e14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-015" sheetId="15" r:id="R507f6ad758c54f3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-016" sheetId="16" r:id="R3a7422a324b0465a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-017" sheetId="17" r:id="Rbc4b27f61b0c4a63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-018" sheetId="18" r:id="R5b5a4242ebfe46a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-019" sheetId="19" r:id="Rdf26e27e817647df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-020" sheetId="20" r:id="Rf0bf0f6b94ba4768"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-021" sheetId="21" r:id="Radc2a298fb244a93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-022" sheetId="22" r:id="Ra9b02ae62bf94948"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-023" sheetId="23" r:id="R16f20d6d462b45c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-024" sheetId="24" r:id="Rbb003898dba74f8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-025" sheetId="25" r:id="R1a92c8ba899a4a81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-026" sheetId="26" r:id="Ra814fa2a3f8b4b0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-027" sheetId="37" r:id="Reb05a109f9834fb3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-028" sheetId="27" r:id="R6b104ccc23564c78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-029" sheetId="28" r:id="R97afb3f8d90c4c41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-030" sheetId="29" r:id="Rf1ab75245c8c4110"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-031" sheetId="30" r:id="R80e2754764a54786"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-032" sheetId="31" r:id="Re4899ecf53d04210"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-033" sheetId="32" r:id="R2d90060736284376"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-034" sheetId="33" r:id="R0c4ebd46480247bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-035" sheetId="34" r:id="R91fc92cb87c74b65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-036" sheetId="35" r:id="R74df7aedc09c4dd2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-037" sheetId="36" r:id="Ra0c5f2e3f9d74b6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-038" sheetId="38" r:id="R214c4806c4804a64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-039" sheetId="39" r:id="Raea840452a2a4e95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-040" sheetId="40" r:id="R505193ec7b414332"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-041" sheetId="41" r:id="R976252189c7641a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-042" sheetId="42" r:id="R8cc3e6f82a2e43b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-043" sheetId="43" r:id="Re32586e690aa45e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-044" sheetId="44" r:id="Rda52f2d3a38441ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-045" sheetId="79" r:id="R1f27c28613974eb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-046" sheetId="46" r:id="Rc3ad41954f084760"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-047" sheetId="47" r:id="R2cf387e2f06d46b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-048" sheetId="52" r:id="R5d432b69f0df476e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-049" sheetId="53" r:id="R2ce1a1c77a3b4206"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-050" sheetId="54" r:id="Re3e536489c3e4549"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-051" sheetId="55" r:id="Rb502b55cdcf64086"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-052" sheetId="56" r:id="R11fd0812c4cd45ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-053" sheetId="57" r:id="R18acae09662e4b65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-054" sheetId="48" r:id="R088b5890b4f34bd7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-055" sheetId="49" r:id="Rd7d20d56caa74cff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-056" sheetId="80" r:id="R7eeabb56c43b4b61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-057" sheetId="70" r:id="R07d2e82871dc4335"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-058" sheetId="58" r:id="R1aef3219c29347a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-059" sheetId="81" r:id="Ra2ad9d2e80f24ee2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-060" sheetId="63" r:id="R9295ca66ffc94eb9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-061" sheetId="82" r:id="R251969822bfa464a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-062" sheetId="64" r:id="R1d7753a6c8594db0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-063" sheetId="65" r:id="R5dff84819d864e32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-064" sheetId="66" r:id="Rafc64599ef564a3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-065" sheetId="67" r:id="R914316d04df241c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-066" sheetId="68" r:id="R091c0dd69f6a44fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-067" sheetId="69" r:id="R0c1829c8420f493c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-068" sheetId="71" r:id="R622a1dab730948c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-069" sheetId="72" r:id="Rbd1bc953bf6a4a23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-070" sheetId="73" r:id="Rebf606570b6f4575"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-071" sheetId="74" r:id="Rf42a2c2145da41ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-072" sheetId="75" r:id="R1fa9348c73dc40dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-073" sheetId="76" r:id="R672cd6701c8d4dcb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-074" sheetId="77" r:id="Rc0f2959263c64354"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-075" sheetId="78" r:id="R6fa511d7a3e44119"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-001" sheetId="1" r:id="Rf686810751fe4d68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-002" sheetId="2" r:id="Ra8011ad2fb864d89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-003" sheetId="3" r:id="Rffd839c4de9649fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-004" sheetId="4" r:id="Rf1d4ae1f86774a6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-005" sheetId="5" r:id="R67a879a598374ee1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-006" sheetId="6" r:id="R856a947654fd47fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-007" sheetId="7" r:id="Rbbe8367cb8e9404e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-008" sheetId="8" r:id="R6a2463e8b88649bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-009" sheetId="9" r:id="Rd6d10fca3cc2413f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-010" sheetId="10" r:id="Rc9577af229544780"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-011" sheetId="11" r:id="R1bad759e45764704"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-012" sheetId="12" r:id="R798648c165074af0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-013" sheetId="13" r:id="R72ed89b42d4d4e9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-014" sheetId="14" r:id="R659aed7c8a65441b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-015" sheetId="15" r:id="R2ffdf17dddf944f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-016" sheetId="16" r:id="R7ce821e416dc45e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-017" sheetId="17" r:id="R316bce1dee824e74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-018" sheetId="18" r:id="R591a234213f64c37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-019" sheetId="19" r:id="R57a9330b0c0f4289"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-020" sheetId="20" r:id="R3991a239326d4630"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-021" sheetId="21" r:id="Rce57e1f3bb4c497e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-022" sheetId="22" r:id="R33b74155f2924354"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-023" sheetId="23" r:id="Ra10fd05be90442ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-024" sheetId="24" r:id="Re4dbdfb9dbd14ec4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-025" sheetId="25" r:id="R043a8422f1794809"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-026" sheetId="26" r:id="R3d6ffc678d4a486b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-027" sheetId="37" r:id="R7a6cd80f98a84f7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-028" sheetId="27" r:id="Rffd96d3bbf7649a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-029" sheetId="28" r:id="Raf1e07e377084a8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-030" sheetId="29" r:id="R7d46c0ee8a414c76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-031" sheetId="30" r:id="Rc8738514743f4a90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-032" sheetId="31" r:id="R8708216bc321499d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-033" sheetId="32" r:id="Rab7130daa005447c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-034" sheetId="33" r:id="R4f1d196ec7a44b7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-035" sheetId="34" r:id="Re99af788f1354b3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-036" sheetId="35" r:id="R406ab449c7c74922"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-037" sheetId="36" r:id="Rcd3f99b5ee4c4565"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-038" sheetId="38" r:id="R410e33190db4407e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-039" sheetId="39" r:id="R4e49618187424b0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-040" sheetId="40" r:id="R76d7dac6ecab4608"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-041" sheetId="41" r:id="Rc3b8501ac0e2472c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-042" sheetId="42" r:id="Rc741462d1047443a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-043" sheetId="43" r:id="R9fad8dd7ed7943b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-044" sheetId="44" r:id="Rd5d531fd49754f94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-045" sheetId="79" r:id="Rc016684d579649dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-046" sheetId="46" r:id="R3add21420b2d4e29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-047" sheetId="47" r:id="Rba84b9c179ad4340"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-048" sheetId="52" r:id="R503eebaf238e482a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-049" sheetId="53" r:id="R509e172818f14cd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-050" sheetId="54" r:id="Raf7f88a22fa446a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-051" sheetId="55" r:id="Rcff2e1bc2fc1472e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-052" sheetId="56" r:id="R4d0c73cb80fd4846"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-053" sheetId="57" r:id="R2a13f7f5e6694a1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-054" sheetId="48" r:id="Rbee5a001ef9e4a7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-055" sheetId="49" r:id="R502f0d51c28941fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-056" sheetId="80" r:id="R54bfd7f31c2445d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-057" sheetId="70" r:id="Rd9440d6dffbd46f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-058" sheetId="58" r:id="R5c7a13eb95194e54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-059" sheetId="81" r:id="R8151e5f210a8495f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-060" sheetId="63" r:id="R84f48c47f8404f35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-061" sheetId="82" r:id="R60f6b69d9f7a495b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-062" sheetId="64" r:id="Rde9348b969dd489b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-063" sheetId="65" r:id="R7610585d4d184198"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-064" sheetId="66" r:id="Re7cfa79e9c4b47c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-065" sheetId="67" r:id="Ra03a08e139fa4f86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-066" sheetId="68" r:id="Rd2d3e69b40c24dd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-067" sheetId="69" r:id="R58200b61814343f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-068" sheetId="71" r:id="R1a81ccfd03df44d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-069" sheetId="72" r:id="Rc8b19ed7e3e54756"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-070" sheetId="73" r:id="R04b675fe77974344"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-071" sheetId="74" r:id="Rce21db7d5f6b47a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-072" sheetId="75" r:id="R98594971f23f4c22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-073" sheetId="76" r:id="Raeee1dbf3f35424b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-074" sheetId="77" r:id="R79dde9fdad034be4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-075" sheetId="78" r:id="R4107ca8b06d94454"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -36146,8 +36146,8 @@
       <x:c r="P21" s="18"/>
       <x:c r="Q21" s="18"/>
       <x:c r="R21" s="18"/>
-      <x:c r="S21" s="20" t="s">
-        <x:v>208</x:v>
+      <x:c r="S21" s="20" t="str">
+        <x:v>tb1.氏名、tb1.メール</x:v>
       </x:c>
       <x:c r="T21" s="18"/>
       <x:c r="U21" s="18"/>
@@ -36166,7 +36166,9 @@
       <x:c r="AH21" s="18"/>
       <x:c r="AI21" s="18"/>
       <x:c r="AJ21" s="18"/>
-      <x:c r="AK21" s="17"/>
+      <x:c r="AK21" s="17" t="str">
+        <x:v>COALESCE(tb1.氏名, tb1.メール)</x:v>
+      </x:c>
       <x:c r="AL21" s="18"/>
       <x:c r="AM21" s="18"/>
       <x:c r="AN21" s="18"/>
@@ -36242,8 +36244,8 @@
       <x:c r="P22" s="18"/>
       <x:c r="Q22" s="18"/>
       <x:c r="R22" s="18"/>
-      <x:c r="S22" s="20" t="s">
-        <x:v>209</x:v>
+      <x:c r="S22" s="20" t="str">
+        <x:v>tb2.注文ID</x:v>
       </x:c>
       <x:c r="T22" s="18"/>
       <x:c r="U22" s="18"/>
@@ -36262,7 +36264,9 @@
       <x:c r="AH22" s="18"/>
       <x:c r="AI22" s="18"/>
       <x:c r="AJ22" s="18"/>
-      <x:c r="AK22" s="17"/>
+      <x:c r="AK22" s="17" t="str">
+        <x:v>COUNT(tb2.注文ID)</x:v>
+      </x:c>
       <x:c r="AL22" s="18"/>
       <x:c r="AM22" s="18"/>
       <x:c r="AN22" s="18"/>
@@ -42494,8 +42498,8 @@
       <x:c r="P24" s="18"/>
       <x:c r="Q24" s="18"/>
       <x:c r="R24" s="18"/>
-      <x:c r="S24" s="20" t="s">
-        <x:v>208</x:v>
+      <x:c r="S24" s="20" t="str">
+        <x:v>tb1.氏名、tb1.メール</x:v>
       </x:c>
       <x:c r="T24" s="18"/>
       <x:c r="U24" s="18"/>
@@ -42514,7 +42518,9 @@
       <x:c r="AH24" s="18"/>
       <x:c r="AI24" s="18"/>
       <x:c r="AJ24" s="18"/>
-      <x:c r="AK24" s="17"/>
+      <x:c r="AK24" s="17" t="str">
+        <x:v>COALESCE(tb1.氏名, tb1.メール)</x:v>
+      </x:c>
       <x:c r="AL24" s="18"/>
       <x:c r="AM24" s="18"/>
       <x:c r="AN24" s="18"/>
@@ -42590,8 +42596,8 @@
       <x:c r="P25" s="18"/>
       <x:c r="Q25" s="18"/>
       <x:c r="R25" s="18"/>
-      <x:c r="S25" s="20" t="s">
-        <x:v>209</x:v>
+      <x:c r="S25" s="20" t="str">
+        <x:v>tb2.注文ID</x:v>
       </x:c>
       <x:c r="T25" s="18"/>
       <x:c r="U25" s="18"/>
@@ -42610,7 +42616,9 @@
       <x:c r="AH25" s="18"/>
       <x:c r="AI25" s="18"/>
       <x:c r="AJ25" s="18"/>
-      <x:c r="AK25" s="17"/>
+      <x:c r="AK25" s="17" t="str">
+        <x:v>COUNT(tb2.注文ID)</x:v>
+      </x:c>
       <x:c r="AL25" s="18"/>
       <x:c r="AM25" s="18"/>
       <x:c r="AN25" s="18"/>

</xml_diff>